<commit_message>
[Excel & YAML] Update OWASP Top 10 Web 2021 & 2025
Remove local file links (Redirections to local `.md` files)
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2021.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFBFAC48-5B22-4BF3-BB3A-09AF7CF2036A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A449FA7A-F64D-42EB-8450-B343B488CF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="768" windowWidth="20280" windowHeight="11784" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -2488,77 +2488,6 @@
 有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A04_2021-Insecure_Design/</t>
   </si>
   <si>
-    <t>The application might be vulnerable if the application is:
--   Missing appropriate security hardening across any part of the
-    application stack or improperly configured permissions on cloud
-    services.
--   Unnecessary features are enabled or installed (e.g., unnecessary
-    ports, services, pages, accounts, or privileges).
--   Default accounts and their passwords are still enabled and
-    unchanged.
--   Error handling reveals stack traces or other overly informative
-    error messages to users.
--   For upgraded systems, the latest security features are disabled or
-    not configured securely.
--   The security settings in the application servers, application
-    frameworks (e.g., Struts, Spring, ASP.NET), libraries, databases,
-    etc., are not set to secure values.
--   The server does not send security headers or directives, or they are
-    not set to secure values.
--   The software is out of date or vulnerable (see [A06:2021-Vulnerable
-    and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Without a concerted, repeatable application security configuration
-process, systems are at a higher risk.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
-## How to prevent
-Secure installation processes should be implemented, including:
--   A repeatable hardening process makes it fast and easy to deploy
-    another environment that is appropriately locked down. Development,
-    QA, and production environments should all be configured
-    identically, with different credentials used in each environment.
-    This process should be automated to minimize the effort required to
-    set up a new secure environment.
--   A minimal platform without any unnecessary features, components,
-    documentation, and samples. Remove or do not install unused features
-    and frameworks.
--   A task to review and update the configurations appropriate to all
-    security notes, updates, and patches as part of the patch management
-    process (see [A06:2021-Vulnerable
-    and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)). Review
-    cloud storage permissions (e.g., S3 bucket permissions).
--   A segmented application architecture provides effective and secure
-    separation between components or tenants, with segmentation,
-    containerization, or cloud security groups (ACLs).
--   Sending security directives to clients, e.g., Security Headers.
--   An automated process to verify the effectiveness of the
-    configurations and settings in all environments.
-## Example attack scenarios
-**Scenario #1:** The application server comes with sample applications
-not removed from the production server. These sample applications have
-known security flaws attackers use to compromise the server. Suppose one
-of these applications is the admin console, and default accounts weren't
-changed. In that case, the attacker logs in with default passwords and
-takes over.
-**Scenario #2:** Directory listing is not disabled on the server. An
-attacker discovers they can simply list directories. The attacker finds
-and downloads the compiled Java classes, which they decompile and
-reverse engineer to view the code. The attacker then finds a severe
-access control flaw in the application.
-**Scenario #3:** The application server's configuration allows detailed
-error messages, e.g., stack traces, to be returned to users. This
-potentially exposes sensitive information or underlying flaws such as
-component versions that are known to be vulnerable.
-**Scenario #4:** A cloud service provider (CSP) has default sharing
-permissions open to the Internet by other CSP users. This allows
-sensitive data stored within cloud storage to be accessed.
-For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2021/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
     <t>الإعدادات الأمنية الخاطئة</t>
   </si>
   <si>
@@ -2598,107 +2527,10 @@
     <t>Sicherheitsrelevante Fehlkonfiguration</t>
   </si>
   <si>
-    <t>Die Anwendung besitzt möglicherweise Schwachstellen, wenn folgendes zutrifft:
-- Mangelhafte Sicherheitshärtung des Anwendungsstacks oder ungeeignet konfigurierte Berechtigungen auf Cloud-Diensten.
-- Nicht benötigte Features sind aktiviert oder installiert (z. B. unnötige Ports, Dienste, Seiten, Accounts oder Rechte).
-- Standardkonten und -passwörter sind aktiviert bzw. unverändert.
-- Die Fehlerbehandlung gibt Stack-Traces oder andere interne technische Fehlermeldungen an Anwendende preis.
-- Für aktualisierte Systeme sind die neuesten Sicherheitsfeatures deaktiviert oder nicht sicher konfiguriert.
-- Die Sicherheitseinstellungen in den Anwendungsservern und -frameworks (z. B. Struts, Spring, ASP.NET), Bibliotheken, Datenbanken etc. sind nicht auf sichere Werte gesetzt.
-- Der Server sendet keine Sicherheits-Header oder -Direktiven, bzw. diese sind nicht sicher konfiguriert.
-- Die Software ist veraltet oder verwundbar (siehe [A06:2021-Unsichere oder veraltete Komponenten](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Ohne einen abgestimmten und reproduzierbaren Prozess zur sicheren Konfiguration sind Systeme einem höheren Risiko ausgesetzt!</t>
-  </si>
-  <si>
-    <t>## Score table
-| Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 20          | 19.84 %             | 4.51 %              | 8.12                 | 6.56                | 89.58 %       | 44.84 %       | 208,387           | 789        |
-## How to prevent
-Es sollten sichere Installationsprozesse implementiert werden, darunter:
-- Ein wiederholbarer Härtungsprozess ermöglicht die schnelle und einfache Bereitstellung zusätzlicher Umgebungen, die entsprechend abgesichert sind. Entwicklungs-, Qualitätssicherungs- und Produktionsumgebungen sollten alle identisch konfiguriert sein, wobei in jeder Umgebung unterschiedliche Anmeldeinformationen verwendet werden sollten. Dieser Prozess sollte automatisiert werden, um den Aufwand für die Einrichtung einer neuen sicheren Umgebung zu minimieren.
-- Eine minimale Plattform ohne unnötige Funktionen, Komponenten, Dokumentation und Beispiele: Entfernen Sie Funktionen und Frameworks die Sie nicht verwenden oder installieren Sie diese erst gar nicht.
-- Überprüfen und Aktualisieren der Konfigurationen, die für alle Sicherheitshinweise, Updates und Patches im Rahmen des Patch-Verwaltungsprozesses geeignet sind (siehe [A06:2021-Unsichere oder veraltete Komponenten](A06_2021-Vulnerable_and_Outdated_Components.md)). Überprüfen Sie die Cloud-Speicherberechtigungen (z. B. S3-Bucket-Berechtigungen).
-- Eine segmentierte Anwendungsarchitektur sorgt durch Segmentierung, Containerisierung oder Cloud-Sicherheitsgruppen (ACLs) für eine effektive und sichere Trennung zwischen Komponenten oder Mandanten.
-- Senden von Sicherheitsanweisungen an Clients, z. B. Sicherheits-Header.
-- Ein automatisierter Prozess zur Überprüfung der Wirksamkeit der Konfigurationen und Einstellungen in allen Umgebungen.
-## Example attack scenarios
-**Szenario Nr. 1:** Der Anwendungsserver wird mit Beispielanwendungen geliefert, die nicht vom Produktionsserver entfernt wurden. Diese Beispielanwendungen weisen bekannte Sicherheitslücken auf, die Angreifende nutzen, um den Server zu gefährden. Angenommen, eine dieser Anwendungen ist die Admin-Konsole und die Standardkonten wurden nicht geändert. In diesem Fall meldet sich die angreifende Person mit Standardkennwörtern an und übernimmt die Kontrolle.
-**Szenario Nr. 2:** Die Directory Listings wurden auf dem Server nicht deaktiviert. Angreifende entdecken, dass Verzeichnisse einfach aufgelistet werden können. Die angreifende Person findet die kompilierten Java-Klassen und lädt sie herunter, dekompiliert sie und betreibt Reverse Engineering, um den Code anzuzeigen. Dies ermöglicht das Findet eines schwerwiegenden Fehlers in der Zugriffskontrolle in der Anwendung.
-**Szenario Nr. 3:** Die Konfiguration des Anwendungsservers ermöglicht die Rückgabe detaillierter Fehlermeldungen an Anwendende, z. B. Stack-Traces. Dadurch werden möglicherweise vertrauliche Informationen oder zugrunde liegende Fehler wie Komponentenversionen offengelegt, die bekanntermaßen anfällig sind.
-**Szenario Nr. 4:** Ein Cloud-Dienstanbieter (CSP) enthält Standardfreigaben, die aus dem Internet für andere Cloud-Nutzende erreichbar sind und ermöglicht dadurch Zugriff auf sensitive Daten in der Cloud.
-Weitere Informationen zu den Referenzen und zur Liste der zugeordneten CWEs: https://top10.owasp.org/2021/de/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
     <t>Configuración de Seguridad Incorrecta</t>
   </si>
   <si>
-    <t>La aplicación puede ser vulnerable si:
--   Le falta el *hardening* de seguridad adecuado en cualquier parte del *stack tecnológico* o permisos configurados incorrectamente en los servicios en la nube.
--   Tiene funciones innecesarias habilitadas o instaladas (puertos, servicios, páginas, cuentas o privilegios innecesarios, por ejemplo).
--   Las cuentas predeterminadas y sus contraseñas aún están habilitadas y sin cambios.
--   El manejo de errores revela a los usuarios rastros de pila u otros mensajes de error demasiado informativos.
--   Para sistemas actualizados, las últimas funciones de seguridad están deshabilitadas o no configuradas de forma segura.
--   Las configuraciones de seguridad en los servidores de aplicaciones, frameworks de aplicaciones (Struts, Spring o ASP.NET por ejemplo), bibliotecas, bases de datos, etc., no poseen configurados valores seguros.
--   El servidor no envía encabezados o directivas de seguridad, o no poseen configurados valores seguros.
--   El software está desactualizado o es vulnerable (consulte [A06:2021-Componentes Vulnerables y Desactualizados](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Sin un proceso de configuración de seguridad de aplicaciones coordinado y repetible, los sistemas corren un mayor riesgo.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
-## How to prevent
-Deben implementarse procesos de instalación seguros, incluyendo:
--   Un proceso de *hardening* repetible agiliza y facilita la implementación de otro entorno que esté debidamente inaccesible. Los entornos de desarrollo, control de calidad y producción deben configurarse de forma idéntica, con diferentes credenciales utilizadas en cada uno.
-    Este proceso debe automatizarse para minimizar el esfuerzo necesario para configurar un nuevo entorno seguro.
--   Una plataforma mínima sin funciones, componentes, documentación ni ejemplos innecesarios. Elimine o no instale características y frameworks no utilizados.
--   Una tarea para revisar y actualizar las configuraciones apropiadas para todas las notas de seguridad, actualizaciones y parches como parte del proceso de administración de parches (consulte [A06: 2021-Componentes Vulnerables y Desactualizados](A06_2021-Vulnerable_and_Outdated_Components.md)). Revise los permisos de almacenamiento en la nube (por ejemplo, Permisos de bucket de S3).
--   Una arquitectura de aplicación segmentada proporciona una separación efectiva y segura entre componentes o instancias, con segmentación, organización en contenedores o grupos de seguridad en la nube (ACLs).
--   Envío de directivas de seguridad a los clientes, por ejemplo, encabezados de seguridad.
--   Un proceso automatizado para verificar la efectividad de las configuraciones y ajustes en todos los entornos.
-## Example attack scenarios
-**Escenario #1:** El servidor de aplicaciones contiene aplicaciones de ejemplo que no se eliminan del servidor de producción. Estas aplicaciones de ejemplo poseen fallas de seguridad conocidas que los atacantes utilizan para comprometer el servidor. Supongamos que una de estas aplicaciones es la consola de administración y no se modificaron las cuentas predeterminadas. En ese caso, el atacante inicia sesión con las contraseñas predeterminadas y toma el control.
-**Escenario #2:** El listado de directorios no se encuentra deshabilitado en el servidor. Un atacante descubre que simplemente puede enumerar directorios. El atacante detecta y descarga las clases Java compiladas, que decompila y aplica ingeniería inversa para ver el código. El atacante luego encuentra una falla severa de control de acceso en la aplicación.
-**Escenario #3:** La configuración del servidor de aplicaciones permite que se retornen a los usuarios mensajes de error detallados, por ejemplo, trazas de pila(stack traces). Esto potencialmente expone información confidencial o fallas subyacentes, como versiones de componentes que se sabe son vulnerables.
-**Escenario #4:** Un proveedor de servicios en la nube (CSP) posee permisos de uso compartido predeterminados abiertos a Internet a otros usuarios. Esto permite acceder a los datos confidenciales almacenados en el almacenamiento en la nube.
-Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2021/es/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
     <t>Mauvaise configuration de sécurité</t>
-  </si>
-  <si>
-    <t>L'application peut être vulnérable si :
--   elle n'a pas fait l'objet d'un durcissement de la sécurité approprié sur l'ensemble des couches protocolaires applicatives, ou si les permissions sont mal configurées sur les services cloud ;
--   des fonctionnalités inutiles sont activées ou installées (ex : des ports, des services, des pages, des comptes ou des privilèges inutiles) ;
--   les comptes par défaut et leurs mots de passe sont toujours activés et inchangés ;
--   le traitement des erreurs révèle aux utilisateurs des traces des piles protocolaires ou d'autres messages d'erreur laissant transpirer trop d'informations ;
--   pour les systèmes à jour ou mis à niveau, les dernières fonctionnalités de sécurité sont désactivées ou ne sont pas configurées de manière sécurisée ;
--   les paramètres de sécurité dans les serveurs d'application, les frameworks applicatifs (ex : Struts, Spring, ASP.NET), les bibliothèques, les bases de données, etc. ne sont pas paramétrés avec des valeurs correctes du point de vue de la sécurité ;
--   le serveur n'envoie pas d'en-têtes ou de directives de sécurité, ou s'ils ne sont pas paramétrés avec des valeurs correctes du point de vue de la sécurité ;
--   La version du logiciel est obsolète ou vulnérable (voir [A06:2021-Composants vulnérables et obsolètes](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Sans un processus concerté et répétable de configuration de la sécurité des applications, les systèmes courent un risque plus élevé.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs associées | Taux d'incidence max | Taux d'incidence moyen | Exploitation pondérée moyenne | Impact pondéré moyen | Couverture max | Couverture moyenne | Nombre total d'occurrences | Nombre total de CVEs |
-|:--------------:|:--------------------:|:----------------------:|:-----------------------------:|:--------------------:|:--------------:|:------------------:|:--------------------------:|:--------------------:|
-|       20       |       19,84 %        |         4,51 %         |             8,12              |         6,56         |    89,58 %     |      44,84 %       |          208 387           |         789          |
-## How to prevent
-Des processus d'installation sécurisés doivent être mis en œuvre, avec notamment :
-- un processus de durcissement répétable qui permette de déployer rapidement et facilement un autre environnement correctement sécurisé avec une configuration verrouillée. Les environnements de développement, d'assurance qualité et de production doivent tous être configurés de manière identique, avec des droits différents pour chaque environnement. Ce processus devrait être automatisé afin de réduire au minimum les efforts requis pour mettre en place un nouvel environnement sécurisé ;
-- une plate-forme minimale sans fonctionnalité, composant, documentation et échantillon inutile. Supprimer ou ne pas installer des fonctionnalités et frameworks inutilisés ;
-- une tâche pour revoir et mettre à jour les configurations appropriées à tous les avis de sécurité, toutes les mises à jour et tous les correctifs dans le cadre du processus de gestion des correctifs (voir [A06:2021-Composants vulnérables et obsolètes](A06_2021-Vulnerable_and_Outdated_Components.md)). En particulier, examiner les permissions de stockage dans le Cloud (ex. les permissions des buckets AWS S3) ;
-- une architecture d'application segmentée qui fournit une séparation efficace et sécurisée entre les composants ou les environnements hébergés, avec de la segmentation, de la mise en conteneurs ou l'utilisation de groupes de sécurité dans le Cloud (ACL) ;
-- l'envoi de directives de sécurité aux clients, par exemple [En-têtes de sécurité](https://wiki.owasp.org/index.php/OWASP_Secure_Headers_Project) ;
-- un processus automatisé pour vérifier l'efficacité des configurations et des réglages dans tous les environnements.
-## Example attack scenarios
-**Scénario 1** : Le serveur d'application est livré avec des applications classiques qui ne sont pas supprimées du serveur mis en production. Ces mêmes applications ont des failles de sécurité connues que les attaquants utilisent afin de compromettre le serveur. Si l'une de ces applications est la console d'administration, et que les comptes par défaut n'ont pas été modifiés, l'attaquant se connecte avec les mots de passe par défaut et prend la main sur la cible.
-**Scénario 2** : La fonctionnalité de listage des répertoires n'est pas désactivée sur le serveur. Un attaquant découvre qu'il peut simplement lister les répertoires. L'attaquant trouve et télécharge les classes Java compilées, qu'il décompose et fait de l'ingénierie inversée pour visualiser le code. L'attaquant trouve alors un grave défaut dans le contrôle d'accès de l'application.
-**Scénario 3** : La configuration du serveur d'application permet de renvoyer aux utilisateurs des messages d'erreur détaillés, par exemple avec des traces des couches protocolaires applicatives. Cela peut ainsi exposer des informations sensibles ou des vulnérabilités sous-jacentes telles que les versions de composants dont on sait qu'elles sont vulnérables.
-**Scénario 4** : Un fournisseur de services Cloud (CSP) a positionné des droits de partage par défaut qui sont ouverts sur Internet par d'autres utilisateurs du CSP. Cela permet d'accéder à des données sensibles stockées dans le stockage Cloud.
-Pour plus d’informations sur les références et la liste des CWE mappées : https://top10.owasp.org/2021/fr/A05_2021-Security_Misconfiguration/</t>
   </si>
   <si>
     <t>Kesalahan Konfigurasi Keamanan</t>
@@ -2736,222 +2568,10 @@
 Untuk informasi lebih lanjut tentang referensi dan daftar CWE yang dipetakan: https://top10.owasp.org/2021/id/A05_2021-Security_Misconfiguration/</t>
   </si>
   <si>
-    <t>L'applicazione potrebbe risultare vulnerabile se:
--   Manca l'hardening di sicurezza appropriato in qualsiasi parte dello
-    stack applicativo o permessi configurati in modo improprio sui servizi
-    cloud.
--   Sono abilitate o installate funzioni non necessarie (ad es.
-    porte, servizi, pagine, account o privilegi non necessari).
--   Gli account di default sono ancora abilitati e presentano password predefinite.
--   A seguito di condizioni di errore, vengono rivelate agli utenti stack traces o altri messaggi  di errore troppo verbosi.
--   Per i sistemi aggiornati, le ultime funzionalità di sicurezza sono disabilitate o
-    non configurate in modo adeguato.
--   Le impostazioni di sicurezza negli application server, nei framework
-    (ad esempio, Struts, Spring, ASP.NET), nelle librerie, database, ecc. non sono configurate su valori sicuri.
--   Il server non invia header o direttive di sicurezza o non sono impostati su valori sicuri.
--   Il software non è aggiornato o è vulnerabile (vedere [A06:2021-Vulnerable
-    and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Senza un processo coordinato e ripetibile per la configurazione della sicurezza delle applicazioni, 
-i sistemi presentano un rischio maggiore.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs corrispondenti | Tasso di incidenza Max | Tasso di incidenza Medio | Sfruttabilità pesata | Impatto Medio | Copertura Max | Copertura media | Occorrenze Totali | CVE Totali |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
-## How to prevent
-Dovrebbero essere implementati processi di installazione sicuri, tra cui:
--   Un processo di hardening ripetibile rende veloce e facile il deploy di
-    un altro ambiente preconfigurato in modo sicuro. Gli ambienti di sviluppo,
-    QA e di produzione dovrebbero essere tutti configurati in modo speculare, con credenziali diverse per ogni ambiente.
-    Questo processo dovrebbe essere automatizzato per minimizzare lo sforzo richiesto per
-    impostare un nuovo ambiente configurato in modo sicuro.
--   Una piattaforma minimale senza funzionalità,componenti,
-    documentazione ed esempi inutili. Rimuovere o non installare funzionalità e
-    framework inutilizzati.
--   Un task per rivedere e aggiornare le configurazioni appropriate a tutte le
-    security notes, aggiornamenti e patch come parte del processo di gestione delle patch
-    (vedere [A06:2021-Vulnerable
-    and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)). Revisionare
-    i permessi del cloud storage (ad esempio, i permessi dei bucket S3).
--   Un'architettura applicativa segmentata fornisce un'efficace e sicura
-    separazione tra componenti o tenant, con segmentazione,
-    containerizzazione, o cloud security groups (ACL).
--   L'invio di direttive di sicurezza ai client, ad esempio, i Security Headers.
--   Un processo automatizzato per verificare l'efficacia delle
-    configurazioni e impostazioni in tutti gli ambienti.
-## Example attack scenarios
-**Scenario #1:** L'application server viene fornito con applicazioni di esempio
-non rimosse dal server di produzione. Queste applicazioni di esempio hanno
-falle di sicurezza note che gli attaccanti usano per compromettere il server. Supponiamo che una
-di queste applicazioni sia la console di amministrazione e che gli account predefiniti non siano stati cambiati. In questo caso, l'attaccante accede con le password predefinite e
-prende il controllo.
-**Scenario #2:** La funzionalità di directory listing non è disabilitata sul server. Un
-attaccante scopre che si possono elencare tutte le directory. L'attaccante trova
-e scarica le classi Java compilate, su cui esegue la decompilazione e il reverse engineering per visualizzare il codice sorgente. L'attaccante trova poi una grave
-difetto di controllo degli accessi nell'applicazione.
-**Scenario #3:** La configurazione dell'application server permette di restituire agli utenti
-messaggi di errore dettagliati, ad esempio la stack trace. Questa problematica
-potenzialmente espone informazioni sensibili o problematiche come
-versioni dei componenti che sono note per essere vulnerabili.
-**Scenario #4:** Un cloud service provider ha dei permessi di condivisione predefiniti
-aperti a Internet da altri utenti nell'header Content Security Policy (CSP). Questo permette
-l'accesso ai dati sensibili memorizzati nel cloud storage.
-Per maggiori informazioni sui riferimenti e sull'elenco delle CWE mappate: https://top10.owasp.org/2021/it/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
     <t>セキュリティの設定ミス</t>
   </si>
   <si>
-    <t>アプリケーションが下記のようなら、恐らく脆弱です:
--   アプリケーションスタックのいずれかの部分におけるセキュリティ堅牢化の不足、あるいはクラウドサービスでパーミッションが不適切に設定されている
--   必要のない機能が有効、あるいはインストールされている(例えば、必要のないポートやサービス、ページ、アカウント、特権)
--   デフォルトのアカウントとパスワードが有効になったまま変更されていない
--   エラー処理がユーザに対して、スタックトレースやその他余計な情報を含むエラーメッセージを見せる
--   アップグレードしたシステムでは、最新のセキュリティ機能が無効になっているか正しく設定されていない
--   アプリケーションサーバやアプリケーションフレームワーク(例えば、Struts、Spring、 ASP.NET)、ライブラリ、データベース等のセキュリティの設定が、安全な値に設定されていない
--   サーバがセキュリテイヘッダーやディレクティブを送らなかったり、安全な値に設定されていなかったりする
--   ソフトウェアが古いか脆弱である。([# A06:2021 – 脆弱で古くなったコンポーネント](A06_2021-Vulnerable_and_Outdated_Components.md) を参照)
-アプリケーションのセキュリティを設定するプロセスを協調して繰り返すことができなければ、システムはより高いリスクにさらされます。</t>
-  </si>
-  <si>
-    <t>## Score table
-| 対応する CWE 数 | 最大発生率 | 平均発生率 |  加重平均（攻撃の難易度） | 加重平均（攻撃による影響） | 最大網羅率 | 平均網羅率 | 総発生数 | CVE 合計件数 |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 20          | 19.84%             | 4.51%              | 89.58%       | 44.84%       | 8.12                 | 6.56                | 208,387           | 789        |
-## How to prevent
-安全にインストールするプロセスにおいて、以下のことを実施すべきです:
--   繰り返し堅牢化するプロセスは、素早くかつ容易に他の環境に展開され、正しくロックダウンすること。
-    開発やQA、本番環境は完全に同じように設定し、それぞれの環境で別々の認証情報を使用すること。
-    このプロセスを自動化し、新しい安全な環境をセットアップする際には、手間を最小限にすること。
--   プラットフォームは最小限のものとし、必要のない機能やコンポーネント、ドキュメント、サンプルを除くこと。
-    使用しない機能とフレームワークは、削除もしくはインストールしないこと。
--   レビューを実施して、セキュリティ関連の記録と更新の全てに加え、パッチを管理するプロセスの一環としてパッチの設定を適切に更新すること([# A06:2021 – 脆弱で古くなったコンポーネント](A06_2021-Vulnerable_and_Outdated_Components.md) を参照)。
-    クラウドストレージのパーミッションは、詳細にレビューすること (例えば、S3 バケットのパーミッション)。
--   セグメント化したアプリケーションアーキテクチャは、セグメンテーションやコンテナリゼーション、クラウドのセキュリティグループ(ACL)をともなったコンポーネントやテナント間に、効果的で安全な仕切りをもたらす。
--   セキュリティディレクティブをクライアントへ送ること。例としては セキュリティヘッダー が挙げられる。
--   プロセスを自動化して設定の有効性を検証し、環境すべてに適用すること。
-## Example attack scenarios
-**シナリオ #1:** 
-アプリケーションのサンプルが付属しているアプリケーションサーバであるにもかかわらず、プロダクションサーバからサンプルが削除されていません。
-このサンプルアプリケーションには、攻撃者がサーバに侵入する際によく使う既知の脆弱性があります。
-そのアプリケーションが管理用のコンソールでデフォルトのアカウントが変更されていないと、攻撃者はデフォルトのパスワードを使ってログインし、乗っ取ってしまいます。
-**シナリオ #2:** 
-ディレクトリリスティングがサーバ上で無効になっていません。攻撃者はそれを見つけ出し、やすやすとディレクトリを表示してしまいます。
-攻撃者はコンパイル済みのJavaクラスを見つけてダウンロードし、デコンパイルしてからリバースエンジニアリングしてコードを見ます。
-そして攻撃者は、そのアプリケーションの深刻なアクセス制御上の穴を見つけます。
-**シナリオ #3:** 
-アプリケーションサーバの設定が、詳細なエラーメッセージ(例えば、スタックトレース)をユーザに返すようになっています。
-これによって機微な情報や脆弱であるとされているコンポーネントのバージョンといった潜在的な欠陥がさらされる恐れがあります。
-**シナリオ #4:** 
-クラウドサービスプロバイダ (CSP) は、他のCSPユーザによるデフォルトでインターネットに公開された共有パーミッションを用意しています。
-こうなると、機微な情報がクラウドストレージに保存され、アクセスされてしまいます。
-参考資料およびマッピングされたCWEの一覧について、詳しくはこちら： https://top10.owasp.org/2021/ja/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
     <t>Configuração Incorreta de Segurança</t>
-  </si>
-  <si>
-    <t>A aplicação pode ser vulnerável se for:
-- Falta de proteção de segurança apropriada em qualquer parte
-    da _stack_ das aplicações ou permissões configuradas incorretamente
-    em serviços em nuvem.
-- Recursos desnecessários são ativados ou instalados (por exemplo,
-    portas, serviços, páginas, contas ou privilégios desnecessários).
-- As contas padrão e suas senhas ainda estão ativadas e inalteradas.
-- O tratamento de erros revela _stack traces_ ou outras
-    mensagens de erro excessivamente informativas aos usuários.
-- Para sistemas atualizados, os recursos de segurança mais recentes
-    estão desabilitados ou não estão configurados com segurança.
-- As configurações de segurança nos servidores das aplicações, nos
-    _frameworks_ (por exemplo, Struts, Spring, ASP.NET), bibliotecas,
-    bancos de dados, etc., não estão definidas para proteger os valores.
-- O servidor não envia cabeçalhos ou diretivas de segurança, ou eles
-    não estão configurados para proteger os valores.
-- O software está desatualizado ou vulnerável (consulte
-  [A06: 2021-Componentes Vulneráveis e Desatualizados](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Sem um processo de configuração de segurança de aplicações que seja integrado e
-repetível, os sistemas correm um risco maior.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
-|:-------------:|:-------------------------:|:------------------------:|:--------------------------:|:-----------------------:|:----------------:|:---------------:|:--------------------:|:-------------:|
-| 20            | 19.84%                    | 4.51%                    | 8.12                       | 6.56                    | 89.58%           | 44.84%          | 208,387              | 789           |
-## How to prevent
-Devem ser implementados processos de instalação segura, incluindo:
-- Um processo de proteção repetível torna mais rápido e fácil implantar
-    outro ambiente que esteja devidamente bloqueado. Os ambientes de
-    desenvolvimento, controle de qualidade e produção devem ser todos
-    configurados de forma idêntica, com credenciais diferentes usadas
-    em cada ambiente. Este processo deve ser automatizado para minimizar
-    o esforço necessário para configurar um novo ambiente seguro.
-- Uma plataforma mínima sem recursos, componentes, documentação e outros
-    desnecessários. Remova ou não instale recursos e estruturas não utilizados.
-- Uma tarefa para revisar e atualizar as configurações apropriadas para todas
-    as notas de segurança, atualizações e patches como parte do processo de
-    gerenciamento de patch (consulte
-    [A06: 2021-Componentes Vulneráveis e Desatualizados](A06_2021-Vulnerable_and_Outdated_Components.md)).
-    Revise as permissões de armazenamento em nuvem (por exemplo, _S3 bucket permissions_).
-- Uma arquitetura de aplicação segmentada fornece separação eficaz e
-    segura entre componentes ou _tenants_, com segmentação,
-    conteinerização ou grupos de segurança em nuvem (ACLs).
-- Envio de diretivas de segurança para clientes, por exemplo, _Security Headers_.
-- Um processo automatizado para verificar a eficácia das configurações
-    em todos os ambientes.
-## Example attack scenarios
-**Cenário #1:** O servidor da aplicação é fornecido com os sistemas de amostra
-não removidos do servidor de produção. Esses aplicativos de amostra têm
-falhas de segurança conhecidas que os invasores usam para comprometer o
-servidor. Suponha que um desses aplicativos seja o console de administração
-e as contas padrão não tenham sido alteradas. Nesse caso, o invasor
-efetua login com as senhas padrão e assume o controle.
-**Cenário #2:** A listagem do diretório não está desabilitada no servidor.
-Um invasor descobre que pode simplesmente listar diretórios. O invasor
-encontra e baixa as classes Java compiladas, que ele descompila e
-faz engenharia reversa para visualizar o código. O invasor então
-encontra uma falha grave de controle de acesso no aplicativo.
-**Cenário #3:** A configuração do servidor de aplicações permite que os
-detalhes das mensagens de erro, por exemplo, _stack trace_, sejam retornadas
-aos usuários. Isso potencialmente expõe informações confidenciais ou falhas
-subjacentes, como versões de componentes que são conhecidas por serem vulneráveis.
-**Cenário #4:** Um provedor de serviços de nuvem tem permissões de
-compartilhamento padrão abertas para a Internet por outros usuários de
-_Content Security Policy header (CSP)_. Isso permite que dados confidenciais
-armazenados no armazenamento em nuvem sejam acessados.
-Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A05_2021-Security_Misconfiguration/</t>
-  </si>
-  <si>
-    <t>Uygulama aşağıdaki durumlarda zafiyete açık olabilir:
-* Application stack’in herhangi bir bölümünde uygun security hardening eksikse veya cloud servislerinde izinler yanlış konfigüre edildiyse.
-* Gereksiz özellikler etkinleştirilmiş ya da kurulmuşsa (ör. gereksiz port’lar, servisler, sayfalar, hesaplar veya ayrıcalıklar).
-* Varsayılan hesaplar ve bunların parolaları hâlâ etkin ve değişmemişse.
-* Error handling, kullanıcıya stack trace’ler veya aşırı bilgi içeren hata mesajları gösteriyorsa.
-* Yükseltilmiş sistemlerde, en yeni security özellikleri devre dışıysa veya güvenli şekilde konfigüre edilmemişse.
-* Application server’ları, application framework’leri (ör. Struts, Spring, ASP.NET), kütüphaneler, veritabanları vb. içindeki security ayarları güvenli değerlere set edilmemişse.
-* Server, security header’ları veya directive’leri göndermiyorsa ya da bunlar güvenli değerlere set edilmemişse.
-* Yazılım güncel değilse veya zafiyetliyse (bkz. [A06:2021 – Vulnerable and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)).
-Planlı ve tekrarlanabilir bir application security configuration süreci olmadan sistemler daha yüksek risk altındadır.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Eşleştirildi | Maks Görülme Oranı | Ort. Görülme Oranı | Ort. Ağırlıklı Exploit | Ort. Ağırlıklı Impact | Maks Coverage | Ort. Coverage | Toplam Olay | Toplam CVE |
-| :---------------: | :----------------: | :----------------: | :--------------------: | :-------------------: | :-----------: | :-----------: | :---------: | :--------: |
-|         20        |       19.84%       |        4.51%       |          8.12          |          6.56         |     89.58%    |     44.84%    |   208,387   |     789    |
-## How to prevent
-Güvenli kurulum süreçleri uygulanmalıdır; bunlar şunları içerir:
-* Tekrarlanabilir bir hardening süreci, uygun şekilde kilitlenmiş başka bir ortamın hızlı ve kolay şekilde deploy edilmesini sağlar. Development, QA ve production ortamları aynı şekilde konfigüre edilmeli; her ortamda farklı credential’lar kullanılmalıdır. Yeni güvenli bir ortam kurulumunda eforu minimize etmek için bu süreç otomatikleştirilmelidir.
-* Gereksiz özellikler, bileşenler, dokümantasyon ve örnekler olmadan minimal bir platform. Kullanılmayan feature ve framework’leri kaldırın ya da hiç kurmayın.
-* Patch management sürecinin bir parçası olarak, tüm security notlarına, update ve patch’lere uygun konfigürasyonları gözden geçirip güncelleme görevi (bkz. [A06:2021 – Vulnerable and Outdated Components](A06_2021-Vulnerable_and_Outdated_Components.md)). Cloud storage izinlerini (ör. S3 bucket permission’ları) gözden geçirin.
-* Segmentasyon, containerization veya cloud security group’ları (ACL’ler) ile bileşenler veya tenant’lar arasında etkili ve güvenli ayrım sağlayan segmented bir application architecture.
-* Client’lara security directive’leri göndermek; ör. Security Headers.
-* Tüm ortamlarda konfigürasyon ve ayarların etkinliğini doğrulayan otomatik bir süreç.
-## Example attack scenarios
-**Senaryo #1:** Application server, production’da kaldırılmamış sample application’larla birlikte geliyor. Bu sample’ların bilinen security açıkları vardır ve saldırganlar server’ı ele geçirmek için bunları kullanır. Bu uygulamalardan biri admin console ise ve varsayılan hesaplar değiştirilmemişse, saldırgan default password’lerle giriş yapar ve kontrolü ele geçirir.
-**Senaryo #2:** Server’da directory listing devre dışı değildir. Bir saldırgan, dizinleri basitçe listeyebildiğini keşfeder. Derlenmiş Java class’larını bulur ve indirir; bunları decompile ederek kodu inceler. Ardından uygulamada ciddi bir access control açığı bulur.
-**Senaryo #3:** Application server konfigürasyonu, detaylı hata mesajlarının (ör. stack trace’ler) kullanıcılara döndürülmesine izin verir. Bu, potansiyel olarak hassas bilgileri veya bilinen zafiyetlere sahip bileşen versiyonları gibi temel açıkları ortaya çıkarabilir.
-**Senaryo #4:** Bir cloud service provider (CSP), diğer CSP kullanıcıları tarafından Internet’e açık varsayılan paylaşım izinlerine sahiptir. Bu durum, cloud storage içinde saklanan hassas verilere erişilmesine olanak tanır.
-Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A05_2021-Security_Misconfiguration/</t>
   </si>
   <si>
     <t>安全设定缺陷</t>
@@ -2989,73 +2609,6 @@
 有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A05_2021-Security_Misconfiguration/</t>
   </si>
   <si>
-    <t>You are likely vulnerable:
--   If you do not know the versions of all components you use (both
-    client-side and server-side). This includes components you directly
-    use as well as nested dependencies.
--   If the software is vulnerable, unsupported, or out of date. This
-    includes the OS, web/application server, database management system
-    (DBMS), applications, APIs and all components, runtime environments,
-    and libraries.
--   If you do not scan for vulnerabilities regularly and subscribe to
-    security bulletins related to the components you use.
--   If you do not fix or upgrade the underlying platform, frameworks,
-    and dependencies in a risk-based, timely fashion. This commonly
-    happens in environments when patching is a monthly or quarterly task
-    under change control, leaving organizations open to days or months
-    of unnecessary exposure to fixed vulnerabilities.
--   If software developers do not test the compatibility of updated,
-    upgraded, or patched libraries.
--   If you do not secure the components’ configurations (see
-    [A05:2021-Security Misconfiguration](A05_2021-Security_Misconfiguration.md)).</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Max Coverage | Avg Coverage | Avg Weighted Exploit | Avg Weighted Impact | Total Occurrences | Total CVEs |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 3           | 27.96%             | 8.77%              | 51.78%       | 22.47%       | 5.00                 | 5.00                | 30,457            | 0          |
-## How to prevent
-There should be a patch management process in place to:
--   Remove unused dependencies, unnecessary features, components, files,
-    and documentation.
--   Continuously inventory the versions of both client-side and
-    server-side components (e.g., frameworks, libraries) and their
-    dependencies using tools like versions, OWASP Dependency Check,
-    retire.js, etc. Continuously monitor sources like Common Vulnerability and 
-    Exposures (CVE) and National Vulnerability Database (NVD) for
-    vulnerabilities in the components. Use software composition analysis
-    tools to automate the process. Subscribe to email alerts for
-    security vulnerabilities related to components you use.
--   Only obtain components from official sources over secure links.
-    Prefer signed packages to reduce the chance of including a modified,
-    malicious component (see [A08:2021-Software and Data Integrity
-    Failures](A08_2021-Software_and_Data_Integrity_Failures.md)).
--   Monitor for libraries and components that are unmaintained or do not
-    create security patches for older versions. If patching is not
-    possible, consider deploying a virtual patch to monitor, detect, or
-    protect against the discovered issue.
-Every organization must ensure an ongoing plan for monitoring, triaging,
-and applying updates or configuration changes for the lifetime of the
-application or portfolio.
-## Example attack scenarios
-**Scenario #1:** Components typically run with the same privileges as
-the application itself, so flaws in any component can result in serious
-impact. Such flaws can be accidental (e.g., coding error) or intentional
-(e.g., a backdoor in a component). Some example exploitable component
-vulnerabilities discovered are:
--   CVE-2017-5638, a Struts 2 remote code execution vulnerability that
-    enables the execution of arbitrary code on the server, has been
-    blamed for significant breaches.
--   While the internet of things (IoT) is frequently difficult or
-    impossible to patch, the importance of patching them can be great
-    (e.g., biomedical devices).
-There are automated tools to help attackers find unpatched or
-misconfigured systems. For example, the Shodan IoT search engine can
-help you find devices that still suffer from Heartbleed vulnerability
-patched in April 2014.
-For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2021/A06_2021-Vulnerable_and_Outdated_Components/</t>
-  </si>
-  <si>
     <t>الثغرات و الانظمة الغير قابلة للتحديثات</t>
   </si>
   <si>
@@ -3091,66 +2644,7 @@
     <t>Unsichere oder veraltete Komponenten</t>
   </si>
   <si>
-    <t>Die Anwendung besitzt möglicherweise Schwachstellen, wenn folgendes zutrifft:
-- Fehlende Kenntnis über die Versionen aller verwendeten Komponenten der in der Anwendung (sowohl client- als auch serverseitig). Dies beinhaltet sowohl direkte als auch indirekte, verschachtelte Abhängigkeiten.
-- Die verwendete Software besitzt Schwachstellen, wird nicht mehr unterstützt oder ist veraltet. Dies beinhaltet das Betriebssystem, den Web-/Applikationsserver, das Datenbankmanagementsystem (DBMS), Anwendungen, APIs und alle verwendeten Komponenten, Laufzeitumgebungen sowie Bibliotheken.
-- Schwachstellenscans werden nicht regelmäßig durchgeführt und die sicherheitsrelevanten Bulletins der verwendeten Komponenten sind nicht abonniert.
-- Die zugrundeliegende Plattform, die Frameworks und die Abhängigkeiten werden nicht risikobasiert und rechtzeitig repariert oder aktualisiert. Dies geschiet in der Regel in Umgebungen, in denen Patchen eine monatliche oder quartalsweise Tätigkeit ist und einer Änderungskontrolle unterliegt. Dies setzt die Organisation unnötigerweise über Tage oder Monate dem Risiko von Schwachstellen aus, für die schon Patches existieren.
-- Softwareentwickler führen keine Kompatibilitäts-Tests der aktualisierten oder gepatchten Bibliotheken durch.
-- Die Komponenten sind nicht sicher konfiguriert (siehe [A05:2021-Sicherheitsrelevante Fehlkonfiguration](A05_2021-Security_Misconfiguration.md)).
-&lt;!-- TODO OSIB Link --&gt;</t>
-  </si>
-  <si>
-    <t>## Score table
-| Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 3          | 27.96 %             | 8.77 %              | 5.00                 | 5.00                | 51.78 %       | 22.47 %       | 30,457           | 0        |
-## How to prevent
-Es sollte ein Patch-Management-Prozess vorhanden sein:
-- Entfernen Sie ungenutzte Abhängigkeiten, unnötige Funktionen, Komponenten, Dateien und Dokumentation.
-- Kontinuierliche Bestandsaufnahme der Versionen sowohl der clientseitigen als auch der serverseitigen Komponenten (z. B. Frameworks, Bibliotheken) und ihrer Abhängigkeiten mithilfe von Tools wie "versions", "OWASP Dependency Check", "retire.js" usw. Überwachen Sie kontinuierlich Quellen wie Common Vulnerability and Exposures (CVE) und die National Vulnerability Database (NVD) für Schwachstellen in den Komponenten. Verwenden Sie Software-Tools zur Analyse der Softwarebestandteile, um den Prozess zu automatisieren. Abonnieren Sie E-Mail-Benachrichtigungen zu Sicherheitslücken im Zusammenhang mit den verwendeten Komponenten.
-- Beziehen Sie Komponenten nur von offiziellen Quellen über sichere Links. Bevorzugen Sie signierte Pakete, um die Wahrscheinlichkeit zu verringern, dass eine modifizierte, bösartige Komponente enthalten ist (siehe [A08:2021-Fehlerhafte Prüfung der Software- und Datenintegrität](A08_2021-Software_and_Data_Integrity_Failures.md)).
-- Überwachen Sie Bibliotheken und Komponenten, die nicht gewartet werden oder keine Sicherheitspatches für ältere Versionen erstellen. Wenn das Patchen nicht möglich ist, erwägen Sie die Bereitstellung eines virtuellen Patches zur Überwachung, Erkennung oder zum Schutz vor dem entdeckten Problem.
-Jede Organisation muss einen fortlaufenden Plan für die Überwachung, Triage und Anwendung von Updates oder Konfigurationsänderungen während der gesamten Lebensdauer der Anwendung oder des Portfolios sicherstellen.
-## Example attack scenarios
-**Szenario Nr. 1:** Komponenten werden normalerweise mit denselben Berechtigungen wie die Anwendung selbst ausgeführt, sodass Fehler in einer Komponente schwerwiegende Auswirkungen haben können. Solche Fehler können zufällig (z. B. ein Programmierfehler) oder absichtlich (z. B. eine Backdoor in einer Komponente) sein. Einige Beispiele für entdeckte ausnutzbare Komponentenschwachstellen sind:
-- CVE-2017-5638, eine Remote Code Execution Schwachstelle in Struts 2, die Angreifende ermächtigt, beliebigen Code auf dem Server auszuführen, wurde für einige erhebliche Sicherheitsvorfälle verantwortlich gemacht.
-- Obwohl das Patchen von Internet of Things (IoT) Geräten oft nur sehr schwierig oder unmöglich ist,
-kann dies sehr wichtig sein (z. B. für biomedizinische Geräte).
-Es existieren automatisierte Tools, die Angreifenden helfen, nicht gepatchte oder falsch konfigurierte Systeme zu finden. Die Shodan IoT-Suchmaschine kann Ihnen beispielsweise dabei helfen, Geräte zu finden, die immer noch für die im April 2014 gepatchte Heartbleed-Sicherheitslücke verwundbar sind.
-Weitere Informationen zu den Referenzen und zur Liste der zugeordneten CWEs: https://top10.owasp.org/2021/de/A06_2021-Vulnerable_and_Outdated_Components/</t>
-  </si>
-  <si>
     <t>Componentes Vulnerables y Desactualizados</t>
-  </si>
-  <si>
-    <t>Usted probablemente sea vulnerable:
--   Si no conoce las versiones de todos los componentes que utiliza (tanto en el cliente como en el servidor). Esto incluye los componentes que usa directamente, así como las dependencias anidadas.
--   Si el software es vulnerable, carece de soporte o no está actualizado. Esto incluye el sistema operativo, el servidor web/de aplicaciones, el sistema de administración de bases de datos (DBMS), las aplicaciones, las API y todos los componentes, los entornos de ejecución y las bibliotecas.
--   Si no analiza en búsqueda de vulnerabilidades de forma regular y no se suscribe a los boletines de seguridad relacionados con los componentes que utiliza.
--   Si no repara o actualiza la plataforma subyacente, frameworks y dependencias de manera oportuna y basada en el riesgo. Esto suele ocurrir en entornos en los que la aplicación de parches de seguridad es una tarea mensual o trimestral bajo control de cambios, lo que deja a las organizaciones abiertas a días o meses de exposición innecesaria a vulnerabilidades con soluciones disponibles.
--   Si los desarrolladores de software no testean la compatibilidad de las bibliotecas actualizadas, actualizadas o parcheadas.
--   Si no asegura las configuraciones de los componentes (consulte [A05:2021 – Configuración de Seguridad Incorrecta](A05_2021-Security_Misconfiguration.md)).</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 3           | 27.96%             | 8.77%              | 51.78%       | 22.47%       | 5.00                 | 5.00                | 30,457            | 0          |
-## How to prevent
-Debe existir un proceso de administración de parches que:
--   Elimine las dependencias que no son utilizadas, funcionalidades, componentes, archivos y documentación innecesarios.
--   Realice un inventario continuo de las versiones de los componentes en el cliente y en el servidor (por ejemplo, frameworks, bibliotecas) y sus dependencias utilizando herramientas como: versions, OWASP Dependency Check, retire.js, etc. Supervise continuamente fuentes como Common Vulnerability and Exposures (CVE) y National Vulnerability Database (NVD) para detectar vulnerabilidades en los componentes. Utilice herramientas de análisis de composición de software para automatizar el proceso. Suscríbase para recibir alertas por correo electrónico sobre vulnerabilidades de seguridad relacionadas con los componentes que utiliza.
--   Solo obtenga componentes de fuentes oficiales a través de enlaces seguros.
-    Prefiera los paquetes firmados para reducir la posibilidad de incluir un componente malicioso modificado (consulte [A08:2021 – Fallas en el Software y en la Integridad de los Datos](A08_2021-Software_and_Data_Integrity_Failures.md)).
--   Supervise las bibliotecas y los componentes que no sea mantenidos o no generen parches de seguridad para versiones anteriores. Si la aplicación de parches no es posible, considere implementar un parche virtual para monitorear, detectar o protegerse contra el problema descubierto.
-Toda organización debe garantizar un plan continuo para monitorear, clasificar y aplicar actualizaciones o cambios de configuración durante la vida útil de la aplicación o portafolio de aplicaciones.
-## Example attack scenarios
-**Escenario #1:** Los componentes normalmente se ejecutan con los mismos privilegios que la propia aplicación, por lo que las fallas en cualquier componente pueden tener un impacto grave. Tales fallas pueden ser accidentales (por ejemplo, error de codificación) o intencionales (por ejemplo, una puerta trasera en un componente). Algunos ejemplos de vulnerabilidades de componentes explotables descubiertos son:
--   CVE-2017-5638, una vulnerabilidad de ejecución remota de código de Struts 2 que permite la ejecución arbitraria de código en el servidor, ha sido culpada de brechas importantes.
--   Si bien el Internet de las Cosas (IoT) es con frecuencia difícil o imposible de parchear, la importancia de parchearlo puede ser grande (por ejemplo, dispositivos biomédicos).
-Existen herramientas automatizadas para ayudar a los atacantes a encontrar sistemas sin parches o mal configurados. Por ejemplo, el motor de búsqueda Shodan IoT puede ayudarlo a encontrar dispositivos que aún sufren la vulnerabilidad Heartbleed parchada en abril de 2014.
-Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2021/es/A06_2021-Vulnerable_and_Outdated_Components/</t>
   </si>
   <si>
     <t>Composants vulnérables et obsolètes</t>
@@ -3326,105 +2820,6 @@
     <t>Componentes Vulneráveis e Desatualizados</t>
   </si>
   <si>
-    <t>Você provavelmente está vulnerável:
-- Se você não souber as versões de todos os componentes que usa
-    (tanto do lado do cliente quanto do lado do servidor). Isso
-    inclui componentes que você usa diretamente, bem como
-    dependências aninhadas.
-- Se o software for vulnerável, sem suporte ou desatualizado.
-    Isso inclui o sistema operacional, servidor _web/application_,
-    sistema de gerenciamento de banco de dados (DBMS), aplicações,
-    APIs e todos os componentes, ambientes de tempo de execução e bibliotecas.
-- Se você não faz a varredura de vulnerabilidades regularmente e
-    não assina os boletins de segurança relacionados aos componentes que você usa.
-- Se você não corrigir ou atualizar a plataforma, as estruturas e as dependências
-    subjacentes de maneira oportuna e baseada em riscos. Isso geralmente acontece
-    em ambientes em que a correção é uma tarefa mensal ou trimestral sob controle
-    de alterações, deixando as organizações abertas a dias ou meses de exposição
-    desnecessária a vulnerabilidades corrigidas.
-- Se os desenvolvedores de software não testarem a compatibilidade de
-   bibliotecas atualizadas, atualizações ou com patches.
-- Se você não proteger as configurações dos componentes
-    (consulte [A05: 2021-Configuração Incorreta de Segurança](A05_2021-Security_Misconfiguration.md)).</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
-|:-------------:|:-------------------------:|:------------------------:|:--------------------------:|:-----------------------:|:----------------:|:---------------:|:--------------------:|:-------------:|
-| 3             | 27.96%                    | 8.77%                    | 51.78%                     | 22.47%                  | 5.00             | 5.00            | 30,457               | 0             |
-## How to prevent
-Deve haver um processo de gerenciamento de dependências para:
-- Remova dependências não utilizadas, recursos, componentes, arquivos
-    e documentação desnecessários.
-- Atualizar continuamente um inventário com as versões dos componentes
-    do lado do cliente e do lado do servidor (por exemplo, estruturas,
-    bibliotecas) e suas dependências usando ferramentas como _versions_,
-    _OWASP Dependency Check_, _retire.js_, etc. Monitore continuamente fontes
-    como _Common Vulnerability and Exposures_ (CVE) e _National Vulnerability
-    Database_ (NVD) para vulnerabilidades nos componentes. Use ferramentas
-    de análise de composição de software para automatizar o processo.
-    Inscreva-se para receber alertas de e-mail sobre vulnerabilidades de
-    segurança relacionadas aos componentes que você usa.
-- Obtenha componentes apenas de fontes oficiais por meio de links seguros.
-    Prefira pacotes assinados para reduzir a chance de incluir um componente
-    malicioso modificado (consulte
-    [A08: 2021-Software e Falhas de Integridade de Dados](A08_2021-Software_and_Data_Integrity_Failures.md)).
-- Monitore bibliotecas e componentes sem manutenção ou que não criem patches
-    de segurança para versões anteriores. Se o patch não for possível,
-    considere implantar um patch virtual para monitorar, detectar ou proteger
-    contra o problema descoberto.
-Cada organização deve garantir um plano contínuo de monitoramento, triagem e
-aplicação de atualizações ou alterações de configuração durante a vida
-útil da aplicação ou portfólio.
-## Example attack scenarios
-**Cenário #1:** Os componentes normalmente são executados com os mesmos
-privilégios da própria aplicação, portanto, as falhas em qualquer componente
-podem resultar em sério impacto. Essas falhas podem ser acidentais
-(por exemplo, erro de codificação) ou intencionais (por exemplo, uma
-_backdoor_ em um componente). Alguns exemplos de vulnerabilidades
-de componentes exploráveis descobertos são:
-- CVE-2017-5638, uma vulnerabilidade de execução remota de código
-    do Struts 2 que permite a execução de código arbitrário no servidor,
-    foi responsabilizada por violações significativas.
-- Embora a Internet das Coisas (IoT) seja frequentemente difícil ou
-    impossível de corrigir, a importância de corrigi-los pode ser
-    grande (por exemplo, dispositivos biomédicos).
-Existem ferramentas automatizadas para ajudar os invasores a encontrar
-sistemas não corrigidos ou configurados incorretamente. Por exemplo,
-o mecanismo de pesquisa Shodan IoT pode ajudá-lo a encontrar
-dispositivos que ainda sofrem com a vulnerabilidade Heartbleed
-corrigida em abril de 2014.
-Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A06_2021-Vulnerable_and_Outdated_Components/</t>
-  </si>
-  <si>
-    <t>Aşağıdaki durumlarda muhtemelen savunmasızsınız:
-* Kullandığınız tüm bileşenlerin (hem client-side hem de server-side) versiyonlarını bilmiyorsanız. Buna doğrudan kullandıklarınızın yanı sıra nested dependency’ler de dahildir.
-* Yazılım (OS, web/application server, database management system (DBMS), uygulamalar, APIs ve tüm bileşenler, runtime environment’lar ve kütüphaneler dâhil) savunmasız, desteklenmiyor veya güncel değilse.
-* Düzenli olarak zafiyet taraması yapmıyor ve kullandığınız bileşenlerle ilgili security bulletin’lere abone olmuyorsanız.
-* Temel platformu, framework’leri ve dependency’leri risk temelli ve zamanında düzeltmiyor veya upgrade etmiyorsanız. Bu genellikle patching’in aylık veya üç aylık bir change control görevi olduğu ortamlarda yaşanır ve kuruluşları düzeltilmiş zafiyetlere karşı günlerce veya aylarca gereksiz açıkta bırakır.
-* Yazılım geliştiriciler, güncellenmiş, upgrade edilmiş veya patch uygulanmış kütüphanelerin uyumluluğunu test etmiyorsa.
-* Bileşenlerin configuration’larını güvence altına almıyorsanız (bkz. [A05:2021-Security Misconfiguration](A05_2021-Security_Misconfiguration.md)).</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Max Coverage | Avg Coverage | Avg Weighted Exploit | Avg Weighted Impact | Total Occurrences | Total CVEs |
-| :---------: | :----------------: | :----------------: | :----------: | :----------: | :------------------: | :-----------------: | :---------------: | :--------: |
-|      3      |       27.96%       |        8.77%       |    51.78%    |    22.47%    |         5.00         |         5.00        |       30,457      |      0     |
-## How to prevent
-Aşağıdakileri kapsayan bir patch management süreci olmalıdır:
-* Kullanılmayan dependency’leri, gereksiz özellikleri, bileşenleri, dosyaları ve dokümantasyonu kaldırın.
-* Hem client-side hem de server-side bileşenlerin (örn. framework’ler, kütüphaneler) ve dependency’lerinin versiyonlarını sürekli olarak envanterleyin; versions, OWASP Dependency Check, retire.js vb. araçları kullanın. Common Vulnerabilities and Exposures (CVE) ve National Vulnerability Database (NVD) gibi kaynakları bileşenlerdeki zafiyetler için sürekli izleyin. Bu süreci otomatikleştirmek için software composition analysis araçlarını kullanın. Kullandığınız bileşenlerle ilgili security vulnerability e-posta uyarılarına abone olun.
-* Bileşenleri yalnızca resmi kaynaklardan ve güvenli bağlantılar üzerinden edinin. Değiştirilmiş, kötü amaçlı bir bileşen ekleme olasılığını azaltmak için imzalı paketleri tercih edin (bkz. [A08:2021-Software and Data Integrity Failures](A08_2021-Software_and_Data_Integrity_Failures.md)).
-* Bakımı yapılmayan veya eski versiyonlar için security patch üretmeyen kütüphane ve bileşenleri izleyin. Patching mümkün değilse, keşfedilen soruna karşı izleme, tespit veya koruma sağlayacak bir virtual patch uygulamayı değerlendirin.
-Her kuruluş, uygulamanın veya portföyün yaşam döngüsü boyunca izleme, önceliklendirme (triage) ve update/konfigürasyon değişikliklerini uygulamaya yönelik sürekli bir plan sağlamalıdır.
-## Example attack scenarios
-**Senaryo #1:** Bileşenler genellikle uygulamanın kendisiyle aynı ayrıcalıklarla çalıştığından, herhangi bir bileşendeki kusurlar ciddi etkilere yol açabilir. Bu kusurlar kazara (örn. coding error) veya kasıtlı (örn. bir bileşende backdoor) olabilir. Keşfedilmiş bazı istismar edilebilir bileşen zafiyetleri şunlardır:
-* CVE-2017-5638, server üzerinde arbitrary code execution’a imkân veren bir Struts 2 remote code execution zafiyeti, büyük ihlallerden sorumlu tutulmuştur.
-* Internet of Things (IoT) genellikle patch’lenmesi zor veya imkânsız olsa da, bunların patch’lenmesinin önemi büyük olabilir (örn. biyomedikal cihazlar).
-Saldırganların patch uygulanmamış veya misconfigured sistemleri bulmasına yardımcı olan otomatik araçlar vardır. Örneğin, Shodan IoT arama motoru, Nisan 2014’te patch’lenen Heartbleed zafiyetinden hâlâ etkilenen cihazları bulmanıza yardımcı olabilir.
-Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A06_2021-Vulnerable_and_Outdated_Components/</t>
-  </si>
-  <si>
     <t>易受攻击和已淘汰的组件(Vulnerable and Outdated Components)</t>
   </si>
   <si>
@@ -3467,27 +2862,6 @@
 - 虽然物联网 (IoT) 设备通常很难或无法修补，但修补它们可能有很高的重要性。 （例如，生物医学设备）。
 有一些自动化工具可以帮助攻击者找到未修补或配置错误的系统。例如，Shodan IoT 搜索引擎可以帮助您找到存在 2014 年 4 月未修补 Heartbleed 漏洞的设备。
 有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A06_2021-Vulnerable_and_Outdated_Components/</t>
-  </si>
-  <si>
-    <t>Confirmation of the user's identity, authentication, and session
-management is critical to protect against authentication-related
-attacks. There may be authentication weaknesses if the application:
--   Permits automated attacks such as credential stuffing, where the
-    attacker has a list of valid usernames and passwords.
--   Permits brute force or other automated attacks.
--   Permits default, weak, or well-known passwords, such as "Password1"
-    or "admin/admin".
--   Uses weak or ineffective credential recovery and forgot-password
-    processes, such as "knowledge-based answers," which cannot be made
-    safe.
--   Uses plain text, encrypted, or weakly hashed passwords data stores (see
-    [A02:2021-Cryptographic Failures](A02_2021-Cryptographic_Failures.md)).
--   Has missing or ineffective multi-factor authentication.
--   Exposes session identifier in the URL.
--   Reuse session identifier after successful login.
--   Does not correctly invalidate Session IDs. User sessions or
-    authentication tokens (mainly single sign-on (SSO) tokens) aren't
-    properly invalidated during logout or a period of inactivity.</t>
   </si>
   <si>
     <t>## Score table
@@ -3572,20 +2946,6 @@
     <t>Fehlerhafte Authentifizierung</t>
   </si>
   <si>
-    <t>Die Überprüfung der Identität des Nutzenden, die Authentifizierung und die Sitzungsverwaltung sind entscheidend für den Schutz vor authentifizierungsbezogenen Angriffen. Schwachstellen bei der Authentifizierung können auftreten, falls die Anwendung:
-- automatisierte Angriffe wie Credential Stuffing zulässt, bei dem Angreifende über eine Liste gültiger Usernamen und Passwörter verfügen.
-- Brute-Force- oder andere automatisierte Angriffe ermöglicht.
-- Standard-, schwache oder gängige Passwörter zulässt, wie z. B. "Passwort1" oder "admin/admin".
-- schwache oder ineffektive Verfahren zur Wiederherstellung von Anmeldeinformationen  und   Verfahren für vergessene Passwörtern, wie z. B. „wissensbasierte Antworten“, die nicht sicher gemacht werden können, 
-verwendet werden.
--  Klartext-, verschlüsselte oder schwach gehashte Kennwortdatenspeicher (siehe
-    [A02:2021-Cryptographic Failures](A02_2021-Cryptographic_Failures.md)) verwendet.
-- Fehlende oder unwirksame Multi-Faktor-Authentifizierung.
-- Die Session-ID wird in der URL angezeigt.
-- Session-IDs nach erfolgreichem Login wieder verwendet werden.
-- Session-IDs werden nicht korrekt ungültig gemacht. Sitzungen von Benutzenden (user sessions) oder Authentifizierungs-Tokens (hauptsächlich Single Sign-On (SSO) Tokens) werden beim Abmelden oder bei Inaktivität nicht ordnungsgemäß invalidiert.</t>
-  </si>
-  <si>
     <t>## Score table
 | Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -3608,18 +2968,6 @@
     <t>Fallas de Identificación y Autenticación</t>
   </si>
   <si>
-    <t>La confirmación de la identidad, la autenticación y la gestión de sesiones del usuario son fundamentales para protegerse contra ataques relacionados con la autenticación. Puede haber debilidades de autenticación si la aplicación:
--   Permite ataques automatizados como la reutilización de credenciales conocidas, donde el atacante posee una lista de pares de usuario y contraseña válidos.
--   Permite ataques de fuerza bruta u otros ataques automatizados.
--   Permite contraseñas por defecto, débiles o bien conocidas, como "Password1" o "admin/admin".
--   Posee procesos débiles o no efectivos para las funcionalidades de olvido de contraseña o recuperación de credenciales, como "respuestas basadas en el conocimiento", las cuales no se pueden implementar de forma segura.
--   Almacena las contraseñas en texto claro, cifradas o utilizando funciones de hash débiles (consulte [A02: 2021-Fallas Criptográficas](A02_2021-Cryptographic_Failures.md)).
--   No posee una autenticación multi-factor o la implementada es ineficaz.
--   Expone el identificador de sesión en la URL.
--   Reutiliza el identificador de sesión después de iniciar sesión.
--   No inválida correctamente los identificadores de sesión. Las sesiones de usuario o los tokens de autenticación (principalmente tokens de inicio de sesión único (SSO)) no son correctamente invalidados durante el cierre de sesión o luego de un período de inactividad.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom | Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -3641,18 +2989,6 @@
   </si>
   <si>
     <t>Identification et authentification de mauvaise qualité</t>
-  </si>
-  <si>
-    <t>La confirmation de l'identité, de l'authentification et de la session de l'utilisateur sont essentielles pour se protéger des attaques liées à l'authentification. Il peut y avoir des faiblesses d'authentification si l'application :
-- autorise les attaques automatisées telles que le bourrage des informations d'identification, où l'attaquant dispose d'une liste de noms d'utilisateurs valides et mots de passe ;
-- permet la force brute ou d'autres attaques automatisées ;
-- autorise les mots de passe par défaut, faibles ou bien connus, tels que "Password1" ou "admin / admin" ;
-- utilise des processus de récupération des informations d'identification faibles ou inefficaces et des processus de mot de passe oublié, tels que «&amp;nbsp;Questions secrètes&amp;nbsp;», qui ne peuvent être sécurisées ;
-- utilise des mots de passe en texte brut, chiffrés ou faiblement hachés (voir [A02:2021 – Défaillances cryptographiques](A02_2021-Cryptographic_Failures.md)) ;
-- absence ou utilisation inefficace de l’authentification multifacteur ;
-- exposition des identifiants de session dans l'URL ;
-- réutilisation de l'identifiant de session après une connexion réussie ;
-- n'invalide pas correctement les identifiants de session. Les sessions utilisateurs ou les jetons d'authentification (en particulier les jetons SSO) ne sont pas correctement invalidés lors de la déconnexion ou après une période d'inactivité.</t>
   </si>
   <si>
     <t>## Score table
@@ -3829,26 +3165,6 @@
     <t>Falhas de identificação e autenticação</t>
   </si>
   <si>
-    <t>Confirmação da identidade, autenticação e sessão do usuário
-gerenciamento é fundamental para proteger contra autenticação relacionada
-ataques. Pode haver pontos fracos de autenticação se o aplicativo:
-- Permite ataques automatizados, como preenchimento de credenciais, onde o
-     invasor tem uma lista de nomes de usuários e senhas válidos.
-- Permite força bruta ou outros ataques automatizados.
-- Permite senhas padrão, fracas ou conhecidas, como "Senha1" ou "admin/admin".
-- Usa recuperação de credenciais fraca ou ineficaz e esqueci a senha
-     processos, como "respostas baseadas em conhecimento", que não podem ser feitas
-     de modo seguro.
-- Usa armazenamento de dados e senhas em texto simples, criptografadas ou com hash fraco (consulte
-    [A02:2021-Falhas Criptográficas](A02_2021-Cryptographic_Failures.md)).
-- Possui multifator de autenticação ausente ou ineficaz.
-- Expõe o identificador de sessão na URL.
-- Reutiliza o identificador de sessão após o login bem-sucedido.
-- Não invalida corretamente IDs de sessão. Sessões de usuário ou
-     tokens de autenticação (principalmente tokens de logon único (SSO)) não são
-     devidamente invalidado durante o logout ou um período de inatividade.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -3882,18 +3198,6 @@
 Em vez de selecionar "sair", o usuário simplesmente fecha a aba do navegador e sai. 
 Uma hora depois, um atacante usa o mesmo navegador, e o usuário ainda está autenticado.
 Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A07_2021-Identification_and_Authentication_Failures/</t>
-  </si>
-  <si>
-    <t>Kullanıcının kimliğinin doğrulanması, authentication ve session yönetimi; authentication kaynaklı saldırılara karşı korunmak için kritiktir. Aşağıdaki durumlar varsa uygulamada authentication zafiyetleri olabilir:
--   Saldırganın geçerli username/password listeleriyle credential stuffing gibi otomatik saldırılar yapmasına izin veriyorsa.
--   Brute force veya diğer otomatik saldırılara izin veriyorsa.
--   “Password1” veya “admin/admin” gibi varsayılan, zayıf veya yaygın parolalara izin veriyorsa.
--   “Bilgiye dayalı sorular” gibi güvenli hâle getirilemeyen zayıf/hatalı credential recovery ve forgot-password süreçleri kullanılıyorsa.
--   Parolalar plain text, şifreli ama hatalı veya zayıf şekilde hash’lenmiş data store’larda tutuluyorsa (bkz. [A02:2021-Cryptographic Failures](A02_2021-Cryptographic_Failures.md)).
--   Multi-factor authentication eksik veya etkisizse.
--   Session identifier URL’de açığa çıkıyorsa.
--   Başarılı login’den sonra aynı session identifier yeniden kullanılıyorsa.
--   Session ID’ler doğru şekilde geçersiz kılınmıyorsa. Kullanıcı session’ları veya authentication token’ları (özellikle single sign-on (SSO) token’ları) logout sırasında veya belli bir inactivity süresinden sonra düzgün biçimde invalid edilmiyorsa.</t>
   </si>
   <si>
     <t>## Score table
@@ -4286,29 +3590,6 @@
 有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A08_2021-Software_and_Data_Integrity_Failures/</t>
   </si>
   <si>
-    <t>Returning to the OWASP Top 10 2021, this category is to help detect,
-escalate, and respond to active breaches. Without logging and
-monitoring, breaches cannot be detected. Insufficient logging,
-detection, monitoring, and active response occurs any time:
--   Auditable events, such as logins, failed logins, and high-value
-    transactions, are not logged.
--   Warnings and errors generate no, inadequate, or unclear log
-    messages.
--   Logs of applications and APIs are not monitored for suspicious
-    activity.
--   Logs are only stored locally.
--   Appropriate alerting thresholds and response escalation processes
-    are not in place or effective.
--   Penetration testing and scans by dynamic application security testing (DAST) tools (such as OWASP ZAP) do
-    not trigger alerts.
--   The application cannot detect, escalate, or alert for active attacks
-    in real-time or near real-time.
--   You are vulnerable to information leakage by making logging and alerting
-events visible to a user or an attacker (see [A01:2021-Broken Access Control](A01_2021-Broken_Access_Control.md)).
--   You are vulnerable to injections or
-    attacks on the logging or monitoring systems if log data is not correctly encoded.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4395,17 +3676,6 @@
     <t>Unzureichendes Logging und Sicherheitsmonitoring</t>
   </si>
   <si>
-    <t>Mit Blick auf die OWASP Top 10 2021 soll diese Kategorie bei der Erkennung, Eskalation und Reaktion auf laufende Angriffe unterstützen. Ohne Protokollierung und Überwachung können Angriffe nicht erkannt werden. Unzureichende Protokollierung, Erkennung, Überwachung und aktive Reaktion sind jederzeit möglich:
-- Nachvollziehbare Ereignisse, wie Anmeldungen, fehlgeschlagene Anmeldungen und wertvolle Transaktionen, werden nicht protokolliert.
-- Warnungen und Fehler erzeugen keine, unangemessene oder unklare Log-Einträge.
-- Die Logs von Anwendungen und APIs werden nicht auf verdächtige Aktivitäten überwacht.
-- Protokolle werden nur lokal gespeichert.
-- Geeignete Schwellenwerte für Warnmeldungen und Eskalationsprozesse für Gegenmaßnahmen sind nicht vorhanden oder nicht wirksam.
-- Penetrationstests und Scans durch DAST-Tools (Dynamic Application Security Testing) (wie OWASP ZAP) lösen keine Alarme aus.
-- Die Anwendungen können Angriffe weder in Echtzeit noch nahezu in Echtzeit erkennen, eskalieren oder Alarm schlagen.
-Es besteht die Gefahr von Informationslecks, falls Sie die Logging- und Alerting Ereignisse für Nutzende oder Angreifende sichtbar gemacht werden (siehe [A01:2021-Broken Access Control](A01_2021-Broken_Access_Control.md)).</t>
-  </si>
-  <si>
     <t>## Score table
 | Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4429,17 +3699,6 @@
     <t>Fallas en el Registro y Monitoreo</t>
   </si>
   <si>
-    <t>Volviendo al OWASP Top 10 2021, la intención es apoyar la detección, escalamiento y respuesta ante brechas activas. Sin registros y monitoreo, las brechas no pueden ser detectadas. Registros, detecciones, monitoreo y respuesta activas insuficientes pueden ocurrir en cualquier momento:
--   Eventos auditables, tales como los inicios de sesión, fallas en el inicio de sesión y transacciones de alto valor no son registradas.
--   Advertencias y errores generan registros poco claros, inadecuados y en algunos casos ni se generan.
--   Registros en aplicaciones y API no son monitoreados para detectar actividades sospechosas.
--   Los registros son únicamente almacenados en forma local.
--   Los umbrales de alerta y procesos de escalamiento no están correctamente implementados o no son efectivos.
--   Las pruebas de penetración y los escaneos utilizando herramientas de pruebas dinámicas de seguridad en aplicaciones (como ser OWASP ZAP) no generan alertas.
--   Las aplicaciones no logran detectar, escalar, o alertar sobre ataques activos en tiempo real ni cercanos al tiempo real.
-Se es vulnerable a la fuga de información haciendo registros y eventos de alertas que sean visibles para un usuario o un atacante (consulte [A01: 2021-Pérdida de Control de Acceso](A01_2021-Broken_Access_Control.md)).</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4461,17 +3720,6 @@
   </si>
   <si>
     <t>Carence des systèmes de contrôle et de journalisation</t>
-  </si>
-  <si>
-    <t>De retour dans le Top 10 2021 de l'OWASP, cette catégorie a pour but d'aider à la détection, à l'escalade et à la réponse aux brèches actives. Sans journalisation et surveillance, les brèches ne peuvent être détectées. Une journalisation, une détection, une surveillance et une réponse active insuffisantes peuvent survenir à tout moment :
-- les traces d’audit, telles que les accès réussis ou échoués et les transactions sensibles, ne sont pas enregistrées ;
-- les alertes et les erreurs générées ne sont pas enregistrées, ou leur journalisation est inadéquate, ou imprécise ;
-- les journaux des applications et des API ne sont pas contrôlés pour détecter les actions suspectes ;
-- les journaux ne sont stockés que localement ;
-- aucun processus de seuil d’alerte convenable ni de remontées d'information pour y répondre n'ont été définis, ou ils sont inadéquats, ou inefficaces ;
-- les tests d'intrusion et de balayage avec des outils de test dynamique de sécurité des applications (DAST), tels que OWASP ZAP, ne génèrent pas d'alertes ;
-- l’application est incapable de détecter, de générer des remontées d'information et des alertes en temps réel, ou assimilé, en cas d’attaque active.
-Vous êtes vulnérable à une fuite d’information en rendant les enregistrements de journalisation et d’alertes accessibles à vos utilisateurs ou attaquants (voir [A01:2021-Contrôles d'accès défaillants](A01_2021-Broken_Access_Control.md)).</t>
   </si>
   <si>
     <t>## Score table
@@ -4565,23 +3813,6 @@
 Untuk informasi lebih lanjut tentang referensi dan daftar CWE yang dipetakan: https://top10.owasp.org/2021/id/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
   </si>
   <si>
-    <t>Tornando alla Top 10 2021 di OWASP, questa categoria è per aiutare a rilevare,
-svolgere escalation e rispondere alle violazioni attive. Senza logging e
-monitoraggio, le violazioni non possono essere rilevate. Il logging,
-il rilevamento, il monitoraggio e la risposta attiva insufficienti si verificano ogni volta che:
--   Gli eventi verificabili, come i login, i login falliti e le transazioni ad alto valore, non vengono registrati.
--   Warning ed errori non generano messaggi di log, oppure sono inadeguati o poco chiari.
--   I log di applicazioni e API non sono monitorati per attività sospette.
--   I file di log vengono memorizzati solo localmente.
--   Non sono presenti o sono inefficaci le soglie di allarme e processi di escalation della risposta
--   I penetration test e le scansioni da parte di strumenti DAST (Dynamic Application Security Testing) (come OWASP ZAP) 
-    non attivano nessun allarme.
--   L'applicazione non è in grado di rilevare, svolgere escalation o avvisare per gli attacchi attivi
-    in real-time o quasi in real-time. 
-Si è vulnerabili alla fuga di informazioni se gli eventi di logging e gli alert sono
-visibili ad un utente o ad un attaccante (vedi [A01:2021-Broken Access Control](A01_2021-Broken_Access_Control.md)).</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs corrispondenti | Tasso di incidenza Max | Tasso di incidenza Medio | Sfruttabilità pesata | Impatto Medio | Copertura Max | Copertura media | Occorrenze Totali | CVE Totali |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4630,19 +3861,6 @@
     <t>セキュリティログとモニタリングの失敗</t>
   </si>
   <si>
-    <t>OWASP Top 10 2021 に話を戻すと、このカテゴリは、アクティブな違反の検出、エスカレーション、および対応を支援するものです。
-ロギングとモニタリングがなければ、侵害を検知することはできません。
-ロギングや検知、モニタリング、適時の対応が十分に行われないという状況は、いつでも発生します:
--   ログイン、失敗したログイン、重要なトランザクションなどの監査可能なイベントがログに記録されていない。
--   警告とエラーが発生してもログメッセージが生成されない、または不十分、不明確なメッセージが生成されている。
--   アプリケーションとAPIのログが、疑わしいアクティビティをモニタリングしていない。
--   ログがローカルにのみ格納されている。
--   アラートの適切なしきい値とレスポンスのエスカレーションプロセスが整えられていない、または有効ではない。
--   ペネトレーションテストやDAST(dynamic application security testing)ツール（OWASP ZAPなど）によるスキャンがアラートをあげない。
--   アプリケーションがリアルタイム、準リアルタイムにアクティブな攻撃を検知、エスカレート、またはアラートすることができない。
-ユーザまたは攻撃者がログやアラートのイベントを閲覧できると、情報の漏えいが発生する可能性があります ([A01:2021-アクセス制御の不備](A01_2021-Broken_Access_Control.md) を参照).</t>
-  </si>
-  <si>
     <t>## Score table
 | 対応する CWE 数 | 最大発生率 | 平均発生率 |  加重平均（攻撃の難易度） | 加重平均（攻撃による影響） | 最大網羅率 | 平均網羅率 | 総発生数 | CVE 合計件数 |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4678,6 +3896,1115 @@
     <t>Falhas de registro e monitoramento de segurança</t>
   </si>
   <si>
+    <t>## Score table
+| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 4           | 19.23%             | 6.51%              | 6.87                 | 4.99                | 53.67%       | 39.97%       | 53,615            | 242        |
+## How to prevent
+Os desenvolvedores devem implementar alguns ou todos os controles a seguir, dependendo do risco da aplicação:
+- Garantir que todas as falhas de login, controle de acesso e validação de entrada no lado do servidor possam ser registradas com contexto de usuário suficiente para identificar contas suspeitas ou maliciosas e mantidas por tempo suficiente para permitir análise forense atrasada.
+- Garantir que os logs sejam gerados em um formato que as soluções de gerenciamento de logs possam facilmente consumir.
+- Garantir que os dados de log sejam codificados corretamente para evitar injeções ou ataques nos sistemas de registro ou monitoramento.
+- Garantir que transações de alto valor tenham uma trilha de auditoria com controles de integridade para evitar adulteração ou exclusão, como tabelas de banco de dados somente para adição ou similares.
+- As equipes de DevSecOps devem estabelecer monitoramento e alerta efetivos para que atividades suspeitas sejam detectadas e respondidas rapidamente.
+- Estabelecer ou adotar um plano de resposta e recuperação de incidentes, como o National Institute of Standards and Technology (NIST) 800-61r2 ou posterior.
+Existem estruturas de proteção de aplicativos comerciais e de código aberto, como o OWASP ModSecurity Core Rule Set, e software de correlação de logs de código aberto, como o Elasticsearch, Logstash, Kibana (ELK) stack, que possuem painéis personalizados e alertas.
+## Example attack scenarios
+**Cenário 1:** O operador do site do provedor de plano de saúde infantil não conseguiu detectar uma violação devido à falta de monitoramento e registro. Uma parte externa informou ao provedor do plano de saúde que um invasor havia acessado e modificado milhares de registros de saúde sensíveis de mais de 3,5 milhões de crianças. Uma revisão pós-incidente descobriu que os desenvolvedores do site não haviam abordado vulnerabilidades significativas. Como não houve registro ou monitoramento do sistema, a violação de dados pode ter estado em andamento desde 2013, um período de mais de sete anos.
+**Cenário 2:** Uma grande companhia aérea indiana teve uma violação de dados envolvendo dados pessoais de milhões de passageiros por mais de dez anos, incluindo dados de passaporte e cartão de crédito. A violação de dados ocorreu em um provedor de hospedagem em nuvem de terceiros, que notificou a companhia aérea da violação depois de algum tempo.
+**Cenário nº 3:** Uma grande companhia aérea europeia sofreu uma violação relatável do GDPR. A violação foi supostamente causada por vulnerabilidades de segurança do aplicativo de pagamento exploradas por invasores, que colheram mais de 400.000 registros de pagamento de clientes. A companhia aérea foi multada em 20 milhões de libras como resultado pelo regulador de privacidade.
+Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
+| :---------: | :----------------: | :----------------: | :------------------: | :-----------------: | :----------: | :----------: | :---------------: | :--------: |
+|      4      |       19.23%       |        6.51%       |         6.87         |         4.99        |    53.67%    |    39.97%    |       53,615      |     242    |
+## How to prevent
+Uygulamanın riskine bağlı olarak geliştiriciler aşağıdaki kontrollerin bir kısmını veya tamamını uygulamalıdır:
+* Tüm login, access control ve server-side input validation hatalarının; şüpheli veya kötü niyetli hesapları tanımlayacak yeterli user context ile log’lanmasını ve gecikmeli adli analiz (forensic analysis) için yeterince uzun süre tutulmasını sağlayın.
+* Log’ların, log management çözümlerinin kolayca tüketebileceği bir formatta üretilmesini sağlayın.
+* Logging veya monitoring sistemlerine injection/saldırıları önlemek için log verisini doğru şekilde encode edin.
+* Yüksek değerli işlemler için, kurcalamayı (tampering) veya silmeyi önleyecek integrity kontrollerine sahip audit trail (ör. append-only database tabloları) sağlayın.
+* DevSecOps ekipleri, şüpheli aktivitelerin hızlıca tespit edilip yanıtlanacağı etkili monitoring ve alerting kurmalıdır.
+* National Institute of Standards and Technology (NIST) 800-61r2 veya daha yenisi gibi bir incident response ve recovery planı oluşturun veya benimseyin.
+OWASP ModSecurity Core Rule Set gibi ticari ve açık kaynak uygulama koruma framework’leri ile Elasticsearch, Logstash, Kibana (ELK) stack gibi açık kaynak log korelasyon yazılımları; custom dashboard ve alerting özellikleri sunar.
+## Example attack scenarios
+**Senaryo #1:** Bir çocuk sağlık planı sağlayıcısının web sitesi işletmecisi, monitoring ve logging eksikliği nedeniyle bir ihlali tespit edemedi. Harici bir taraf, saldırganın 3.5 milyonun üzerinde çocuğa ait binlerce hassas sağlık kaydına erişip bunları değiştirdiğini bildirdi. Olay sonrası incelemede, web sitesi geliştiricilerinin önemli zafiyetleri ele almadığı görüldü. Sistem üzerinde logging veya monitoring olmadığından, veri ihlali 2013’ten beri — yedi yılı aşkın bir süre — devam ediyor olabilirdi.
+**Senaryo #2:** Büyük bir Hint havayolu şirketi, milyonlarca yolcunun on yılı aşkın kişisel verilerini (pasaport ve kredi kartı verileri dâhil) etkileyen bir veri ihlali yaşadı. Veri ihlali, üçüncü taraf bir cloud hosting sağlayıcısında meydana geldi ve ihlal bir süre sonra havayoluna bildirildi.
+**Senaryo #3:** Büyük bir Avrupa havayolu şirketi GDPR kapsamında raporlanabilir bir ihlal yaşadı. İhlalin, saldırganlar tarafından istismar edilen payment application güvenlik zafiyetlerinden kaynaklandığı ve 400.000’den fazla müşteri ödeme kaydının toplandığı bildirildi. Havayolu, gizlilik düzenleyicisi tarafından 20 milyon pound para cezasına çarptırıldı.
+Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
+  </si>
+  <si>
+    <t>在 2021 年 OWASP Top 10，此类型有助于对进行中资安事件之侦测，升级及应变。缺乏记录及监控时无法侦测资安事件发生。不足地记录，侦测，监控及主动应变随时会发生：
+- 可稽核事件未记录，如登入成功，登入失败及高价值交易。
+- 警告或错误发生时未产生，产生不充足或产生不明确日志。
+- 未监控应用程式或应用程式介面(API)日志中的可疑活动。
+- 日志仅储存于本地端。
+- 未设有或设有无效之适当告警阀值及应变升级程序。
+- 渗透测试及 DAST 工具(如 OWASP ZAP)扫描没有触发告警。
+- 应用程式无法接近即时或即时侦测，升级或警告进行中之攻击。
+允许使用者或攻击者读取日志或告警事件可能早成资讯泄漏(参考 A01:2021 权限控制失效)</t>
+  </si>
+  <si>
+    <t>## Score table
+| 可对照 CWEs 数量 | 最大发生率 | 平均发生率 | 最大覆盖范围 | 平均覆盖范围 | 平均加权漏洞 | 平均加权影响 | 总发生数 | 相关 CVEs 总数量 |
+| :--------------: | :--------: | :--------: | :----------: | :----------: | :----------: | :----------: | :------: | :--------------: |
+|        4         |   19.23%   |   6.51%    |    53.67%    |    39.97%    |     6.87     |     4.99     |  53,615  |       242        |
+## How to prevent
+开发者应依据应用程式所面临风险实作下列部分或全部的控制项：
+- 确保记录所有登入，存取控制及服务器端输入验证之失败，日志应包含充足使用者情境以识别可疑或恶意帐号，日志应存留充足时间以利未来可能之鉴识分析要求。
+- 确保日志格式符合一般日志管理系统常用格式。
+- 确保日志经正确编码以防止遭受注入攻击或日志/监控系统遭受攻击。
+- 确保高价值交易进行时产生稽核轨迹(日志)并实作完整性控制以避免窜改或删除，如仅限附加的资料表或类似工具。
+- DevSecOps 团队应建立有效地监控及告警机制以利侦测可疑活动并快速应变。
+- 建立或导入事件应变及复原计画，如 NIST 800-61r2 或更新版本。
+现有多种商业化及开放原始码应用程式保护架构，如 OWASP ModSecurity Core Rule Set 及开放原始码日志关联软体可客制化仪表板及告警，如 ELK stack。
+## Example attack scenarios
+**情境 1**：一家儿童健康计划供应商的网站运营商因缺乏监控和记录无法侦测资安事件。外部通知该健康计划供应商，攻击者已存取及修改超过 350 万名儿童的敏感健康记录。事后审查发现网站开发者没有处理重大弱点。由于系统没有记录或监控，资料泄漏可能从 2013 年开始至今，时间超过七年。
+**情境 2**：印度一家大型航空公司发生涉及数百万乘客超过十年包括护照及信用卡资料等个人资料的资料泄漏。资料泄漏发生在第三方供应商提供的云端服务，该供应商在资料泄漏发生一段时间后通知航空公司。
+情境 3：一家大型欧洲航空公司发生依 GDPR 应报告之个资事故。据报导，攻击者利用支付应用系统之安全漏洞，取得超过 40 万笔客户支付纪录。该航空公司遭隐私主管机关裁罚两千万英镑。
+有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
+  </si>
+  <si>
+    <t>Server-Side Request Forgery (SSRF)</t>
+  </si>
+  <si>
+    <t>SSRF flaws occur whenever a web application is fetching a remote
+resource without validating the user-supplied URL. It allows an attacker
+to coerce the application to send a crafted request to an unexpected
+destination, even when protected by a firewall, VPN, or another type of
+network access control list (ACL).
+As modern web applications provide end-users with convenient features,
+fetching a URL becomes a common scenario. As a result, the incidence of
+SSRF is increasing. Also, the severity of SSRF is becoming higher due to
+cloud services and the complexity of architectures.</t>
+  </si>
+  <si>
+    <t>تزوير الطلبات من جانب الخادم SSRF</t>
+  </si>
+  <si>
+    <t>يتم تزوير طلبات الخادم عندما يقوم تطبيق الويب بجلب موارد عن بعد دون عملية التحقّق من صحة العنوان المقدّم من قِبل المستخدم، حيث يسمح ذلك للمهاجم بإجبار التطبيق على إرسال طلب معدّل إلى وجهة غير متوقعة للخادم، حتى عندما يكون محميّ بجدار حماية، أو شبكة خاصة افتراضية VPN أو أية نوع من قائمة التحكم بالوصول إلى الشبكة.
+نظرًا لأن تطبيقات الويب (المواقع الإلكترونية) الحديثة توفّر للمستخدمين مُميزات متقدّمة، فإن جلب العناوين من الخادم أصبح سيناريو شائع. نتيجة لذلك، فإن معدّل حدوث تزوير لطلبات الخادم آخذ في الازدياد، لذلك أصبح استغلال هذه الثغرة أشد خطورة على الخادم عندما ظهرت الخدمات السحابيّة وكذلك تعقيد البنية التحتيّة.</t>
+  </si>
+  <si>
+    <t>## Score table
+| ربطها مع CWEs | الحد الأقصى للحدوث | متوسط معدل الحدوث | التغطية القصوى | متوسط معدل التغطية | متوسط استغلال الثغرات | متوسط التأثير | إجمالي التكرار | إجمالي نقاط الضعف CVEs |
+|---------------|--------------------|-------------------|----------------|--------------------|-----------------------|---------------|----------------|------------------------|
+| 1             | 2.72%              | 2.72%             | 67.72%         | 67.72%             | 8.28                  | 6.72          | 9,503          | 385                    |
+## How to prevent
+يستطيع المُطوّرين منع تزوير طلبات الخادم بتنفيذ بعض أو كل وسائل الدفاع التالية في ضوابط الدفاع العميق (Defense in Depth) :
+## **من خلال طبقات الشبكة**
+-   تقسيم وظائف الوصول إلى الموارد عن بعد في شبكات مُنفصلة لتقليل تأثير تزوير طلبات الخادم.
+-   فرض سياسات جدار الحماية "الرفض افتراضيًا" أو ضبط آليات التحكّم في الوصول إلى الشبكة لحظر جميع حركات المرور للشبكة الداخلية باستثناء حركات المرور الأساسية.
+## **من خلال طبقات التطبيقات**
+-   التصّفية والتحقّق من صحة جميع بيانات الإدخال المقدّمة من قِبل المستخدم.
+-   استخدام عناوين محدّدة في الروابط، URL استخدام منافذ محدّدة مع تحديد قائمة من العناوين المحدّدة مسبقًا في قائمة مسموح بها.
+-   لا تقم برد الطلبات للعميل على شكل بيانات خام
+-   قم بتعطيل إعادة التوجيه إلى HTTP.
+-   كن على حذر من هجمات إعادة الترتيب الرابط أو الأحرف والتي قد تأتي في بعض الهجمات من خلال بروتوكول DNS أو من خلال استخدام TOCTOU.
+لا تقم بتخفيف المخاطر على هجمات SSRF من خلال استخدام سياسة المنع المبنيّة على قائمة التعبيرات المنطقية أو (Regular Expression). حيث أن المهاجمين لديهم قوائم مُعدّة مسبقًا ومتعدّدة لمحاولة تخطّي عمليات الحجب تلك.
+## Example attack scenarios
+يستطيع المهاجمين استخدام تزوير طلبات الخادم لمهاجمة الأنظمة المحميّة خلف جدران حماية تطبيقات الويب(WAF)، وجدران الحماية أو قائمة التحكّم للوصول للشبكة باستخدام سيناريو مثل:
+**سيناريو #1:** فحص المنافذ للخوادم الداخلية في معمارية الشبكة:
+الشبكات الغير مقسّمة بشكل جيّد تُمكّن المهاجمين من رسم الشبكات الداخلية بشكل دقيق ويصل إلى تمكين المهاجم لمعرفة في حال كانت المنافذ مفتوحة أم مُغلقة للخوادم والخدمات الداخلية من خلال دراسة أو استجابة الخادم لطلبات أو من خلال الوقت المُستغرق لكل طلب على كل منفذ مختلف وذلك لمعرفة في حال كان استغلال SSRF نجح أم فشل.
+**سيناريو #2:** بيانات حساسة غير محميّة والتي يستطيع المهاجم الوصول إليها:
+يستطيع المهاجم الوصول للبيانات الحساسة الداخلية مثل ملف (  file:///etc/passwd)أو حتى للخدمات الداخلية من خلال استغلال هذه الثغرة
+**سيناريو #3:** الوصول إلى تخزين البيانات الوصفيّة للخدمات السحابيّة :
+يمتلك معظم موفرّي السحابة تخزين البيانات الوصفيّة مثل http://169.254.169.254    ويمكن للمهاجم قراءة تلك البيانات الوصفيّة للحصول على معلومات حساسة منها.
+**سيناريو #4:** اختراق الخدمات الداخلية وإساءة استخدامها من قِبل المهاجم:
+يمكن للمهاجم إساءة استخدام الخدمات الداخلية لإجراء مزيد من الهجمات مثل تنفيذ التعليمات البرمجية عن بُعد (RCE) أو هجوم حجب الخدمة (DoS).
+لمزيد من المعلومات حول المراجع وقائمة CWE المعيّنة: https://top10.owasp.org/2021/ar/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
+  </si>
+  <si>
+    <t>SSRF-Schwachstellen treten immer dann auf, wenn eine Webanwendung eine Remote-Ressource abruft, ohne die, vom Nutzenden angegebene URL zu überprüfen. Dadurch kann ein Angreifender die Anwendung dazu zwingen, eine manipulierte Anfrage an ein unerwartetes Ziel zu senden, selbst wenn sie durch eine Firewall, ein VPN oder eine andere Art von Netzwerkzugriffskontrollliste (ACL) geschützt ist.
+Da moderne Webanwendungen Nutzenden komfortable Funktionen bieten, wird das Abrufen einer URL zu einem gängigen Szenario. 
+Infolgedessen nimmt die Häufigkeit von SSRF zu. 
+Außerdem nimmt der Schweregrad von SSRF aufgrund von der Verbreitung von Cloud-Diensten und der Komplexität der Architekturen zu.</t>
+  </si>
+  <si>
+    <t>Falsificación de Solicitudes del Lado del Servidor (SSRF)</t>
+  </si>
+  <si>
+    <t>Las fallas de SSRF ocurren cuando una aplicación web está obteniendo un recurso remoto sin validar la URL proporcionada por el usuario. Permite que un atacante coaccione a la aplicación para que envíe una solicitud falsificada a un destino inesperado, incluso cuando está protegido por un firewall, VPN u otro tipo de lista de control de acceso a la red (ACL).
+Dado que las aplicaciones web modernas brindan a los usuarios finales funciones convenientes, la búsqueda de una URL se convierte en un escenario común. Como resultado, la incidencia de SSRF está aumentando. Además, la gravedad de SSRF es cada vez mayor debido a los servicios en la nube y la complejidad de las arquitecturas.</t>
+  </si>
+  <si>
+    <t>A10 Falsification de requête côté serveur (SSRF)</t>
+  </si>
+  <si>
+    <t>Une faille SSRF se produit lorsqu'une application web récupère une ressource distante sans valider l'URL fournie par l'utilisateur. Elle permet à un attaquant de contraindre l'application à envoyer une requête élaborée à une destination inattendue, même si elle est protégée par un pare-feu, un VPN ou un autre type de liste de contrôle d'accès au réseau (ACL).
+Comme les applications Web modernes offrent aux utilisateurs finaux des fonctions pratiques, la récupération d'une URL devient un scénario courant. Par conséquent, l'incidence d'une SSRF augmente. De même, la gravité de ce phénomène augmente en raison des services en nuage et de la complexité des architectures.</t>
+  </si>
+  <si>
+    <t>Kecacatan _SSRF_ muncul saat sebuah aplikasi web meminta _remote resource_ tanpa melakukan validasi URL yang di berikan oleh pengguna. Ini memperbolehkan penyerang untuk memaksa aplikasi untuk mengirim _crafted request_ ke destinasi yang tidak diharapkan, meskipun sudah dilindungi oleh _firewall_, VPN, atau tipe lain dari daftar aturan akses jaringan - _Access Control List_ (ACL).
+Aplikasi web saat ini menyediakan fitur yang nyaman bagi pengguna akhir, sehingga proses meminta URL menjadi hal yang lumrah. Oleh karena itu, insiden _SSRF_ semakin meningkat. Selain itu, tingkat keparahan _SSRF_ semakin meningkat karena layanan-layanan _cloud_ dan tingkat komplexitas arsitektur _cloud_.</t>
+  </si>
+  <si>
+    <t>Le falle SSRF si verificano ogni volta che un'applicazione web recupera una risorsa remota
+senza validare l'URL fornito dall'utente. Questo permette ad un attaccante
+di forzare l'applicazione ad inviare una richiesta preparata ad hoc ad una destinazione inattesa, 
+anche quando è protetta da un firewall, una VPN o un altro tipo di
+network access control list (ACL).
+Dato che le moderne applicazioni web forniscono agli utenti finali parecchie funzionalità,
+scaricare dati da un URL è uno scenario comune. Di conseguenza, l'incidenza di
+SSRF è in crescita. Inoltre, la gravità di SSRF sta diventando più alta a causa dei
+servizi cloud e alla complessità crescente delle architetture.</t>
+  </si>
+  <si>
+    <t>サーバーサイドリクエストフォージェリ (SSRF)</t>
+  </si>
+  <si>
+    <t>SSRFの欠陥は、Webアプリケーション上からリモートのリソースを取得する際に、ユーザーから提供されたURLを検証せずに使用することで発生します。
+ファイアウォールやVPNあるいはその他の種類のネットワークアクセス制御リスト(ACL)によってアプリケーションが保護されている場合であっても、SSRFによりアプリケーションに対して意図しない宛先へ細工されたリクエストを強制的に発行させることができます。
+モダンなアプリケーションではエンドユーザーに便利な機能を提供するようになり、アプリケーション側でURLを取得することは珍しい状況ではなくなりました。
+そのためSSRFの発生が増加しています。
+またSSRFの深刻度も、クラウドサービスやアーキテクチャの複雑性を背景として、段々と大きくなりつつあります。</t>
+  </si>
+  <si>
+    <t>Falsificação de Solicitação do Lado do Servidor (SSRF)</t>
+  </si>
+  <si>
+    <t>As falhas de SSRF ocorrem sempre que um aplicativo da web busca um recurso remoto sem validar a URL fornecida pelo usuário. Ele permite que um invasor force o aplicativo a enviar uma solicitação criada para um destino inesperado, mesmo quando protegido por um firewall, VPN ou outro tipo de lista de controle de acesso à rede (ACL).
+Como os aplicativos da web modernos fornecem aos usuários finais recursos convenientes, buscar uma URL se torna um cenário comum. Como resultado, a incidência de SSRF está aumentando. Além disso, a gravidade do SSRF está se tornando mais alta devido aos serviços em nuvem e à complexidade crescente das arquiteturas.</t>
+  </si>
+  <si>
+    <t>SSRF hataları, bir web uygulaması kullanıcı tarafından sağlanan URL’yi doğrulamadan uzak bir kaynağı fetch ettiğinde ortaya çıkar. Bu, saldırganın uygulamayı, firewall, VPN veya başka bir network access control list (ACL) ile korunuyor olsa bile beklenmeyen bir hedefe crafted bir istek göndermeye zorlamasına imkân tanır.
+Modern web uygulamaları son kullanıcılara kullanışlı özellikler sundukça, bir URL’i fetch etmek yaygın bir senaryo hâline gelir. Sonuç olarak, SSRF’nin görülme sıklığı artıyor. Ayrıca cloud servisleri ve mimarilerin karmaşıklığı nedeniyle SSRF’nin ciddiyeti de yükseliyor.</t>
+  </si>
+  <si>
+    <t>当网页应用程式正在取得远端资源，却未验证由使用者提供的网址，此时就会发生伪造服务端请求。即便有防火墙、VPN 或其他网路 ACL 保护的情况下，攻击者仍得以强迫网页应用程式发送一个经过捏造的请求给一个非预期的目的端。
+现今的网页应用程式提供终端使用者便利的特色，取得网址已经是常见的了。因此，伪造服务端请求的发生率是在增加当中的。而且，因为云端服务和云端结构的复杂性，伪造服务端请求的严重性将会愈来愈严峻。</t>
+  </si>
+  <si>
+    <t>## Score table
+| 可对照 CWEs 数量 | 最大发生率 | 平均发生率 |最大覆盖范围 | 平均覆盖范围 | 平均加权漏洞 | 平均加权影响 | 出现次数 | 所有相关 CVEs 数量 |
+| :-------------: | :------: | :------: | :--------: | :--------: | :---------: | :--------: | :-----: | :--------------: |
+| 1 | 2.72% | 2.72% | 67.72% | 67.72% | 8.28 | 6.72 | 9,503 | 385 |
+## How to prevent
+开发者可以预防伪造服务端请求，透过实施下列一部分或全部的纵身防御控制措施：
+## **From Network layer** (从网路层着手)
+- 将远端资源存取功能切割成不同子网路以降低伪造服务端请求之冲击
+- 于防火墙政策或于网路存取控制规则实施"预设全拒绝(deny by default)" ，以封锁全部来自外部之网路流量
+## **From Application layer:** (从应用层)
+- 过滤并验证来自于用户端提供之全部输入
+- 以正面表列方式列出 URL、port、目的地清单
+- 不传送原始回应给用户端
+- 停用 HTTP 重新导向
+- 留意网址之一致性，以避免例如 DNS rebinding 攻击、TOCTOU 攻击
+别透过拒绝清单或正规表示式来减缓伪造服务端请求。攻击者有 payload 清单、工具和技巧可以绕过这些拒绝清单
+## Example attack scenarios
+攻击者可以利用伪造服务端请求来攻击在 WAF、防火墙、或网路 ACL 后面的系统，可能采取之情境如下：
+**情境一**：对内部服务器 port scan。如果网路架构未被切割，攻击者可以透过连线结果或连线所经过的时间或拒绝 SSRF payload 连线的状态，加以对应出内部网路并且判断该等 port 在内部服务器是否开启或关闭状态
+**情境二**：机敏资料泄漏。攻击者可以存取本地端档案(例如 &lt;file:///etc/passwd&gt;) 或内部服务已取得机敏资料。
+**情境三**：存取云服务之 metadata storage。大部分云端提供者都有 metadata storage，例如&lt;http://169.254.169.254/&gt;。攻击者可以读取 metadata 以取得机敏资讯。
+**情境四**：渗透内部服务 - 攻击者可以滥用内部服务去执行更进一步的攻击，例如 RCE 或 Dos
+有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
+  </si>
+  <si>
+    <t>annotation</t>
+  </si>
+  <si>
+    <t>name[ar]</t>
+  </si>
+  <si>
+    <t>description[ar]</t>
+  </si>
+  <si>
+    <t>annotation[ar]</t>
+  </si>
+  <si>
+    <t>name[de]</t>
+  </si>
+  <si>
+    <t>description[de]</t>
+  </si>
+  <si>
+    <t>annotation[de]</t>
+  </si>
+  <si>
+    <t>name[es]</t>
+  </si>
+  <si>
+    <t>description[es]</t>
+  </si>
+  <si>
+    <t>annotation[es]</t>
+  </si>
+  <si>
+    <t>name[fr]</t>
+  </si>
+  <si>
+    <t>description[fr]</t>
+  </si>
+  <si>
+    <t>annotation[fr]</t>
+  </si>
+  <si>
+    <t>name[id]</t>
+  </si>
+  <si>
+    <t>description[id]</t>
+  </si>
+  <si>
+    <t>annotation[id]</t>
+  </si>
+  <si>
+    <t>name[it]</t>
+  </si>
+  <si>
+    <t>description[it]</t>
+  </si>
+  <si>
+    <t>annotation[it]</t>
+  </si>
+  <si>
+    <t>name[ja]</t>
+  </si>
+  <si>
+    <t>description[ja]</t>
+  </si>
+  <si>
+    <t>annotation[ja]</t>
+  </si>
+  <si>
+    <t>name[pt]</t>
+  </si>
+  <si>
+    <t>description[pt]</t>
+  </si>
+  <si>
+    <t>annotation[pt]</t>
+  </si>
+  <si>
+    <t>name[tr]</t>
+  </si>
+  <si>
+    <t>description[tr]</t>
+  </si>
+  <si>
+    <t>annotation[tr]</t>
+  </si>
+  <si>
+    <t>name[zh]</t>
+  </si>
+  <si>
+    <t>description[zh]</t>
+  </si>
+  <si>
+    <t>annotation[zh]</t>
+  </si>
+  <si>
+    <t>OWASP Top 10 Web - 2021</t>
+  </si>
+  <si>
+    <t>مرحبًا بكم في أحدث إصدار من أعلى عشرة مخاطر من منظمة أواسب وهي النسخة الحديثة لعام 2021، والتي تأتي بشكل جديد تمامًا ومدعمة برسومات انفوجرافيك التي تستطيع طباعتها واستخدامها ويمكن الحصول عليها من صفحتنا الرئيسية.
+المصدر: https://top10.owasp.org/2021/ar/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>¡Bienvenido a la última entrega del OWASP Top 10! El OWASP Top 10 2021 ha sido totalmente renovado, con un nuevo diseño gráfico y una infografía de una sola página que puedes imprimir u obtener desde nuestra página web.
+Fuente: https://top10.owasp.org/2021/es/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>Bienvenue à cette nouvelle édition de l'OWASP Top 10 ! L'OWASP Top 10 2021 apporte de nombreux changements, avec notamment une nouvelle interface et une nouvelle infographie, disponible sur un format d'une page qu'il est possible de se procurer depuis notre page d'accueil.
+Source: https://top10.owasp.org/2021/fr/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>Selamat datang ke versi terakhir dari OWASP Top 10! OWASP Top 10 2021 semua baru, dengan desain grafis baru dan suatu infografis satu-halaman yang dapat Anda cetak atau dapatkan dari beranda kami.
+Sumber: https://top10.owasp.org/2021/id/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>Ecco a voi l'ultima versione della OWASP Top 10! La OWASP Top 10 2021 è tutta nuova, con un nuovo design grafico e un'infografica di una pagina che potete stampare o scaricare dalla nostra home page.
+Fonte: https://top10.owasp.org/2021/it/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>OWASP トップ 10 の最新版へようこそ! OWASP トップ 10 2021年版は、グラフィックデザインが一新され、1ページのインフォグラフィックになっています。インフォグラフィックは、ホームページから入手でき、印刷することができます。
+出典: https://top10.owasp.org/2021/ja/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>Bem-vindo à última edição do OWASP Top 10! O OWASP Top 10 2021 é totalmente novo, com um novo design gráfico e um infográfico  disponível que você pode imprimir ou obter em nossa página inicial.
+Fonte: https://top10.owasp.org/2021/pt-BR/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>OWASP Top 10’un en güncel sürümüne hoş geldiniz! OWASP Top 10 2021 tamamen yenilendi; yeni bir grafik tasarım ve ana sayfamızdan indirebileceğiniz ya da çıktısını alabileceğiniz tek sayfalık bir infografik ile geliyor.
+Kaynak: https://top10.owasp.org/2021/tr/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>欢迎來到最新版本的 OWASP Top 10！! OWASP Top 10 2021 是一个全新的名单，包含了你可以打印下來的新图示说明，若有需要的话，你可以从我们的网页上面下载。
+來源: https://top10.owasp.org/2021/zh-Hant/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>Willkommen zur neuesten Ausgabe der OWASP Top 10! Die OWASP Top 10:2021 sind völlig neu, mit einem neuen Grafikdesign mit Piktogrammen je Risiko und Mobilgeräte-freundlichen Webseiten.
+Quelle: https://top10.owasp.org/2021/de/A00_2021_Introduction/</t>
+  </si>
+  <si>
+    <t>The application might be vulnerable if the application is:
+-   Missing appropriate security hardening across any part of the
+    application stack or improperly configured permissions on cloud
+    services.
+-   Unnecessary features are enabled or installed (e.g., unnecessary
+    ports, services, pages, accounts, or privileges).
+-   Default accounts and their passwords are still enabled and
+    unchanged.
+-   Error handling reveals stack traces or other overly informative
+    error messages to users.
+-   For upgraded systems, the latest security features are disabled or
+    not configured securely.
+-   The security settings in the application servers, application
+    frameworks (e.g., Struts, Spring, ASP.NET), libraries, databases,
+    etc., are not set to secure values.
+-   The server does not send security headers or directives, or they are
+    not set to secure values.
+-   The software is out of date or vulnerable (see **A06:2021-Vulnerable and Outdated Components**).
+Without a concerted, repeatable application security configuration
+process, systems are at a higher risk.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
+## How to prevent
+Secure installation processes should be implemented, including:
+-   A repeatable hardening process makes it fast and easy to deploy
+    another environment that is appropriately locked down. Development,
+    QA, and production environments should all be configured
+    identically, with different credentials used in each environment.
+    This process should be automated to minimize the effort required to
+    set up a new secure environment.
+-   A minimal platform without any unnecessary features, components,
+    documentation, and samples. Remove or do not install unused features
+    and frameworks.
+-   A task to review and update the configurations appropriate to all
+    security notes, updates, and patches as part of the patch management
+    process (see **A06:2021-Vulnerable and Outdated Components**). Review
+    cloud storage permissions (e.g., S3 bucket permissions).
+-   A segmented application architecture provides effective and secure
+    separation between components or tenants, with segmentation,
+    containerization, or cloud security groups (ACLs).
+-   Sending security directives to clients, e.g., Security Headers.
+-   An automated process to verify the effectiveness of the
+    configurations and settings in all environments.
+## Example attack scenarios
+**Scenario #1:** The application server comes with sample applications
+not removed from the production server. These sample applications have
+known security flaws attackers use to compromise the server. Suppose one
+of these applications is the admin console, and default accounts weren't
+changed. In that case, the attacker logs in with default passwords and
+takes over.
+**Scenario #2:** Directory listing is not disabled on the server. An
+attacker discovers they can simply list directories. The attacker finds
+and downloads the compiled Java classes, which they decompile and
+reverse engineer to view the code. The attacker then finds a severe
+access control flaw in the application.
+**Scenario #3:** The application server's configuration allows detailed
+error messages, e.g., stack traces, to be returned to users. This
+potentially exposes sensitive information or underlying flaws such as
+component versions that are known to be vulnerable.
+**Scenario #4:** A cloud service provider (CSP) has default sharing
+permissions open to the Internet by other CSP users. This allows
+sensitive data stored within cloud storage to be accessed.
+For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2021/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>Die Anwendung besitzt möglicherweise Schwachstellen, wenn folgendes zutrifft:
+- Mangelhafte Sicherheitshärtung des Anwendungsstacks oder ungeeignet konfigurierte Berechtigungen auf Cloud-Diensten.
+- Nicht benötigte Features sind aktiviert oder installiert (z. B. unnötige Ports, Dienste, Seiten, Accounts oder Rechte).
+- Standardkonten und -passwörter sind aktiviert bzw. unverändert.
+- Die Fehlerbehandlung gibt Stack-Traces oder andere interne technische Fehlermeldungen an Anwendende preis.
+- Für aktualisierte Systeme sind die neuesten Sicherheitsfeatures deaktiviert oder nicht sicher konfiguriert.
+- Die Sicherheitseinstellungen in den Anwendungsservern und -frameworks (z. B. Struts, Spring, ASP.NET), Bibliotheken, Datenbanken etc. sind nicht auf sichere Werte gesetzt.
+- Der Server sendet keine Sicherheits-Header oder -Direktiven, bzw. diese sind nicht sicher konfiguriert.
+- Die Software ist veraltet oder verwundbar (siehe **A06:2021-Unsichere oder veraltete Komponenten**).
+Ohne einen abgestimmten und reproduzierbaren Prozess zur sicheren Konfiguration sind Systeme einem höheren Risiko ausgesetzt!</t>
+  </si>
+  <si>
+    <t>## Score table
+| Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 20          | 19.84 %             | 4.51 %              | 8.12                 | 6.56                | 89.58 %       | 44.84 %       | 208,387           | 789        |
+## How to prevent
+Es sollten sichere Installationsprozesse implementiert werden, darunter:
+- Ein wiederholbarer Härtungsprozess ermöglicht die schnelle und einfache Bereitstellung zusätzlicher Umgebungen, die entsprechend abgesichert sind. Entwicklungs-, Qualitätssicherungs- und Produktionsumgebungen sollten alle identisch konfiguriert sein, wobei in jeder Umgebung unterschiedliche Anmeldeinformationen verwendet werden sollten. Dieser Prozess sollte automatisiert werden, um den Aufwand für die Einrichtung einer neuen sicheren Umgebung zu minimieren.
+- Eine minimale Plattform ohne unnötige Funktionen, Komponenten, Dokumentation und Beispiele: Entfernen Sie Funktionen und Frameworks die Sie nicht verwenden oder installieren Sie diese erst gar nicht.
+- Überprüfen und Aktualisieren der Konfigurationen, die für alle Sicherheitshinweise, Updates und Patches im Rahmen des Patch-Verwaltungsprozesses geeignet sind (siehe **A06:2021-Unsichere oder veraltete Komponenten**). Überprüfen Sie die Cloud-Speicherberechtigungen (z. B. S3-Bucket-Berechtigungen).
+- Eine segmentierte Anwendungsarchitektur sorgt durch Segmentierung, Containerisierung oder Cloud-Sicherheitsgruppen (ACLs) für eine effektive und sichere Trennung zwischen Komponenten oder Mandanten.
+- Senden von Sicherheitsanweisungen an Clients, z. B. Sicherheits-Header.
+- Ein automatisierter Prozess zur Überprüfung der Wirksamkeit der Konfigurationen und Einstellungen in allen Umgebungen.
+## Example attack scenarios
+**Szenario Nr. 1:** Der Anwendungsserver wird mit Beispielanwendungen geliefert, die nicht vom Produktionsserver entfernt wurden. Diese Beispielanwendungen weisen bekannte Sicherheitslücken auf, die Angreifende nutzen, um den Server zu gefährden. Angenommen, eine dieser Anwendungen ist die Admin-Konsole und die Standardkonten wurden nicht geändert. In diesem Fall meldet sich die angreifende Person mit Standardkennwörtern an und übernimmt die Kontrolle.
+**Szenario Nr. 2:** Die Directory Listings wurden auf dem Server nicht deaktiviert. Angreifende entdecken, dass Verzeichnisse einfach aufgelistet werden können. Die angreifende Person findet die kompilierten Java-Klassen und lädt sie herunter, dekompiliert sie und betreibt Reverse Engineering, um den Code anzuzeigen. Dies ermöglicht das Findet eines schwerwiegenden Fehlers in der Zugriffskontrolle in der Anwendung.
+**Szenario Nr. 3:** Die Konfiguration des Anwendungsservers ermöglicht die Rückgabe detaillierter Fehlermeldungen an Anwendende, z. B. Stack-Traces. Dadurch werden möglicherweise vertrauliche Informationen oder zugrunde liegende Fehler wie Komponentenversionen offengelegt, die bekanntermaßen anfällig sind.
+**Szenario Nr. 4:** Ein Cloud-Dienstanbieter (CSP) enthält Standardfreigaben, die aus dem Internet für andere Cloud-Nutzende erreichbar sind und ermöglicht dadurch Zugriff auf sensitive Daten in der Cloud.
+Weitere Informationen zu den Referenzen und zur Liste der zugeordneten CWEs: https://top10.owasp.org/2021/de/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>La aplicación puede ser vulnerable si:
+-   Le falta el *hardening* de seguridad adecuado en cualquier parte del *stack tecnológico* o permisos configurados incorrectamente en los servicios en la nube.
+-   Tiene funciones innecesarias habilitadas o instaladas (puertos, servicios, páginas, cuentas o privilegios innecesarios, por ejemplo).
+-   Las cuentas predeterminadas y sus contraseñas aún están habilitadas y sin cambios.
+-   El manejo de errores revela a los usuarios rastros de pila u otros mensajes de error demasiado informativos.
+-   Para sistemas actualizados, las últimas funciones de seguridad están deshabilitadas o no configuradas de forma segura.
+-   Las configuraciones de seguridad en los servidores de aplicaciones, frameworks de aplicaciones (Struts, Spring o ASP.NET por ejemplo), bibliotecas, bases de datos, etc., no poseen configurados valores seguros.
+-   El servidor no envía encabezados o directivas de seguridad, o no poseen configurados valores seguros.
+-   El software está desactualizado o es vulnerable (consulte **A06:2021-Componentes Vulnerables y Desactualizados**).
+Sin un proceso de configuración de seguridad de aplicaciones coordinado y repetible, los sistemas corren un mayor riesgo.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
+## How to prevent
+Deben implementarse procesos de instalación seguros, incluyendo:
+-   Un proceso de *hardening* repetible agiliza y facilita la implementación de otro entorno que esté debidamente inaccesible. Los entornos de desarrollo, control de calidad y producción deben configurarse de forma idéntica, con diferentes credenciales utilizadas en cada uno.
+    Este proceso debe automatizarse para minimizar el esfuerzo necesario para configurar un nuevo entorno seguro.
+-   Una plataforma mínima sin funciones, componentes, documentación ni ejemplos innecesarios. Elimine o no instale características y frameworks no utilizados.
+-   Una tarea para revisar y actualizar las configuraciones apropiadas para todas las notas de seguridad, actualizaciones y parches como parte del proceso de administración de parches (consulte **A06: 2021-Componentes Vulnerables y Desactualizados**). Revise los permisos de almacenamiento en la nube (por ejemplo, Permisos de bucket de S3).
+-   Una arquitectura de aplicación segmentada proporciona una separación efectiva y segura entre componentes o instancias, con segmentación, organización en contenedores o grupos de seguridad en la nube (ACLs).
+-   Envío de directivas de seguridad a los clientes, por ejemplo, encabezados de seguridad.
+-   Un proceso automatizado para verificar la efectividad de las configuraciones y ajustes en todos los entornos.
+## Example attack scenarios
+**Escenario #1:** El servidor de aplicaciones contiene aplicaciones de ejemplo que no se eliminan del servidor de producción. Estas aplicaciones de ejemplo poseen fallas de seguridad conocidas que los atacantes utilizan para comprometer el servidor. Supongamos que una de estas aplicaciones es la consola de administración y no se modificaron las cuentas predeterminadas. En ese caso, el atacante inicia sesión con las contraseñas predeterminadas y toma el control.
+**Escenario #2:** El listado de directorios no se encuentra deshabilitado en el servidor. Un atacante descubre que simplemente puede enumerar directorios. El atacante detecta y descarga las clases Java compiladas, que decompila y aplica ingeniería inversa para ver el código. El atacante luego encuentra una falla severa de control de acceso en la aplicación.
+**Escenario #3:** La configuración del servidor de aplicaciones permite que se retornen a los usuarios mensajes de error detallados, por ejemplo, trazas de pila(stack traces). Esto potencialmente expone información confidencial o fallas subyacentes, como versiones de componentes que se sabe son vulnerables.
+**Escenario #4:** Un proveedor de servicios en la nube (CSP) posee permisos de uso compartido predeterminados abiertos a Internet a otros usuarios. Esto permite acceder a los datos confidenciales almacenados en el almacenamiento en la nube.
+Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2021/es/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>L'application peut être vulnérable si :
+-   elle n'a pas fait l'objet d'un durcissement de la sécurité approprié sur l'ensemble des couches protocolaires applicatives, ou si les permissions sont mal configurées sur les services cloud ;
+-   des fonctionnalités inutiles sont activées ou installées (ex : des ports, des services, des pages, des comptes ou des privilèges inutiles) ;
+-   les comptes par défaut et leurs mots de passe sont toujours activés et inchangés ;
+-   le traitement des erreurs révèle aux utilisateurs des traces des piles protocolaires ou d'autres messages d'erreur laissant transpirer trop d'informations ;
+-   pour les systèmes à jour ou mis à niveau, les dernières fonctionnalités de sécurité sont désactivées ou ne sont pas configurées de manière sécurisée ;
+-   les paramètres de sécurité dans les serveurs d'application, les frameworks applicatifs (ex : Struts, Spring, ASP.NET), les bibliothèques, les bases de données, etc. ne sont pas paramétrés avec des valeurs correctes du point de vue de la sécurité ;
+-   le serveur n'envoie pas d'en-têtes ou de directives de sécurité, ou s'ils ne sont pas paramétrés avec des valeurs correctes du point de vue de la sécurité ;
+-   La version du logiciel est obsolète ou vulnérable (voir **A06:2021-Composants vulnérables et obsolètes**).
+Sans un processus concerté et répétable de configuration de la sécurité des applications, les systèmes courent un risque plus élevé.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs associées | Taux d'incidence max | Taux d'incidence moyen | Exploitation pondérée moyenne | Impact pondéré moyen | Couverture max | Couverture moyenne | Nombre total d'occurrences | Nombre total de CVEs |
+|:--------------:|:--------------------:|:----------------------:|:-----------------------------:|:--------------------:|:--------------:|:------------------:|:--------------------------:|:--------------------:|
+|       20       |       19,84 %        |         4,51 %         |             8,12              |         6,56         |    89,58 %     |      44,84 %       |          208 387           |         789          |
+## How to prevent
+Des processus d'installation sécurisés doivent être mis en œuvre, avec notamment :
+- un processus de durcissement répétable qui permette de déployer rapidement et facilement un autre environnement correctement sécurisé avec une configuration verrouillée. Les environnements de développement, d'assurance qualité et de production doivent tous être configurés de manière identique, avec des droits différents pour chaque environnement. Ce processus devrait être automatisé afin de réduire au minimum les efforts requis pour mettre en place un nouvel environnement sécurisé ;
+- une plate-forme minimale sans fonctionnalité, composant, documentation et échantillon inutile. Supprimer ou ne pas installer des fonctionnalités et frameworks inutilisés ;
+- une tâche pour revoir et mettre à jour les configurations appropriées à tous les avis de sécurité, toutes les mises à jour et tous les correctifs dans le cadre du processus de gestion des correctifs (voir **A06:2021-Composants vulnérables et obsolètes**). En particulier, examiner les permissions de stockage dans le Cloud (ex. les permissions des buckets AWS S3) ;
+- une architecture d'application segmentée qui fournit une séparation efficace et sécurisée entre les composants ou les environnements hébergés, avec de la segmentation, de la mise en conteneurs ou l'utilisation de groupes de sécurité dans le Cloud (ACL) ;
+- l'envoi de directives de sécurité aux clients, par exemple [En-têtes de sécurité](https://wiki.owasp.org/index.php/OWASP_Secure_Headers_Project) ;
+- un processus automatisé pour vérifier l'efficacité des configurations et des réglages dans tous les environnements.
+## Example attack scenarios
+**Scénario 1** : Le serveur d'application est livré avec des applications classiques qui ne sont pas supprimées du serveur mis en production. Ces mêmes applications ont des failles de sécurité connues que les attaquants utilisent afin de compromettre le serveur. Si l'une de ces applications est la console d'administration, et que les comptes par défaut n'ont pas été modifiés, l'attaquant se connecte avec les mots de passe par défaut et prend la main sur la cible.
+**Scénario 2** : La fonctionnalité de listage des répertoires n'est pas désactivée sur le serveur. Un attaquant découvre qu'il peut simplement lister les répertoires. L'attaquant trouve et télécharge les classes Java compilées, qu'il décompose et fait de l'ingénierie inversée pour visualiser le code. L'attaquant trouve alors un grave défaut dans le contrôle d'accès de l'application.
+**Scénario 3** : La configuration du serveur d'application permet de renvoyer aux utilisateurs des messages d'erreur détaillés, par exemple avec des traces des couches protocolaires applicatives. Cela peut ainsi exposer des informations sensibles ou des vulnérabilités sous-jacentes telles que les versions de composants dont on sait qu'elles sont vulnérables.
+**Scénario 4** : Un fournisseur de services Cloud (CSP) a positionné des droits de partage par défaut qui sont ouverts sur Internet par d'autres utilisateurs du CSP. Cela permet d'accéder à des données sensibles stockées dans le stockage Cloud.
+Pour plus d’informations sur les références et la liste des CWE mappées : https://top10.owasp.org/2021/fr/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>L'applicazione potrebbe risultare vulnerabile se:
+-   Manca l'hardening di sicurezza appropriato in qualsiasi parte dello
+    stack applicativo o permessi configurati in modo improprio sui servizi
+    cloud.
+-   Sono abilitate o installate funzioni non necessarie (ad es.
+    porte, servizi, pagine, account o privilegi non necessari).
+-   Gli account di default sono ancora abilitati e presentano password predefinite.
+-   A seguito di condizioni di errore, vengono rivelate agli utenti stack traces o altri messaggi  di errore troppo verbosi.
+-   Per i sistemi aggiornati, le ultime funzionalità di sicurezza sono disabilitate o
+    non configurate in modo adeguato.
+-   Le impostazioni di sicurezza negli application server, nei framework
+    (ad esempio, Struts, Spring, ASP.NET), nelle librerie, database, ecc. non sono configurate su valori sicuri.
+-   Il server non invia header o direttive di sicurezza o non sono impostati su valori sicuri.
+-   Il software non è aggiornato o è vulnerabile (vedere **A06:2021-Vulnerable and Outdated Components**).
+Senza un processo coordinato e ripetibile per la configurazione della sicurezza delle applicazioni, 
+i sistemi presentano un rischio maggiore.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs corrispondenti | Tasso di incidenza Max | Tasso di incidenza Medio | Sfruttabilità pesata | Impatto Medio | Copertura Max | Copertura media | Occorrenze Totali | CVE Totali |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 20          | 19.84%             | 4.51%              | 8.12                 | 6.56                | 89.58%       | 44.84%       | 208,387           | 789        |
+## How to prevent
+Dovrebbero essere implementati processi di installazione sicuri, tra cui:
+-   Un processo di hardening ripetibile rende veloce e facile il deploy di
+    un altro ambiente preconfigurato in modo sicuro. Gli ambienti di sviluppo,
+    QA e di produzione dovrebbero essere tutti configurati in modo speculare, con credenziali diverse per ogni ambiente.
+    Questo processo dovrebbe essere automatizzato per minimizzare lo sforzo richiesto per
+    impostare un nuovo ambiente configurato in modo sicuro.
+-   Una piattaforma minimale senza funzionalità,componenti,
+    documentazione ed esempi inutili. Rimuovere o non installare funzionalità e
+    framework inutilizzati.
+-   Un task per rivedere e aggiornare le configurazioni appropriate a tutte le
+    security notes, aggiornamenti e patch come parte del processo di gestione delle patch
+    (vedere **A06:2021-Vulnerable and Outdated Components**). Revisionare
+    i permessi del cloud storage (ad esempio, i permessi dei bucket S3).
+-   Un'architettura applicativa segmentata fornisce un'efficace e sicura
+    separazione tra componenti o tenant, con segmentazione,
+    containerizzazione, o cloud security groups (ACL).
+-   L'invio di direttive di sicurezza ai client, ad esempio, i Security Headers.
+-   Un processo automatizzato per verificare l'efficacia delle
+    configurazioni e impostazioni in tutti gli ambienti.
+## Example attack scenarios
+**Scenario #1:** L'application server viene fornito con applicazioni di esempio
+non rimosse dal server di produzione. Queste applicazioni di esempio hanno
+falle di sicurezza note che gli attaccanti usano per compromettere il server. Supponiamo che una
+di queste applicazioni sia la console di amministrazione e che gli account predefiniti non siano stati cambiati. In questo caso, l'attaccante accede con le password predefinite e
+prende il controllo.
+**Scenario #2:** La funzionalità di directory listing non è disabilitata sul server. Un
+attaccante scopre che si possono elencare tutte le directory. L'attaccante trova
+e scarica le classi Java compilate, su cui esegue la decompilazione e il reverse engineering per visualizzare il codice sorgente. L'attaccante trova poi una grave
+difetto di controllo degli accessi nell'applicazione.
+**Scenario #3:** La configurazione dell'application server permette di restituire agli utenti
+messaggi di errore dettagliati, ad esempio la stack trace. Questa problematica
+potenzialmente espone informazioni sensibili o problematiche come
+versioni dei componenti che sono note per essere vulnerabili.
+**Scenario #4:** Un cloud service provider ha dei permessi di condivisione predefiniti
+aperti a Internet da altri utenti nell'header Content Security Policy (CSP). Questo permette
+l'accesso ai dati sensibili memorizzati nel cloud storage.
+Per maggiori informazioni sui riferimenti e sull'elenco delle CWE mappate: https://top10.owasp.org/2021/it/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>アプリケーションが下記のようなら、恐らく脆弱です:
+-   アプリケーションスタックのいずれかの部分におけるセキュリティ堅牢化の不足、あるいはクラウドサービスでパーミッションが不適切に設定されている
+-   必要のない機能が有効、あるいはインストールされている(例えば、必要のないポートやサービス、ページ、アカウント、特権)
+-   デフォルトのアカウントとパスワードが有効になったまま変更されていない
+-   エラー処理がユーザに対して、スタックトレースやその他余計な情報を含むエラーメッセージを見せる
+-   アップグレードしたシステムでは、最新のセキュリティ機能が無効になっているか正しく設定されていない
+-   アプリケーションサーバやアプリケーションフレームワーク(例えば、Struts、Spring、 ASP.NET)、ライブラリ、データベース等のセキュリティの設定が、安全な値に設定されていない
+-   サーバがセキュリテイヘッダーやディレクティブを送らなかったり、安全な値に設定されていなかったりする
+-   ソフトウェアが古いか脆弱である。(**# A06:2021 – 脆弱で古くなったコンポーネント** を参照)
+アプリケーションのセキュリティを設定するプロセスを協調して繰り返すことができなければ、システムはより高いリスクにさらされます。</t>
+  </si>
+  <si>
+    <t>## Score table
+| 対応する CWE 数 | 最大発生率 | 平均発生率 |  加重平均（攻撃の難易度） | 加重平均（攻撃による影響） | 最大網羅率 | 平均網羅率 | 総発生数 | CVE 合計件数 |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 20          | 19.84%             | 4.51%              | 89.58%       | 44.84%       | 8.12                 | 6.56                | 208,387           | 789        |
+## How to prevent
+安全にインストールするプロセスにおいて、以下のことを実施すべきです:
+-   繰り返し堅牢化するプロセスは、素早くかつ容易に他の環境に展開され、正しくロックダウンすること。
+    開発やQA、本番環境は完全に同じように設定し、それぞれの環境で別々の認証情報を使用すること。
+    このプロセスを自動化し、新しい安全な環境をセットアップする際には、手間を最小限にすること。
+-   プラットフォームは最小限のものとし、必要のない機能やコンポーネント、ドキュメント、サンプルを除くこと。
+    使用しない機能とフレームワークは、削除もしくはインストールしないこと。
+-   レビューを実施して、セキュリティ関連の記録と更新の全てに加え、パッチを管理するプロセスの一環としてパッチの設定を適切に更新すること(**# A06:2021 – 脆弱で古くなったコンポーネント** を参照)。
+    クラウドストレージのパーミッションは、詳細にレビューすること (例えば、S3 バケットのパーミッション)。
+-   セグメント化したアプリケーションアーキテクチャは、セグメンテーションやコンテナリゼーション、クラウドのセキュリティグループ(ACL)をともなったコンポーネントやテナント間に、効果的で安全な仕切りをもたらす。
+-   セキュリティディレクティブをクライアントへ送ること。例としては セキュリティヘッダー が挙げられる。
+-   プロセスを自動化して設定の有効性を検証し、環境すべてに適用すること。
+## Example attack scenarios
+**シナリオ #1:** 
+アプリケーションのサンプルが付属しているアプリケーションサーバであるにもかかわらず、プロダクションサーバからサンプルが削除されていません。
+このサンプルアプリケーションには、攻撃者がサーバに侵入する際によく使う既知の脆弱性があります。
+そのアプリケーションが管理用のコンソールでデフォルトのアカウントが変更されていないと、攻撃者はデフォルトのパスワードを使ってログインし、乗っ取ってしまいます。
+**シナリオ #2:** 
+ディレクトリリスティングがサーバ上で無効になっていません。攻撃者はそれを見つけ出し、やすやすとディレクトリを表示してしまいます。
+攻撃者はコンパイル済みのJavaクラスを見つけてダウンロードし、デコンパイルしてからリバースエンジニアリングしてコードを見ます。
+そして攻撃者は、そのアプリケーションの深刻なアクセス制御上の穴を見つけます。
+**シナリオ #3:** 
+アプリケーションサーバの設定が、詳細なエラーメッセージ(例えば、スタックトレース)をユーザに返すようになっています。
+これによって機微な情報や脆弱であるとされているコンポーネントのバージョンといった潜在的な欠陥がさらされる恐れがあります。
+**シナリオ #4:** 
+クラウドサービスプロバイダ (CSP) は、他のCSPユーザによるデフォルトでインターネットに公開された共有パーミッションを用意しています。
+こうなると、機微な情報がクラウドストレージに保存され、アクセスされてしまいます。
+参考資料およびマッピングされたCWEの一覧について、詳しくはこちら： https://top10.owasp.org/2021/ja/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>A aplicação pode ser vulnerável se for:
+- Falta de proteção de segurança apropriada em qualquer parte
+    da _stack_ das aplicações ou permissões configuradas incorretamente
+    em serviços em nuvem.
+- Recursos desnecessários são ativados ou instalados (por exemplo,
+    portas, serviços, páginas, contas ou privilégios desnecessários).
+- As contas padrão e suas senhas ainda estão ativadas e inalteradas.
+- O tratamento de erros revela _stack traces_ ou outras
+    mensagens de erro excessivamente informativas aos usuários.
+- Para sistemas atualizados, os recursos de segurança mais recentes
+    estão desabilitados ou não estão configurados com segurança.
+- As configurações de segurança nos servidores das aplicações, nos
+    _frameworks_ (por exemplo, Struts, Spring, ASP.NET), bibliotecas,
+    bancos de dados, etc., não estão definidas para proteger os valores.
+- O servidor não envia cabeçalhos ou diretivas de segurança, ou eles
+    não estão configurados para proteger os valores.
+- O software está desatualizado ou vulnerável (consulte
+  **A06: 2021-Componentes Vulneráveis e Desatualizados**).
+Sem um processo de configuração de segurança de aplicações que seja integrado e
+repetível, os sistemas correm um risco maior.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
+|:-------------:|:-------------------------:|:------------------------:|:--------------------------:|:-----------------------:|:----------------:|:---------------:|:--------------------:|:-------------:|
+| 20            | 19.84%                    | 4.51%                    | 8.12                       | 6.56                    | 89.58%           | 44.84%          | 208,387              | 789           |
+## How to prevent
+Devem ser implementados processos de instalação segura, incluindo:
+- Um processo de proteção repetível torna mais rápido e fácil implantar
+    outro ambiente que esteja devidamente bloqueado. Os ambientes de
+    desenvolvimento, controle de qualidade e produção devem ser todos
+    configurados de forma idêntica, com credenciais diferentes usadas
+    em cada ambiente. Este processo deve ser automatizado para minimizar
+    o esforço necessário para configurar um novo ambiente seguro.
+- Uma plataforma mínima sem recursos, componentes, documentação e outros
+    desnecessários. Remova ou não instale recursos e estruturas não utilizados.
+- Uma tarefa para revisar e atualizar as configurações apropriadas para todas
+    as notas de segurança, atualizações e patches como parte do processo de
+    gerenciamento de patch (consulte
+    **A06: 2021-Componentes Vulneráveis e Desatualizados**).
+    Revise as permissões de armazenamento em nuvem (por exemplo, _S3 bucket permissions_).
+- Uma arquitetura de aplicação segmentada fornece separação eficaz e
+    segura entre componentes ou _tenants_, com segmentação,
+    conteinerização ou grupos de segurança em nuvem (ACLs).
+- Envio de diretivas de segurança para clientes, por exemplo, _Security Headers_.
+- Um processo automatizado para verificar a eficácia das configurações
+    em todos os ambientes.
+## Example attack scenarios
+**Cenário #1:** O servidor da aplicação é fornecido com os sistemas de amostra
+não removidos do servidor de produção. Esses aplicativos de amostra têm
+falhas de segurança conhecidas que os invasores usam para comprometer o
+servidor. Suponha que um desses aplicativos seja o console de administração
+e as contas padrão não tenham sido alteradas. Nesse caso, o invasor
+efetua login com as senhas padrão e assume o controle.
+**Cenário #2:** A listagem do diretório não está desabilitada no servidor.
+Um invasor descobre que pode simplesmente listar diretórios. O invasor
+encontra e baixa as classes Java compiladas, que ele descompila e
+faz engenharia reversa para visualizar o código. O invasor então
+encontra uma falha grave de controle de acesso no aplicativo.
+**Cenário #3:** A configuração do servidor de aplicações permite que os
+detalhes das mensagens de erro, por exemplo, _stack trace_, sejam retornadas
+aos usuários. Isso potencialmente expõe informações confidenciais ou falhas
+subjacentes, como versões de componentes que são conhecidas por serem vulneráveis.
+**Cenário #4:** Um provedor de serviços de nuvem tem permissões de
+compartilhamento padrão abertas para a Internet por outros usuários de
+_Content Security Policy header (CSP)_. Isso permite que dados confidenciais
+armazenados no armazenamento em nuvem sejam acessados.
+Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>Uygulama aşağıdaki durumlarda zafiyete açık olabilir:
+* Application stack’in herhangi bir bölümünde uygun security hardening eksikse veya cloud servislerinde izinler yanlış konfigüre edildiyse.
+* Gereksiz özellikler etkinleştirilmiş ya da kurulmuşsa (ör. gereksiz port’lar, servisler, sayfalar, hesaplar veya ayrıcalıklar).
+* Varsayılan hesaplar ve bunların parolaları hâlâ etkin ve değişmemişse.
+* Error handling, kullanıcıya stack trace’ler veya aşırı bilgi içeren hata mesajları gösteriyorsa.
+* Yükseltilmiş sistemlerde, en yeni security özellikleri devre dışıysa veya güvenli şekilde konfigüre edilmemişse.
+* Application server’ları, application framework’leri (ör. Struts, Spring, ASP.NET), kütüphaneler, veritabanları vb. içindeki security ayarları güvenli değerlere set edilmemişse.
+* Server, security header’ları veya directive’leri göndermiyorsa ya da bunlar güvenli değerlere set edilmemişse.
+* Yazılım güncel değilse veya zafiyetliyse (bkz. **A06:2021 – Vulnerable and Outdated Components**).
+Planlı ve tekrarlanabilir bir application security configuration süreci olmadan sistemler daha yüksek risk altındadır.</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Eşleştirildi | Maks Görülme Oranı | Ort. Görülme Oranı | Ort. Ağırlıklı Exploit | Ort. Ağırlıklı Impact | Maks Coverage | Ort. Coverage | Toplam Olay | Toplam CVE |
+| :---------------: | :----------------: | :----------------: | :--------------------: | :-------------------: | :-----------: | :-----------: | :---------: | :--------: |
+|         20        |       19.84%       |        4.51%       |          8.12          |          6.56         |     89.58%    |     44.84%    |   208,387   |     789    |
+## How to prevent
+Güvenli kurulum süreçleri uygulanmalıdır; bunlar şunları içerir:
+* Tekrarlanabilir bir hardening süreci, uygun şekilde kilitlenmiş başka bir ortamın hızlı ve kolay şekilde deploy edilmesini sağlar. Development, QA ve production ortamları aynı şekilde konfigüre edilmeli; her ortamda farklı credential’lar kullanılmalıdır. Yeni güvenli bir ortam kurulumunda eforu minimize etmek için bu süreç otomatikleştirilmelidir.
+* Gereksiz özellikler, bileşenler, dokümantasyon ve örnekler olmadan minimal bir platform. Kullanılmayan feature ve framework’leri kaldırın ya da hiç kurmayın.
+* Patch management sürecinin bir parçası olarak, tüm security notlarına, update ve patch’lere uygun konfigürasyonları gözden geçirip güncelleme görevi (bkz. **A06:2021 – Vulnerable and Outdated Components**). Cloud storage izinlerini (ör. S3 bucket permission’ları) gözden geçirin.
+* Segmentasyon, containerization veya cloud security group’ları (ACL’ler) ile bileşenler veya tenant’lar arasında etkili ve güvenli ayrım sağlayan segmented bir application architecture.
+* Client’lara security directive’leri göndermek; ör. Security Headers.
+* Tüm ortamlarda konfigürasyon ve ayarların etkinliğini doğrulayan otomatik bir süreç.
+## Example attack scenarios
+**Senaryo #1:** Application server, production’da kaldırılmamış sample application’larla birlikte geliyor. Bu sample’ların bilinen security açıkları vardır ve saldırganlar server’ı ele geçirmek için bunları kullanır. Bu uygulamalardan biri admin console ise ve varsayılan hesaplar değiştirilmemişse, saldırgan default password’lerle giriş yapar ve kontrolü ele geçirir.
+**Senaryo #2:** Server’da directory listing devre dışı değildir. Bir saldırgan, dizinleri basitçe listeyebildiğini keşfeder. Derlenmiş Java class’larını bulur ve indirir; bunları decompile ederek kodu inceler. Ardından uygulamada ciddi bir access control açığı bulur.
+**Senaryo #3:** Application server konfigürasyonu, detaylı hata mesajlarının (ör. stack trace’ler) kullanıcılara döndürülmesine izin verir. Bu, potansiyel olarak hassas bilgileri veya bilinen zafiyetlere sahip bileşen versiyonları gibi temel açıkları ortaya çıkarabilir.
+**Senaryo #4:** Bir cloud service provider (CSP), diğer CSP kullanıcıları tarafından Internet’e açık varsayılan paylaşım izinlerine sahiptir. Bu durum, cloud storage içinde saklanan hassas verilere erişilmesine olanak tanır.
+Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A05_2021-Security_Misconfiguration/</t>
+  </si>
+  <si>
+    <t>You are likely vulnerable:
+-   If you do not know the versions of all components you use (both
+    client-side and server-side). This includes components you directly
+    use as well as nested dependencies.
+-   If the software is vulnerable, unsupported, or out of date. This
+    includes the OS, web/application server, database management system
+    (DBMS), applications, APIs and all components, runtime environments,
+    and libraries.
+-   If you do not scan for vulnerabilities regularly and subscribe to
+    security bulletins related to the components you use.
+-   If you do not fix or upgrade the underlying platform, frameworks,
+    and dependencies in a risk-based, timely fashion. This commonly
+    happens in environments when patching is a monthly or quarterly task
+    under change control, leaving organizations open to days or months
+    of unnecessary exposure to fixed vulnerabilities.
+-   If software developers do not test the compatibility of updated,
+    upgraded, or patched libraries.
+-   If you do not secure the components’ configurations (see
+    **A05:2021-Security Misconfiguration**).</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Max Coverage | Avg Coverage | Avg Weighted Exploit | Avg Weighted Impact | Total Occurrences | Total CVEs |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 3           | 27.96%             | 8.77%              | 51.78%       | 22.47%       | 5.00                 | 5.00                | 30,457            | 0          |
+## How to prevent
+There should be a patch management process in place to:
+-   Remove unused dependencies, unnecessary features, components, files,
+    and documentation.
+-   Continuously inventory the versions of both client-side and
+    server-side components (e.g., frameworks, libraries) and their
+    dependencies using tools like versions, OWASP Dependency Check,
+    retire.js, etc. Continuously monitor sources like Common Vulnerability and 
+    Exposures (CVE) and National Vulnerability Database (NVD) for
+    vulnerabilities in the components. Use software composition analysis
+    tools to automate the process. Subscribe to email alerts for
+    security vulnerabilities related to components you use.
+-   Only obtain components from official sources over secure links.
+    Prefer signed packages to reduce the chance of including a modified,
+    malicious component (see **A08:2021-Software and Data Integrity Failures**).
+-   Monitor for libraries and components that are unmaintained or do not
+    create security patches for older versions. If patching is not
+    possible, consider deploying a virtual patch to monitor, detect, or
+    protect against the discovered issue.
+Every organization must ensure an ongoing plan for monitoring, triaging,
+and applying updates or configuration changes for the lifetime of the
+application or portfolio.
+## Example attack scenarios
+**Scenario #1:** Components typically run with the same privileges as
+the application itself, so flaws in any component can result in serious
+impact. Such flaws can be accidental (e.g., coding error) or intentional
+(e.g., a backdoor in a component). Some example exploitable component
+vulnerabilities discovered are:
+-   CVE-2017-5638, a Struts 2 remote code execution vulnerability that
+    enables the execution of arbitrary code on the server, has been
+    blamed for significant breaches.
+-   While the internet of things (IoT) is frequently difficult or
+    impossible to patch, the importance of patching them can be great
+    (e.g., biomedical devices).
+There are automated tools to help attackers find unpatched or
+misconfigured systems. For example, the Shodan IoT search engine can
+help you find devices that still suffer from Heartbleed vulnerability
+patched in April 2014.
+For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2021/A06_2021-Vulnerable_and_Outdated_Components/</t>
+  </si>
+  <si>
+    <t>## Score table
+| Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 3          | 27.96 %             | 8.77 %              | 5.00                 | 5.00                | 51.78 %       | 22.47 %       | 30,457           | 0        |
+## How to prevent
+Es sollte ein Patch-Management-Prozess vorhanden sein:
+- Entfernen Sie ungenutzte Abhängigkeiten, unnötige Funktionen, Komponenten, Dateien und Dokumentation.
+- Kontinuierliche Bestandsaufnahme der Versionen sowohl der clientseitigen als auch der serverseitigen Komponenten (z. B. Frameworks, Bibliotheken) und ihrer Abhängigkeiten mithilfe von Tools wie "versions", "OWASP Dependency Check", "retire.js" usw. Überwachen Sie kontinuierlich Quellen wie Common Vulnerability and Exposures (CVE) und die National Vulnerability Database (NVD) für Schwachstellen in den Komponenten. Verwenden Sie Software-Tools zur Analyse der Softwarebestandteile, um den Prozess zu automatisieren. Abonnieren Sie E-Mail-Benachrichtigungen zu Sicherheitslücken im Zusammenhang mit den verwendeten Komponenten.
+- Beziehen Sie Komponenten nur von offiziellen Quellen über sichere Links. Bevorzugen Sie signierte Pakete, um die Wahrscheinlichkeit zu verringern, dass eine modifizierte, bösartige Komponente enthalten ist (siehe **A08:2021-Fehlerhafte Prüfung der Software- und Datenintegrität**).
+- Überwachen Sie Bibliotheken und Komponenten, die nicht gewartet werden oder keine Sicherheitspatches für ältere Versionen erstellen. Wenn das Patchen nicht möglich ist, erwägen Sie die Bereitstellung eines virtuellen Patches zur Überwachung, Erkennung oder zum Schutz vor dem entdeckten Problem.
+Jede Organisation muss einen fortlaufenden Plan für die Überwachung, Triage und Anwendung von Updates oder Konfigurationsänderungen während der gesamten Lebensdauer der Anwendung oder des Portfolios sicherstellen.
+## Example attack scenarios
+**Szenario Nr. 1:** Komponenten werden normalerweise mit denselben Berechtigungen wie die Anwendung selbst ausgeführt, sodass Fehler in einer Komponente schwerwiegende Auswirkungen haben können. Solche Fehler können zufällig (z. B. ein Programmierfehler) oder absichtlich (z. B. eine Backdoor in einer Komponente) sein. Einige Beispiele für entdeckte ausnutzbare Komponentenschwachstellen sind:
+- CVE-2017-5638, eine Remote Code Execution Schwachstelle in Struts 2, die Angreifende ermächtigt, beliebigen Code auf dem Server auszuführen, wurde für einige erhebliche Sicherheitsvorfälle verantwortlich gemacht.
+- Obwohl das Patchen von Internet of Things (IoT) Geräten oft nur sehr schwierig oder unmöglich ist,
+kann dies sehr wichtig sein (z. B. für biomedizinische Geräte).
+Es existieren automatisierte Tools, die Angreifenden helfen, nicht gepatchte oder falsch konfigurierte Systeme zu finden. Die Shodan IoT-Suchmaschine kann Ihnen beispielsweise dabei helfen, Geräte zu finden, die immer noch für die im April 2014 gepatchte Heartbleed-Sicherheitslücke verwundbar sind.
+Weitere Informationen zu den Referenzen und zur Liste der zugeordneten CWEs: https://top10.owasp.org/2021/de/A06_2021-Vulnerable_and_Outdated_Components/</t>
+  </si>
+  <si>
+    <t>Usted probablemente sea vulnerable:
+-   Si no conoce las versiones de todos los componentes que utiliza (tanto en el cliente como en el servidor). Esto incluye los componentes que usa directamente, así como las dependencias anidadas.
+-   Si el software es vulnerable, carece de soporte o no está actualizado. Esto incluye el sistema operativo, el servidor web/de aplicaciones, el sistema de administración de bases de datos (DBMS), las aplicaciones, las API y todos los componentes, los entornos de ejecución y las bibliotecas.
+-   Si no analiza en búsqueda de vulnerabilidades de forma regular y no se suscribe a los boletines de seguridad relacionados con los componentes que utiliza.
+-   Si no repara o actualiza la plataforma subyacente, frameworks y dependencias de manera oportuna y basada en el riesgo. Esto suele ocurrir en entornos en los que la aplicación de parches de seguridad es una tarea mensual o trimestral bajo control de cambios, lo que deja a las organizaciones abiertas a días o meses de exposición innecesaria a vulnerabilidades con soluciones disponibles.
+-   Si los desarrolladores de software no testean la compatibilidad de las bibliotecas actualizadas, actualizadas o parcheadas.
+-   Si no asegura las configuraciones de los componentes (consulte **A05:2021 – Configuración de Seguridad Incorrecta**).</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
+|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
+| 3           | 27.96%             | 8.77%              | 51.78%       | 22.47%       | 5.00                 | 5.00                | 30,457            | 0          |
+## How to prevent
+Debe existir un proceso de administración de parches que:
+-   Elimine las dependencias que no son utilizadas, funcionalidades, componentes, archivos y documentación innecesarios.
+-   Realice un inventario continuo de las versiones de los componentes en el cliente y en el servidor (por ejemplo, frameworks, bibliotecas) y sus dependencias utilizando herramientas como: versions, OWASP Dependency Check, retire.js, etc. Supervise continuamente fuentes como Common Vulnerability and Exposures (CVE) y National Vulnerability Database (NVD) para detectar vulnerabilidades en los componentes. Utilice herramientas de análisis de composición de software para automatizar el proceso. Suscríbase para recibir alertas por correo electrónico sobre vulnerabilidades de seguridad relacionadas con los componentes que utiliza.
+-   Solo obtenga componentes de fuentes oficiales a través de enlaces seguros.
+    Prefiera los paquetes firmados para reducir la posibilidad de incluir un componente malicioso modificado (consulte **A08:2021 – Fallas en el Software y en la Integridad de los Datos**).
+-   Supervise las bibliotecas y los componentes que no sea mantenidos o no generen parches de seguridad para versiones anteriores. Si la aplicación de parches no es posible, considere implementar un parche virtual para monitorear, detectar o protegerse contra el problema descubierto.
+Toda organización debe garantizar un plan continuo para monitorear, clasificar y aplicar actualizaciones o cambios de configuración durante la vida útil de la aplicación o portafolio de aplicaciones.
+## Example attack scenarios
+**Escenario #1:** Los componentes normalmente se ejecutan con los mismos privilegios que la propia aplicación, por lo que las fallas en cualquier componente pueden tener un impacto grave. Tales fallas pueden ser accidentales (por ejemplo, error de codificación) o intencionales (por ejemplo, una puerta trasera en un componente). Algunos ejemplos de vulnerabilidades de componentes explotables descubiertos son:
+-   CVE-2017-5638, una vulnerabilidad de ejecución remota de código de Struts 2 que permite la ejecución arbitraria de código en el servidor, ha sido culpada de brechas importantes.
+-   Si bien el Internet de las Cosas (IoT) es con frecuencia difícil o imposible de parchear, la importancia de parchearlo puede ser grande (por ejemplo, dispositivos biomédicos).
+Existen herramientas automatizadas para ayudar a los atacantes a encontrar sistemas sin parches o mal configurados. Por ejemplo, el motor de búsqueda Shodan IoT puede ayudarlo a encontrar dispositivos que aún sufren la vulnerabilidad Heartbleed parchada en abril de 2014.
+Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2021/es/A06_2021-Vulnerable_and_Outdated_Components/</t>
+  </si>
+  <si>
+    <t>Você provavelmente está vulnerável:
+- Se você não souber as versões de todos os componentes que usa
+    (tanto do lado do cliente quanto do lado do servidor). Isso
+    inclui componentes que você usa diretamente, bem como
+    dependências aninhadas.
+- Se o software for vulnerável, sem suporte ou desatualizado.
+    Isso inclui o sistema operacional, servidor _web/application_,
+    sistema de gerenciamento de banco de dados (DBMS), aplicações,
+    APIs e todos os componentes, ambientes de tempo de execução e bibliotecas.
+- Se você não faz a varredura de vulnerabilidades regularmente e
+    não assina os boletins de segurança relacionados aos componentes que você usa.
+- Se você não corrigir ou atualizar a plataforma, as estruturas e as dependências
+    subjacentes de maneira oportuna e baseada em riscos. Isso geralmente acontece
+    em ambientes em que a correção é uma tarefa mensal ou trimestral sob controle
+    de alterações, deixando as organizações abertas a dias ou meses de exposição
+    desnecessária a vulnerabilidades corrigidas.
+- Se os desenvolvedores de software não testarem a compatibilidade de
+   bibliotecas atualizadas, atualizações ou com patches.
+- Se você não proteger as configurações dos componentes
+    (consulte **A05: 2021-Configuração Incorreta de Segurança**).</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
+|:-------------:|:-------------------------:|:------------------------:|:--------------------------:|:-----------------------:|:----------------:|:---------------:|:--------------------:|:-------------:|
+| 3             | 27.96%                    | 8.77%                    | 51.78%                     | 22.47%                  | 5.00             | 5.00            | 30,457               | 0             |
+## How to prevent
+Deve haver um processo de gerenciamento de dependências para:
+- Remova dependências não utilizadas, recursos, componentes, arquivos
+    e documentação desnecessários.
+- Atualizar continuamente um inventário com as versões dos componentes
+    do lado do cliente e do lado do servidor (por exemplo, estruturas,
+    bibliotecas) e suas dependências usando ferramentas como _versions_,
+    _OWASP Dependency Check_, _retire.js_, etc. Monitore continuamente fontes
+    como _Common Vulnerability and Exposures_ (CVE) e _National Vulnerability
+    Database_ (NVD) para vulnerabilidades nos componentes. Use ferramentas
+    de análise de composição de software para automatizar o processo.
+    Inscreva-se para receber alertas de e-mail sobre vulnerabilidades de
+    segurança relacionadas aos componentes que você usa.
+- Obtenha componentes apenas de fontes oficiais por meio de links seguros.
+    Prefira pacotes assinados para reduzir a chance de incluir um componente
+    malicioso modificado (consulte
+    **A08: 2021-Software e Falhas de Integridade de Dados**).
+- Monitore bibliotecas e componentes sem manutenção ou que não criem patches
+    de segurança para versões anteriores. Se o patch não for possível,
+    considere implantar um patch virtual para monitorar, detectar ou proteger
+    contra o problema descoberto.
+Cada organização deve garantir um plano contínuo de monitoramento, triagem e
+aplicação de atualizações ou alterações de configuração durante a vida
+útil da aplicação ou portfólio.
+## Example attack scenarios
+**Cenário #1:** Os componentes normalmente são executados com os mesmos
+privilégios da própria aplicação, portanto, as falhas em qualquer componente
+podem resultar em sério impacto. Essas falhas podem ser acidentais
+(por exemplo, erro de codificação) ou intencionais (por exemplo, uma
+_backdoor_ em um componente). Alguns exemplos de vulnerabilidades
+de componentes exploráveis descobertos são:
+- CVE-2017-5638, uma vulnerabilidade de execução remota de código
+    do Struts 2 que permite a execução de código arbitrário no servidor,
+    foi responsabilizada por violações significativas.
+- Embora a Internet das Coisas (IoT) seja frequentemente difícil ou
+    impossível de corrigir, a importância de corrigi-los pode ser
+    grande (por exemplo, dispositivos biomédicos).
+Existem ferramentas automatizadas para ajudar os invasores a encontrar
+sistemas não corrigidos ou configurados incorretamente. Por exemplo,
+o mecanismo de pesquisa Shodan IoT pode ajudá-lo a encontrar
+dispositivos que ainda sofrem com a vulnerabilidade Heartbleed
+corrigida em abril de 2014.
+Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A06_2021-Vulnerable_and_Outdated_Components/</t>
+  </si>
+  <si>
+    <t>Aşağıdaki durumlarda muhtemelen savunmasızsınız:
+* Kullandığınız tüm bileşenlerin (hem client-side hem de server-side) versiyonlarını bilmiyorsanız. Buna doğrudan kullandıklarınızın yanı sıra nested dependency’ler de dahildir.
+* Yazılım (OS, web/application server, database management system (DBMS), uygulamalar, APIs ve tüm bileşenler, runtime environment’lar ve kütüphaneler dâhil) savunmasız, desteklenmiyor veya güncel değilse.
+* Düzenli olarak zafiyet taraması yapmıyor ve kullandığınız bileşenlerle ilgili security bulletin’lere abone olmuyorsanız.
+* Temel platformu, framework’leri ve dependency’leri risk temelli ve zamanında düzeltmiyor veya upgrade etmiyorsanız. Bu genellikle patching’in aylık veya üç aylık bir change control görevi olduğu ortamlarda yaşanır ve kuruluşları düzeltilmiş zafiyetlere karşı günlerce veya aylarca gereksiz açıkta bırakır.
+* Yazılım geliştiriciler, güncellenmiş, upgrade edilmiş veya patch uygulanmış kütüphanelerin uyumluluğunu test etmiyorsa.
+* Bileşenlerin configuration’larını güvence altına almıyorsanız (bkz. **A05:2021-Security Misconfiguration**).</t>
+  </si>
+  <si>
+    <t>## Score table
+| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Max Coverage | Avg Coverage | Avg Weighted Exploit | Avg Weighted Impact | Total Occurrences | Total CVEs |
+| :---------: | :----------------: | :----------------: | :----------: | :----------: | :------------------: | :-----------------: | :---------------: | :--------: |
+|      3      |       27.96%       |        8.77%       |    51.78%    |    22.47%    |         5.00         |         5.00        |       30,457      |      0     |
+## How to prevent
+Aşağıdakileri kapsayan bir patch management süreci olmalıdır:
+* Kullanılmayan dependency’leri, gereksiz özellikleri, bileşenleri, dosyaları ve dokümantasyonu kaldırın.
+* Hem client-side hem de server-side bileşenlerin (örn. framework’ler, kütüphaneler) ve dependency’lerinin versiyonlarını sürekli olarak envanterleyin; versions, OWASP Dependency Check, retire.js vb. araçları kullanın. Common Vulnerabilities and Exposures (CVE) ve National Vulnerability Database (NVD) gibi kaynakları bileşenlerdeki zafiyetler için sürekli izleyin. Bu süreci otomatikleştirmek için software composition analysis araçlarını kullanın. Kullandığınız bileşenlerle ilgili security vulnerability e-posta uyarılarına abone olun.
+* Bileşenleri yalnızca resmi kaynaklardan ve güvenli bağlantılar üzerinden edinin. Değiştirilmiş, kötü amaçlı bir bileşen ekleme olasılığını azaltmak için imzalı paketleri tercih edin (bkz. **A08:2021-Software and Data Integrity Failures**).
+* Bakımı yapılmayan veya eski versiyonlar için security patch üretmeyen kütüphane ve bileşenleri izleyin. Patching mümkün değilse, keşfedilen soruna karşı izleme, tespit veya koruma sağlayacak bir virtual patch uygulamayı değerlendirin.
+Her kuruluş, uygulamanın veya portföyün yaşam döngüsü boyunca izleme, önceliklendirme (triage) ve update/konfigürasyon değişikliklerini uygulamaya yönelik sürekli bir plan sağlamalıdır.
+## Example attack scenarios
+**Senaryo #1:** Bileşenler genellikle uygulamanın kendisiyle aynı ayrıcalıklarla çalıştığından, herhangi bir bileşendeki kusurlar ciddi etkilere yol açabilir. Bu kusurlar kazara (örn. coding error) veya kasıtlı (örn. bir bileşende backdoor) olabilir. Keşfedilmiş bazı istismar edilebilir bileşen zafiyetleri şunlardır:
+* CVE-2017-5638, server üzerinde arbitrary code execution’a imkân veren bir Struts 2 remote code execution zafiyeti, büyük ihlallerden sorumlu tutulmuştur.
+* Internet of Things (IoT) genellikle patch’lenmesi zor veya imkânsız olsa da, bunların patch’lenmesinin önemi büyük olabilir (örn. biyomedikal cihazlar).
+Saldırganların patch uygulanmamış veya misconfigured sistemleri bulmasına yardımcı olan otomatik araçlar vardır. Örneğin, Shodan IoT arama motoru, Nisan 2014’te patch’lenen Heartbleed zafiyetinden hâlâ etkilenen cihazları bulmanıza yardımcı olabilir.
+Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A06_2021-Vulnerable_and_Outdated_Components/</t>
+  </si>
+  <si>
+    <t>Confirmation of the user's identity, authentication, and session
+management is critical to protect against authentication-related
+attacks. There may be authentication weaknesses if the application:
+-   Permits automated attacks such as credential stuffing, where the
+    attacker has a list of valid usernames and passwords.
+-   Permits brute force or other automated attacks.
+-   Permits default, weak, or well-known passwords, such as "Password1"
+    or "admin/admin".
+-   Uses weak or ineffective credential recovery and forgot-password
+    processes, such as "knowledge-based answers," which cannot be made
+    safe.
+-   Uses plain text, encrypted, or weakly hashed passwords data stores (see
+    **A02:2021-Cryptographic Failures**).
+-   Has missing or ineffective multi-factor authentication.
+-   Exposes session identifier in the URL.
+-   Reuse session identifier after successful login.
+-   Does not correctly invalidate Session IDs. User sessions or
+    authentication tokens (mainly single sign-on (SSO) tokens) aren't
+    properly invalidated during logout or a period of inactivity.</t>
+  </si>
+  <si>
+    <t>Die Überprüfung der Identität des Nutzenden, die Authentifizierung und die Sitzungsverwaltung sind entscheidend für den Schutz vor authentifizierungsbezogenen Angriffen. Schwachstellen bei der Authentifizierung können auftreten, falls die Anwendung:
+- automatisierte Angriffe wie Credential Stuffing zulässt, bei dem Angreifende über eine Liste gültiger Usernamen und Passwörter verfügen.
+- Brute-Force- oder andere automatisierte Angriffe ermöglicht.
+- Standard-, schwache oder gängige Passwörter zulässt, wie z. B. "Passwort1" oder "admin/admin".
+- schwache oder ineffektive Verfahren zur Wiederherstellung von Anmeldeinformationen  und   Verfahren für vergessene Passwörtern, wie z. B. „wissensbasierte Antworten“, die nicht sicher gemacht werden können, 
+verwendet werden.
+-  Klartext-, verschlüsselte oder schwach gehashte Kennwortdatenspeicher (siehe
+    **A02:2021-Cryptographic Failures**) verwendet.
+- Fehlende oder unwirksame Multi-Faktor-Authentifizierung.
+- Die Session-ID wird in der URL angezeigt.
+- Session-IDs nach erfolgreichem Login wieder verwendet werden.
+- Session-IDs werden nicht korrekt ungültig gemacht. Sitzungen von Benutzenden (user sessions) oder Authentifizierungs-Tokens (hauptsächlich Single Sign-On (SSO) Tokens) werden beim Abmelden oder bei Inaktivität nicht ordnungsgemäß invalidiert.</t>
+  </si>
+  <si>
+    <t>La confirmación de la identidad, la autenticación y la gestión de sesiones del usuario son fundamentales para protegerse contra ataques relacionados con la autenticación. Puede haber debilidades de autenticación si la aplicación:
+-   Permite ataques automatizados como la reutilización de credenciales conocidas, donde el atacante posee una lista de pares de usuario y contraseña válidos.
+-   Permite ataques de fuerza bruta u otros ataques automatizados.
+-   Permite contraseñas por defecto, débiles o bien conocidas, como "Password1" o "admin/admin".
+-   Posee procesos débiles o no efectivos para las funcionalidades de olvido de contraseña o recuperación de credenciales, como "respuestas basadas en el conocimiento", las cuales no se pueden implementar de forma segura.
+-   Almacena las contraseñas en texto claro, cifradas o utilizando funciones de hash débiles (consulte **A02: 2021-Fallas Criptográficas**).
+-   No posee una autenticación multi-factor o la implementada es ineficaz.
+-   Expone el identificador de sesión en la URL.
+-   Reutiliza el identificador de sesión después de iniciar sesión.
+-   No inválida correctamente los identificadores de sesión. Las sesiones de usuario o los tokens de autenticación (principalmente tokens de inicio de sesión único (SSO)) no son correctamente invalidados durante el cierre de sesión o luego de un período de inactividad.</t>
+  </si>
+  <si>
+    <t>La confirmation de l'identité, de l'authentification et de la session de l'utilisateur sont essentielles pour se protéger des attaques liées à l'authentification. Il peut y avoir des faiblesses d'authentification si l'application :
+- autorise les attaques automatisées telles que le bourrage des informations d'identification, où l'attaquant dispose d'une liste de noms d'utilisateurs valides et mots de passe ;
+- permet la force brute ou d'autres attaques automatisées ;
+- autorise les mots de passe par défaut, faibles ou bien connus, tels que "Password1" ou "admin / admin" ;
+- utilise des processus de récupération des informations d'identification faibles ou inefficaces et des processus de mot de passe oublié, tels que «&amp;nbsp;Questions secrètes&amp;nbsp;», qui ne peuvent être sécurisées ;
+- utilise des mots de passe en texte brut, chiffrés ou faiblement hachés (voir **A02:2021 – Défaillances cryptographiques**) ;
+- absence ou utilisation inefficace de l’authentification multifacteur ;
+- exposition des identifiants de session dans l'URL ;
+- réutilisation de l'identifiant de session après une connexion réussie ;
+- n'invalide pas correctement les identifiants de session. Les sessions utilisateurs ou les jetons d'authentification (en particulier les jetons SSO) ne sont pas correctement invalidés lors de la déconnexion ou après une période d'inactivité.</t>
+  </si>
+  <si>
+    <t>Confirmação da identidade, autenticação e sessão do usuário
+gerenciamento é fundamental para proteger contra autenticação relacionada
+ataques. Pode haver pontos fracos de autenticação se o aplicativo:
+- Permite ataques automatizados, como preenchimento de credenciais, onde o
+     invasor tem uma lista de nomes de usuários e senhas válidos.
+- Permite força bruta ou outros ataques automatizados.
+- Permite senhas padrão, fracas ou conhecidas, como "Senha1" ou "admin/admin".
+- Usa recuperação de credenciais fraca ou ineficaz e esqueci a senha
+     processos, como "respostas baseadas em conhecimento", que não podem ser feitas
+     de modo seguro.
+- Usa armazenamento de dados e senhas em texto simples, criptografadas ou com hash fraco (consulte
+    **A02:2021-Falhas Criptográficas**).
+- Possui multifator de autenticação ausente ou ineficaz.
+- Expõe o identificador de sessão na URL.
+- Reutiliza o identificador de sessão após o login bem-sucedido.
+- Não invalida corretamente IDs de sessão. Sessões de usuário ou
+     tokens de autenticação (principalmente tokens de logon único (SSO)) não são
+     devidamente invalidado durante o logout ou um período de inatividade.</t>
+  </si>
+  <si>
+    <t>Kullanıcının kimliğinin doğrulanması, authentication ve session yönetimi; authentication kaynaklı saldırılara karşı korunmak için kritiktir. Aşağıdaki durumlar varsa uygulamada authentication zafiyetleri olabilir:
+-   Saldırganın geçerli username/password listeleriyle credential stuffing gibi otomatik saldırılar yapmasına izin veriyorsa.
+-   Brute force veya diğer otomatik saldırılara izin veriyorsa.
+-   “Password1” veya “admin/admin” gibi varsayılan, zayıf veya yaygın parolalara izin veriyorsa.
+-   “Bilgiye dayalı sorular” gibi güvenli hâle getirilemeyen zayıf/hatalı credential recovery ve forgot-password süreçleri kullanılıyorsa.
+-   Parolalar plain text, şifreli ama hatalı veya zayıf şekilde hash’lenmiş data store’larda tutuluyorsa (bkz. **A02:2021-Cryptographic Failures**).
+-   Multi-factor authentication eksik veya etkisizse.
+-   Session identifier URL’de açığa çıkıyorsa.
+-   Başarılı login’den sonra aynı session identifier yeniden kullanılıyorsa.
+-   Session ID’ler doğru şekilde geçersiz kılınmıyorsa. Kullanıcı session’ları veya authentication token’ları (özellikle single sign-on (SSO) token’ları) logout sırasında veya belli bir inactivity süresinden sonra düzgün biçimde invalid edilmiyorsa.</t>
+  </si>
+  <si>
+    <t>Returning to the OWASP Top 10 2021, this category is to help detect,
+escalate, and respond to active breaches. Without logging and
+monitoring, breaches cannot be detected. Insufficient logging,
+detection, monitoring, and active response occurs any time:
+-   Auditable events, such as logins, failed logins, and high-value
+    transactions, are not logged.
+-   Warnings and errors generate no, inadequate, or unclear log
+    messages.
+-   Logs of applications and APIs are not monitored for suspicious
+    activity.
+-   Logs are only stored locally.
+-   Appropriate alerting thresholds and response escalation processes
+    are not in place or effective.
+-   Penetration testing and scans by dynamic application security testing (DAST) tools (such as OWASP ZAP) do
+    not trigger alerts.
+-   The application cannot detect, escalate, or alert for active attacks
+    in real-time or near real-time.
+-   You are vulnerable to information leakage by making logging and alerting
+events visible to a user or an attacker (see **A01:2021-Broken Access Control**).
+-   You are vulnerable to injections or
+    attacks on the logging or monitoring systems if log data is not correctly encoded.</t>
+  </si>
+  <si>
+    <t>Mit Blick auf die OWASP Top 10 2021 soll diese Kategorie bei der Erkennung, Eskalation und Reaktion auf laufende Angriffe unterstützen. Ohne Protokollierung und Überwachung können Angriffe nicht erkannt werden. Unzureichende Protokollierung, Erkennung, Überwachung und aktive Reaktion sind jederzeit möglich:
+- Nachvollziehbare Ereignisse, wie Anmeldungen, fehlgeschlagene Anmeldungen und wertvolle Transaktionen, werden nicht protokolliert.
+- Warnungen und Fehler erzeugen keine, unangemessene oder unklare Log-Einträge.
+- Die Logs von Anwendungen und APIs werden nicht auf verdächtige Aktivitäten überwacht.
+- Protokolle werden nur lokal gespeichert.
+- Geeignete Schwellenwerte für Warnmeldungen und Eskalationsprozesse für Gegenmaßnahmen sind nicht vorhanden oder nicht wirksam.
+- Penetrationstests und Scans durch DAST-Tools (Dynamic Application Security Testing) (wie OWASP ZAP) lösen keine Alarme aus.
+- Die Anwendungen können Angriffe weder in Echtzeit noch nahezu in Echtzeit erkennen, eskalieren oder Alarm schlagen.
+Es besteht die Gefahr von Informationslecks, falls Sie die Logging- und Alerting Ereignisse für Nutzende oder Angreifende sichtbar gemacht werden (siehe **A01:2021-Broken Access Control**).</t>
+  </si>
+  <si>
+    <t>Volviendo al OWASP Top 10 2021, la intención es apoyar la detección, escalamiento y respuesta ante brechas activas. Sin registros y monitoreo, las brechas no pueden ser detectadas. Registros, detecciones, monitoreo y respuesta activas insuficientes pueden ocurrir en cualquier momento:
+-   Eventos auditables, tales como los inicios de sesión, fallas en el inicio de sesión y transacciones de alto valor no son registradas.
+-   Advertencias y errores generan registros poco claros, inadecuados y en algunos casos ni se generan.
+-   Registros en aplicaciones y API no son monitoreados para detectar actividades sospechosas.
+-   Los registros son únicamente almacenados en forma local.
+-   Los umbrales de alerta y procesos de escalamiento no están correctamente implementados o no son efectivos.
+-   Las pruebas de penetración y los escaneos utilizando herramientas de pruebas dinámicas de seguridad en aplicaciones (como ser OWASP ZAP) no generan alertas.
+-   Las aplicaciones no logran detectar, escalar, o alertar sobre ataques activos en tiempo real ni cercanos al tiempo real.
+Se es vulnerable a la fuga de información haciendo registros y eventos de alertas que sean visibles para un usuario o un atacante (consulte **A01: 2021-Pérdida de Control de Acceso**).</t>
+  </si>
+  <si>
+    <t>De retour dans le Top 10 2021 de l'OWASP, cette catégorie a pour but d'aider à la détection, à l'escalade et à la réponse aux brèches actives. Sans journalisation et surveillance, les brèches ne peuvent être détectées. Une journalisation, une détection, une surveillance et une réponse active insuffisantes peuvent survenir à tout moment :
+- les traces d’audit, telles que les accès réussis ou échoués et les transactions sensibles, ne sont pas enregistrées ;
+- les alertes et les erreurs générées ne sont pas enregistrées, ou leur journalisation est inadéquate, ou imprécise ;
+- les journaux des applications et des API ne sont pas contrôlés pour détecter les actions suspectes ;
+- les journaux ne sont stockés que localement ;
+- aucun processus de seuil d’alerte convenable ni de remontées d'information pour y répondre n'ont été définis, ou ils sont inadéquats, ou inefficaces ;
+- les tests d'intrusion et de balayage avec des outils de test dynamique de sécurité des applications (DAST), tels que OWASP ZAP, ne génèrent pas d'alertes ;
+- l’application est incapable de détecter, de générer des remontées d'information et des alertes en temps réel, ou assimilé, en cas d’attaque active.
+Vous êtes vulnérable à une fuite d’information en rendant les enregistrements de journalisation et d’alertes accessibles à vos utilisateurs ou attaquants (voir **A01:2021-Contrôles d'accès défaillants**).</t>
+  </si>
+  <si>
+    <t>Tornando alla Top 10 2021 di OWASP, questa categoria è per aiutare a rilevare,
+svolgere escalation e rispondere alle violazioni attive. Senza logging e
+monitoraggio, le violazioni non possono essere rilevate. Il logging,
+il rilevamento, il monitoraggio e la risposta attiva insufficienti si verificano ogni volta che:
+-   Gli eventi verificabili, come i login, i login falliti e le transazioni ad alto valore, non vengono registrati.
+-   Warning ed errori non generano messaggi di log, oppure sono inadeguati o poco chiari.
+-   I log di applicazioni e API non sono monitorati per attività sospette.
+-   I file di log vengono memorizzati solo localmente.
+-   Non sono presenti o sono inefficaci le soglie di allarme e processi di escalation della risposta
+-   I penetration test e le scansioni da parte di strumenti DAST (Dynamic Application Security Testing) (come OWASP ZAP) 
+    non attivano nessun allarme.
+-   L'applicazione non è in grado di rilevare, svolgere escalation o avvisare per gli attacchi attivi
+    in real-time o quasi in real-time. 
+Si è vulnerabili alla fuga di informazioni se gli eventi di logging e gli alert sono
+visibili ad un utente o ad un attaccante (vedi **A01:2021-Broken Access Control**).</t>
+  </si>
+  <si>
+    <t>OWASP Top 10 2021 に話を戻すと、このカテゴリは、アクティブな違反の検出、エスカレーション、および対応を支援するものです。
+ロギングとモニタリングがなければ、侵害を検知することはできません。
+ロギングや検知、モニタリング、適時の対応が十分に行われないという状況は、いつでも発生します:
+-   ログイン、失敗したログイン、重要なトランザクションなどの監査可能なイベントがログに記録されていない。
+-   警告とエラーが発生してもログメッセージが生成されない、または不十分、不明確なメッセージが生成されている。
+-   アプリケーションとAPIのログが、疑わしいアクティビティをモニタリングしていない。
+-   ログがローカルにのみ格納されている。
+-   アラートの適切なしきい値とレスポンスのエスカレーションプロセスが整えられていない、または有効ではない。
+-   ペネトレーションテストやDAST(dynamic application security testing)ツール（OWASP ZAPなど）によるスキャンがアラートをあげない。
+-   アプリケーションがリアルタイム、準リアルタイムにアクティブな攻撃を検知、エスカレート、またはアラートすることができない。
+ユーザまたは攻撃者がログやアラートのイベントを閲覧できると、情報の漏えいが発生する可能性があります (**A01:2021-アクセス制御の不備** を参照).</t>
+  </si>
+  <si>
     <t>Retornando à lista OWASP Top 10 de 2021, essa categoria ajuda a detectar, escalonar e responder a violações ativas. Sem o monitoramento e registro, as violações não podem ser detectadas. A falta de registro, detecção, monitoramento e resposta ativa ocorre sempre que:
 - Eventos auditáveis, como logins, logins falhos e transações de alto valor, não são registrados.
 - Avisos e erros geram mensagens de log inexistentes, inadequadas ou confusas.
@@ -4687,27 +5014,7 @@
 - Testes de penetração e varreduras por ferramentas de teste de segurança de aplicativos dinâmicos (DAST), como OWASP ZAP, não acionam alertas.
 - A aplicação não pode detectar, escalonar ou alertar para ataques ativos em tempo real ou quase em tempo real.
 Você está vulnerável a vazamento de informações tornando eventos de registro e alerta visíveis para um usuário ou um atacante 
-(veja [A01:2021-Quebra de Controle de Acesso](A01_2021-Broken_Access_Control.md)).</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapeados | Taxa de Incidência Máxima | Taxa de Incidência Média | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Cobertura Média | Total de ocorrências | Total de CVEs |
-|:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
-| 4           | 19.23%             | 6.51%              | 6.87                 | 4.99                | 53.67%       | 39.97%       | 53,615            | 242        |
-## How to prevent
-Os desenvolvedores devem implementar alguns ou todos os controles a seguir, dependendo do risco da aplicação:
-- Garantir que todas as falhas de login, controle de acesso e validação de entrada no lado do servidor possam ser registradas com contexto de usuário suficiente para identificar contas suspeitas ou maliciosas e mantidas por tempo suficiente para permitir análise forense atrasada.
-- Garantir que os logs sejam gerados em um formato que as soluções de gerenciamento de logs possam facilmente consumir.
-- Garantir que os dados de log sejam codificados corretamente para evitar injeções ou ataques nos sistemas de registro ou monitoramento.
-- Garantir que transações de alto valor tenham uma trilha de auditoria com controles de integridade para evitar adulteração ou exclusão, como tabelas de banco de dados somente para adição ou similares.
-- As equipes de DevSecOps devem estabelecer monitoramento e alerta efetivos para que atividades suspeitas sejam detectadas e respondidas rapidamente.
-- Estabelecer ou adotar um plano de resposta e recuperação de incidentes, como o National Institute of Standards and Technology (NIST) 800-61r2 ou posterior.
-Existem estruturas de proteção de aplicativos comerciais e de código aberto, como o OWASP ModSecurity Core Rule Set, e software de correlação de logs de código aberto, como o Elasticsearch, Logstash, Kibana (ELK) stack, que possuem painéis personalizados e alertas.
-## Example attack scenarios
-**Cenário 1:** O operador do site do provedor de plano de saúde infantil não conseguiu detectar uma violação devido à falta de monitoramento e registro. Uma parte externa informou ao provedor do plano de saúde que um invasor havia acessado e modificado milhares de registros de saúde sensíveis de mais de 3,5 milhões de crianças. Uma revisão pós-incidente descobriu que os desenvolvedores do site não haviam abordado vulnerabilidades significativas. Como não houve registro ou monitoramento do sistema, a violação de dados pode ter estado em andamento desde 2013, um período de mais de sete anos.
-**Cenário 2:** Uma grande companhia aérea indiana teve uma violação de dados envolvendo dados pessoais de milhões de passageiros por mais de dez anos, incluindo dados de passaporte e cartão de crédito. A violação de dados ocorreu em um provedor de hospedagem em nuvem de terceiros, que notificou a companhia aérea da violação depois de algum tempo.
-**Cenário nº 3:** Uma grande companhia aérea europeia sofreu uma violação relatável do GDPR. A violação foi supostamente causada por vulnerabilidades de segurança do aplicativo de pagamento exploradas por invasores, que colheram mais de 400.000 registros de pagamento de clientes. A companhia aérea foi multada em 20 milhões de libras como resultado pelo regulador de privacidade.
-Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
+(veja **A01:2021-Quebra de Controle de Acesso**).</t>
   </si>
   <si>
     <t>OWASP Top 10 2021’e geri dönen bu kategori, aktif ihlallerin tespiti, yükseltilmesi (escalate) ve bunlara yanıt verilmesine yardımcı olur. Logging ve monitoring olmadan ihlaller tespit edilemez. Yetersiz logging, detection, monitoring ve aktif yanıt aşağıdaki durumların herhangi birinde gerçekleşir:
@@ -4718,73 +5025,8 @@
 * Uygun alerting eşikleri ve response escalation süreçleri yoksa veya etkisizse.
 * Dynamic application security testing (DAST) araçları (ör. OWASP ZAP) ile yapılan penetration test ve taramalar alert tetiklemiyorsa.
 * Uygulama aktif saldırıları gerçek zamanlı veya near real-time olarak tespit, escalate veya alert edemiyorsa.
-* Logging ve alerting event’lerini bir kullanıcıya veya saldırgana görünür kılarak bilgi sızıntısına (information leakage) açık hale geliniyorsa (bkz. [A01:2021-Broken Access Control](A01_2021-Broken_Access_Control.md)).
+* Logging ve alerting event’lerini bir kullanıcıya veya saldırgana görünür kılarak bilgi sızıntısına (information leakage) açık hale geliniyorsa (bkz. **A01:2021-Broken Access Control**).
 * Log verisi doğru şekilde encode edilmezse logging veya monitoring sistemlerine injection veya saldırılara açık olunuyorsa.</t>
-  </si>
-  <si>
-    <t>## Score table
-| CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
-| :---------: | :----------------: | :----------------: | :------------------: | :-----------------: | :----------: | :----------: | :---------------: | :--------: |
-|      4      |       19.23%       |        6.51%       |         6.87         |         4.99        |    53.67%    |    39.97%    |       53,615      |     242    |
-## How to prevent
-Uygulamanın riskine bağlı olarak geliştiriciler aşağıdaki kontrollerin bir kısmını veya tamamını uygulamalıdır:
-* Tüm login, access control ve server-side input validation hatalarının; şüpheli veya kötü niyetli hesapları tanımlayacak yeterli user context ile log’lanmasını ve gecikmeli adli analiz (forensic analysis) için yeterince uzun süre tutulmasını sağlayın.
-* Log’ların, log management çözümlerinin kolayca tüketebileceği bir formatta üretilmesini sağlayın.
-* Logging veya monitoring sistemlerine injection/saldırıları önlemek için log verisini doğru şekilde encode edin.
-* Yüksek değerli işlemler için, kurcalamayı (tampering) veya silmeyi önleyecek integrity kontrollerine sahip audit trail (ör. append-only database tabloları) sağlayın.
-* DevSecOps ekipleri, şüpheli aktivitelerin hızlıca tespit edilip yanıtlanacağı etkili monitoring ve alerting kurmalıdır.
-* National Institute of Standards and Technology (NIST) 800-61r2 veya daha yenisi gibi bir incident response ve recovery planı oluşturun veya benimseyin.
-OWASP ModSecurity Core Rule Set gibi ticari ve açık kaynak uygulama koruma framework’leri ile Elasticsearch, Logstash, Kibana (ELK) stack gibi açık kaynak log korelasyon yazılımları; custom dashboard ve alerting özellikleri sunar.
-## Example attack scenarios
-**Senaryo #1:** Bir çocuk sağlık planı sağlayıcısının web sitesi işletmecisi, monitoring ve logging eksikliği nedeniyle bir ihlali tespit edemedi. Harici bir taraf, saldırganın 3.5 milyonun üzerinde çocuğa ait binlerce hassas sağlık kaydına erişip bunları değiştirdiğini bildirdi. Olay sonrası incelemede, web sitesi geliştiricilerinin önemli zafiyetleri ele almadığı görüldü. Sistem üzerinde logging veya monitoring olmadığından, veri ihlali 2013’ten beri — yedi yılı aşkın bir süre — devam ediyor olabilirdi.
-**Senaryo #2:** Büyük bir Hint havayolu şirketi, milyonlarca yolcunun on yılı aşkın kişisel verilerini (pasaport ve kredi kartı verileri dâhil) etkileyen bir veri ihlali yaşadı. Veri ihlali, üçüncü taraf bir cloud hosting sağlayıcısında meydana geldi ve ihlal bir süre sonra havayoluna bildirildi.
-**Senaryo #3:** Büyük bir Avrupa havayolu şirketi GDPR kapsamında raporlanabilir bir ihlal yaşadı. İhlalin, saldırganlar tarafından istismar edilen payment application güvenlik zafiyetlerinden kaynaklandığı ve 400.000’den fazla müşteri ödeme kaydının toplandığı bildirildi. Havayolu, gizlilik düzenleyicisi tarafından 20 milyon pound para cezasına çarptırıldı.
-Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
-  </si>
-  <si>
-    <t>在 2021 年 OWASP Top 10，此类型有助于对进行中资安事件之侦测，升级及应变。缺乏记录及监控时无法侦测资安事件发生。不足地记录，侦测，监控及主动应变随时会发生：
-- 可稽核事件未记录，如登入成功，登入失败及高价值交易。
-- 警告或错误发生时未产生，产生不充足或产生不明确日志。
-- 未监控应用程式或应用程式介面(API)日志中的可疑活动。
-- 日志仅储存于本地端。
-- 未设有或设有无效之适当告警阀值及应变升级程序。
-- 渗透测试及 DAST 工具(如 OWASP ZAP)扫描没有触发告警。
-- 应用程式无法接近即时或即时侦测，升级或警告进行中之攻击。
-允许使用者或攻击者读取日志或告警事件可能早成资讯泄漏(参考 A01:2021 权限控制失效)</t>
-  </si>
-  <si>
-    <t>## Score table
-| 可对照 CWEs 数量 | 最大发生率 | 平均发生率 | 最大覆盖范围 | 平均覆盖范围 | 平均加权漏洞 | 平均加权影响 | 总发生数 | 相关 CVEs 总数量 |
-| :--------------: | :--------: | :--------: | :----------: | :----------: | :----------: | :----------: | :------: | :--------------: |
-|        4         |   19.23%   |   6.51%    |    53.67%    |    39.97%    |     6.87     |     4.99     |  53,615  |       242        |
-## How to prevent
-开发者应依据应用程式所面临风险实作下列部分或全部的控制项：
-- 确保记录所有登入，存取控制及服务器端输入验证之失败，日志应包含充足使用者情境以识别可疑或恶意帐号，日志应存留充足时间以利未来可能之鉴识分析要求。
-- 确保日志格式符合一般日志管理系统常用格式。
-- 确保日志经正确编码以防止遭受注入攻击或日志/监控系统遭受攻击。
-- 确保高价值交易进行时产生稽核轨迹(日志)并实作完整性控制以避免窜改或删除，如仅限附加的资料表或类似工具。
-- DevSecOps 团队应建立有效地监控及告警机制以利侦测可疑活动并快速应变。
-- 建立或导入事件应变及复原计画，如 NIST 800-61r2 或更新版本。
-现有多种商业化及开放原始码应用程式保护架构，如 OWASP ModSecurity Core Rule Set 及开放原始码日志关联软体可客制化仪表板及告警，如 ELK stack。
-## Example attack scenarios
-**情境 1**：一家儿童健康计划供应商的网站运营商因缺乏监控和记录无法侦测资安事件。外部通知该健康计划供应商，攻击者已存取及修改超过 350 万名儿童的敏感健康记录。事后审查发现网站开发者没有处理重大弱点。由于系统没有记录或监控，资料泄漏可能从 2013 年开始至今，时间超过七年。
-**情境 2**：印度一家大型航空公司发生涉及数百万乘客超过十年包括护照及信用卡资料等个人资料的资料泄漏。资料泄漏发生在第三方供应商提供的云端服务，该供应商在资料泄漏发生一段时间后通知航空公司。
-情境 3：一家大型欧洲航空公司发生依 GDPR 应报告之个资事故。据报导，攻击者利用支付应用系统之安全漏洞，取得超过 40 万笔客户支付纪录。该航空公司遭隐私主管机关裁罚两千万英镑。
-有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A09_2021-Security_Logging_and_Monitoring_Failures/</t>
-  </si>
-  <si>
-    <t>Server-Side Request Forgery (SSRF)</t>
-  </si>
-  <si>
-    <t>SSRF flaws occur whenever a web application is fetching a remote
-resource without validating the user-supplied URL. It allows an attacker
-to coerce the application to send a crafted request to an unexpected
-destination, even when protected by a firewall, VPN, or another type of
-network access control list (ACL).
-As modern web applications provide end-users with convenient features,
-fetching a URL becomes a common scenario. As a result, the incidence of
-SSRF is increasing. Also, the severity of SSRF is becoming higher due to
-cloud services and the complexity of architectures.</t>
   </si>
   <si>
     <t>## Score table
@@ -4802,7 +5044,7 @@
     *Hints:*&lt;br&gt; 
     ~ Establish an ownership and a lifecycle for firewall rules based on applications.&lt;br/&gt;
     ~ Log all accepted *and* blocked network flows on firewalls
-    (see [A09:2021-Security Logging and Monitoring Failures](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+    (see **A09:2021-Security Logging and Monitoring Failures**).
 ### **From Application layer:**
 -   Sanitize and validate all client-supplied input data
 -   Enforce the URL schema, port, and destination with a positive allow
@@ -4838,48 +5080,6 @@
 For more information about the references and the list of mapped CWEs: https://top10.owasp.org/2021/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>تزوير الطلبات من جانب الخادم SSRF</t>
-  </si>
-  <si>
-    <t>يتم تزوير طلبات الخادم عندما يقوم تطبيق الويب بجلب موارد عن بعد دون عملية التحقّق من صحة العنوان المقدّم من قِبل المستخدم، حيث يسمح ذلك للمهاجم بإجبار التطبيق على إرسال طلب معدّل إلى وجهة غير متوقعة للخادم، حتى عندما يكون محميّ بجدار حماية، أو شبكة خاصة افتراضية VPN أو أية نوع من قائمة التحكم بالوصول إلى الشبكة.
-نظرًا لأن تطبيقات الويب (المواقع الإلكترونية) الحديثة توفّر للمستخدمين مُميزات متقدّمة، فإن جلب العناوين من الخادم أصبح سيناريو شائع. نتيجة لذلك، فإن معدّل حدوث تزوير لطلبات الخادم آخذ في الازدياد، لذلك أصبح استغلال هذه الثغرة أشد خطورة على الخادم عندما ظهرت الخدمات السحابيّة وكذلك تعقيد البنية التحتيّة.</t>
-  </si>
-  <si>
-    <t>## Score table
-| ربطها مع CWEs | الحد الأقصى للحدوث | متوسط معدل الحدوث | التغطية القصوى | متوسط معدل التغطية | متوسط استغلال الثغرات | متوسط التأثير | إجمالي التكرار | إجمالي نقاط الضعف CVEs |
-|---------------|--------------------|-------------------|----------------|--------------------|-----------------------|---------------|----------------|------------------------|
-| 1             | 2.72%              | 2.72%             | 67.72%         | 67.72%             | 8.28                  | 6.72          | 9,503          | 385                    |
-## How to prevent
-يستطيع المُطوّرين منع تزوير طلبات الخادم بتنفيذ بعض أو كل وسائل الدفاع التالية في ضوابط الدفاع العميق (Defense in Depth) :
-## **من خلال طبقات الشبكة**
--   تقسيم وظائف الوصول إلى الموارد عن بعد في شبكات مُنفصلة لتقليل تأثير تزوير طلبات الخادم.
--   فرض سياسات جدار الحماية "الرفض افتراضيًا" أو ضبط آليات التحكّم في الوصول إلى الشبكة لحظر جميع حركات المرور للشبكة الداخلية باستثناء حركات المرور الأساسية.
-## **من خلال طبقات التطبيقات**
--   التصّفية والتحقّق من صحة جميع بيانات الإدخال المقدّمة من قِبل المستخدم.
--   استخدام عناوين محدّدة في الروابط، URL استخدام منافذ محدّدة مع تحديد قائمة من العناوين المحدّدة مسبقًا في قائمة مسموح بها.
--   لا تقم برد الطلبات للعميل على شكل بيانات خام
--   قم بتعطيل إعادة التوجيه إلى HTTP.
--   كن على حذر من هجمات إعادة الترتيب الرابط أو الأحرف والتي قد تأتي في بعض الهجمات من خلال بروتوكول DNS أو من خلال استخدام TOCTOU.
-لا تقم بتخفيف المخاطر على هجمات SSRF من خلال استخدام سياسة المنع المبنيّة على قائمة التعبيرات المنطقية أو (Regular Expression). حيث أن المهاجمين لديهم قوائم مُعدّة مسبقًا ومتعدّدة لمحاولة تخطّي عمليات الحجب تلك.
-## Example attack scenarios
-يستطيع المهاجمين استخدام تزوير طلبات الخادم لمهاجمة الأنظمة المحميّة خلف جدران حماية تطبيقات الويب(WAF)، وجدران الحماية أو قائمة التحكّم للوصول للشبكة باستخدام سيناريو مثل:
-**سيناريو #1:** فحص المنافذ للخوادم الداخلية في معمارية الشبكة:
-الشبكات الغير مقسّمة بشكل جيّد تُمكّن المهاجمين من رسم الشبكات الداخلية بشكل دقيق ويصل إلى تمكين المهاجم لمعرفة في حال كانت المنافذ مفتوحة أم مُغلقة للخوادم والخدمات الداخلية من خلال دراسة أو استجابة الخادم لطلبات أو من خلال الوقت المُستغرق لكل طلب على كل منفذ مختلف وذلك لمعرفة في حال كان استغلال SSRF نجح أم فشل.
-**سيناريو #2:** بيانات حساسة غير محميّة والتي يستطيع المهاجم الوصول إليها:
-يستطيع المهاجم الوصول للبيانات الحساسة الداخلية مثل ملف (  file:///etc/passwd)أو حتى للخدمات الداخلية من خلال استغلال هذه الثغرة
-**سيناريو #3:** الوصول إلى تخزين البيانات الوصفيّة للخدمات السحابيّة :
-يمتلك معظم موفرّي السحابة تخزين البيانات الوصفيّة مثل http://169.254.169.254    ويمكن للمهاجم قراءة تلك البيانات الوصفيّة للحصول على معلومات حساسة منها.
-**سيناريو #4:** اختراق الخدمات الداخلية وإساءة استخدامها من قِبل المهاجم:
-يمكن للمهاجم إساءة استخدام الخدمات الداخلية لإجراء مزيد من الهجمات مثل تنفيذ التعليمات البرمجية عن بُعد (RCE) أو هجوم حجب الخدمة (DoS).
-لمزيد من المعلومات حول المراجع وقائمة CWE المعيّنة: https://top10.owasp.org/2021/ar/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
-  </si>
-  <si>
-    <t>SSRF-Schwachstellen treten immer dann auf, wenn eine Webanwendung eine Remote-Ressource abruft, ohne die, vom Nutzenden angegebene URL zu überprüfen. Dadurch kann ein Angreifender die Anwendung dazu zwingen, eine manipulierte Anfrage an ein unerwartetes Ziel zu senden, selbst wenn sie durch eine Firewall, ein VPN oder eine andere Art von Netzwerkzugriffskontrollliste (ACL) geschützt ist.
-Da moderne Webanwendungen Nutzenden komfortable Funktionen bieten, wird das Abrufen einer URL zu einem gängigen Szenario. 
-Infolgedessen nimmt die Häufigkeit von SSRF zu. 
-Außerdem nimmt der Schweregrad von SSRF aufgrund von der Verbreitung von Cloud-Diensten und der Komplexität der Architekturen zu.</t>
-  </si>
-  <si>
     <t>## Score table
 | Zugeordnete CWEs | Maximale Häufigkeit | Durchschn. Häufigkeit | Durchschn. Ausnutzbarkeit (gewichtet) | Durchschn. Auswirkungen (gewichtet) | Maximale Abdeckung | Durchschnittliche Abdeckung | Gesamtanzahl | CVEs insgesamt |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4891,7 +5091,7 @@
 - Setzen Sie standardmäßig blockierende Firewall-Richtlinien oder Netzwerkzugriffskontrollregeln ein, um den gesamten Intranet-Verkehr zu blockieren, der nicht unbedingt erforderlich ist.
 &lt;br/&gt; *Hinweise:*&lt;br&gt; 
 ~ Legen Sie eine Zuständigkeit und einen Lebenszyklus für Firewall-Regeln auf der Grundlage von Anwendungen fest.&lt;br/&gt;
-~ Protokollieren aller akzeptierten *und* blockierten Netzströme auf Firewalls (siehe [A09:2021 – Fehler beim Logging und Monitoring](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+~ Protokollieren aller akzeptierten *und* blockierten Netzströme auf Firewalls (siehe **A09:2021 – Fehler beim Logging und Monitoring**).
 ### **Auf der Anwendungsebene:**
 * Bereinigung und Validierung aller vom Client gelieferten Eingabedaten
 * Erzwingen Sie das URL-Schema, den Port und das Ziel mit einer Positivliste
@@ -4911,13 +5111,6 @@
 Weitere Informationen zu den Referenzen und zur Liste der zugeordneten CWEs: https://top10.owasp.org/2021/de/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>Falsificación de Solicitudes del Lado del Servidor (SSRF)</t>
-  </si>
-  <si>
-    <t>Las fallas de SSRF ocurren cuando una aplicación web está obteniendo un recurso remoto sin validar la URL proporcionada por el usuario. Permite que un atacante coaccione a la aplicación para que envíe una solicitud falsificada a un destino inesperado, incluso cuando está protegido por un firewall, VPN u otro tipo de lista de control de acceso a la red (ACL).
-Dado que las aplicaciones web modernas brindan a los usuarios finales funciones convenientes, la búsqueda de una URL se convierte en un escenario común. Como resultado, la incidencia de SSRF está aumentando. Además, la gravedad de SSRF es cada vez mayor debido a los servicios en la nube y la complejidad de las arquitecturas.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs mapeadas | Tasa de incidencia máx | Tasa de incidencia prom | Explotabilidad ponderada prom| Impacto ponderado prom | Cobertura máx | Cobertura prom | Incidencias totales | Total CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -4929,7 +5122,7 @@
 -   Haga cumplir las políticas de firewall "denegar por defecto" o las reglas de control de acceso a la red para bloquear todo el tráfico de la intranet excepto el esencial.&lt;br/&gt; 
     *Consejos:*&lt;br&gt; 
     ~ Establezca la propiedad y un ciclo de vida para las reglas de firewall basadas en aplicaciones.&lt;br/&gt;
-    ~ Registre en logs todos los flujos de red aceptados y bloqueados en firewalls (consulte [A09: 2021-Fallas en el Registro y Monitoreo](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+    ~ Registre en logs todos los flujos de red aceptados y bloqueados en firewalls (consulte **A09: 2021-Fallas en el Registro y Monitoreo**).
 ### **Desde la capa de aplicación:**
 -   Sanitice y valide todos los datos de entrada proporcionados por el cliente
 -   Haga cumplir el esquema de URL, el puerto y destino a través de una lista positiva de items permitidos 
@@ -4949,13 +5142,6 @@
 Para obtener más información sobre las referencias y la lista de CWE asociadas: https://top10.owasp.org/2021/es/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>A10 Falsification de requête côté serveur (SSRF)</t>
-  </si>
-  <si>
-    <t>Une faille SSRF se produit lorsqu'une application web récupère une ressource distante sans valider l'URL fournie par l'utilisateur. Elle permet à un attaquant de contraindre l'application à envoyer une requête élaborée à une destination inattendue, même si elle est protégée par un pare-feu, un VPN ou un autre type de liste de contrôle d'accès au réseau (ACL).
-Comme les applications Web modernes offrent aux utilisateurs finaux des fonctions pratiques, la récupération d'une URL devient un scénario courant. Par conséquent, l'incidence d'une SSRF augmente. De même, la gravité de ce phénomène augmente en raison des services en nuage et de la complexité des architectures.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs associées | Taux d'incidence max | Taux d'incidence moyen | Exploitation pondérée moyenne | Impact pondéré moyen | Couverture max | Couverture moyenne | Nombre total d'occurrences | Nombre total de CVEs |
 |:--------------:|:--------------------:|:----------------------:|:-----------------------------:|:--------------------:|:--------------:|:------------------:|:--------------------------:|:--------------------:|
@@ -4967,7 +5153,7 @@
 - appliquer des politiques de pare-feu ou des règles de contrôle d'accès au réseau "refusant par défaut" afin de bloquer tout le trafic intranet sauf celui qui est essentiel.&lt;br/&gt; 
     *Conseils:*&lt;br&gt; 
     - Établir une propriété et un cycle de vie pour les règles du pare-feu en fonction des applications.&lt;br/&gt;
-    - Consigner tous les flux réseau acceptés *et* bloqués sur les pare-feu (voir [A09:2021-Carence des systèmes de contrôle et de journalisation](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+    - Consigner tous les flux réseau acceptés *et* bloqués sur les pare-feu (voir **A09:2021-Carence des systèmes de contrôle et de journalisation**).
 ### **Couche applicative :**
 - assainir et valider toutes les données d'entrée fournies par le client ;
 - imposer le schéma d'URL, le port et la destination avec une liste positive d'autorisation ;
@@ -4987,10 +5173,6 @@
 Pour plus d’informations sur les références et la liste des CWE mappées : https://top10.owasp.org/2021/fr/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>Kecacatan _SSRF_ muncul saat sebuah aplikasi web meminta _remote resource_ tanpa melakukan validasi URL yang di berikan oleh pengguna. Ini memperbolehkan penyerang untuk memaksa aplikasi untuk mengirim _crafted request_ ke destinasi yang tidak diharapkan, meskipun sudah dilindungi oleh _firewall_, VPN, atau tipe lain dari daftar aturan akses jaringan - _Access Control List_ (ACL).
-Aplikasi web saat ini menyediakan fitur yang nyaman bagi pengguna akhir, sehingga proses meminta URL menjadi hal yang lumrah. Oleh karena itu, insiden _SSRF_ semakin meningkat. Selain itu, tingkat keparahan _SSRF_ semakin meningkat karena layanan-layanan _cloud_ dan tingkat komplexitas arsitektur _cloud_.</t>
-  </si>
-  <si>
     <t>## Score table
 | Klasifikasi CWE | Tingkat Kejadian Maksimum | Rata - Rata Tingkat Kejadian  | Cakupan Maximum | Rata - Rata Cakupan | Rata - Rata Bobot Exploitasi | Rata - Rata Bobot Dampak | Total Kejadian | Total CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -5002,7 +5184,7 @@
 - Terapkan kebijakan firewall _deny by default_ atau aturan kontrol akses jaringan untuk memblokir semua lalu lintas eksternal kecuali lalu lintas intranet yang penting.  
   _Petunjuk:_  
   ~ Buat / Bangunlah siklus hidup dan hak kepemilikan untuk peraturan firewall berdasarkan aplikasinya.  
-  ~ Catat semua akses jaringan yang melewati firewall baik akses jaringan yang diterima ataupun yang diblokir/tolak (lihat [A09:2021-Security Logging and Monitoring Failures](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+  ~ Catat semua akses jaringan yang melewati firewall baik akses jaringan yang diterima ataupun yang diblokir/tolak (lihat **A09:2021-Security Logging and Monitoring Failures**).
 ### Dari Application Layer
 - Bersihkan dan validasi semua data inputan yang dimasukkan oleh klien
 - Terapkan skema URL, port, dan destinasi dengan daftar izin positif
@@ -5024,17 +5206,6 @@
 Untuk informasi lebih lanjut tentang referensi dan daftar CWE yang dipetakan: https://top10.owasp.org/2021/id/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>Le falle SSRF si verificano ogni volta che un'applicazione web recupera una risorsa remota
-senza validare l'URL fornito dall'utente. Questo permette ad un attaccante
-di forzare l'applicazione ad inviare una richiesta preparata ad hoc ad una destinazione inattesa, 
-anche quando è protetta da un firewall, una VPN o un altro tipo di
-network access control list (ACL).
-Dato che le moderne applicazioni web forniscono agli utenti finali parecchie funzionalità,
-scaricare dati da un URL è uno scenario comune. Di conseguenza, l'incidenza di
-SSRF è in crescita. Inoltre, la gravità di SSRF sta diventando più alta a causa dei
-servizi cloud e alla complessità crescente delle architetture.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs corrispondenti | Tasso di incidenza Max | Tasso di incidenza Medio | Sfruttabilità pesata | Impatto Medio | Copertura Max | Copertura media | Occorrenze Totali | CVE Totali |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -5050,7 +5221,7 @@
     *Suggerimenti:*&lt;br&gt; 
     ~ Stabilire una ownership e un ciclo di vita per le regole del firewall basate sulle applicazioni.&lt;br/&gt;
     ~ Registrare tutti i flussi di rete accettati *e* bloccati sui firewall
-    (vedi [A09:2021-Security Logging and Monitoring Failures](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+    (vedi **A09:2021-Security Logging and Monitoring Failures**).
 ### **Dal layer applicativo:**
 -   Sanitizzare e convalidare tutti i dati di input forniti dal cliente
 -   Far rispettare lo URL schema, la porta e la destinazione con una allow list
@@ -5084,16 +5255,6 @@
 Per maggiori informazioni sui riferimenti e sull'elenco delle CWE mappate: https://top10.owasp.org/2021/it/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>サーバーサイドリクエストフォージェリ (SSRF)</t>
-  </si>
-  <si>
-    <t>SSRFの欠陥は、Webアプリケーション上からリモートのリソースを取得する際に、ユーザーから提供されたURLを検証せずに使用することで発生します。
-ファイアウォールやVPNあるいはその他の種類のネットワークアクセス制御リスト(ACL)によってアプリケーションが保護されている場合であっても、SSRFによりアプリケーションに対して意図しない宛先へ細工されたリクエストを強制的に発行させることができます。
-モダンなアプリケーションではエンドユーザーに便利な機能を提供するようになり、アプリケーション側でURLを取得することは珍しい状況ではなくなりました。
-そのためSSRFの発生が増加しています。
-またSSRFの深刻度も、クラウドサービスやアーキテクチャの複雑性を背景として、段々と大きくなりつつあります。</t>
-  </si>
-  <si>
     <t>## Score table
 | 対応する CWE 数 | 最大発生率 | 平均発生率 |  加重平均（攻撃の難易度） | 加重平均（攻撃による影響） | 最大網羅率 | 平均網羅率 | 総発生数 | CVE 合計件数 |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -5106,7 +5267,7 @@
     *ヒント:*&lt;br&gt;
     ~ アプリケーションに応じて、ファイアウォールルールの所有権とライフサイクルを明確化します。&lt;br/&gt;
     ~ ファイアウォールにおいて許可されたネットワークフロー、*そして*ブロックされたネットワークフローを全てログとして記録します
-    ([A09:2021-セキュリティログとモニタリングの失敗](A09_2021-Security_Logging_and_Monitoring_Failures.md)を参照)。
+    (**A09:2021-セキュリティログとモニタリングの失敗**を参照)。
 ### **アプリケーション層から:**
 -   クライアントが提供した全ての入力データをサニタイズし、検証します。
 -   明確な許可リスト用いてURLスキーム、ポート、宛先を強制します。
@@ -5126,13 +5287,6 @@
 参考資料およびマッピングされたCWEの一覧について、詳しくはこちら： https://top10.owasp.org/2021/ja/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>Falsificação de Solicitação do Lado do Servidor (SSRF)</t>
-  </si>
-  <si>
-    <t>As falhas de SSRF ocorrem sempre que um aplicativo da web busca um recurso remoto sem validar a URL fornecida pelo usuário. Ele permite que um invasor force o aplicativo a enviar uma solicitação criada para um destino inesperado, mesmo quando protegido por um firewall, VPN ou outro tipo de lista de controle de acesso à rede (ACL).
-Como os aplicativos da web modernos fornecem aos usuários finais recursos convenientes, buscar uma URL se torna um cenário comum. Como resultado, a incidência de SSRF está aumentando. Além disso, a gravidade do SSRF está se tornando mais alta devido aos serviços em nuvem e à complexidade crescente das arquiteturas.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs Mapeadas | Taxa de Incidência Máxima | Taxa Média de Incidência | Exploração Média Ponderada | Impacto Médio Ponderado | Cobertura Máxima | Média de Cobertura | Total de Ocorrências | Total de CVEs |
 |:-------------:|:--------------------:|:--------------------:|:--------------:|:--------------:|:----------------------:|:---------------------:|:-------------------:|:------------:|
@@ -5145,7 +5299,7 @@
 - *Dicas:*
 ~ Estabeleça uma propriedade e um ciclo de vida para regras de firewall baseadas em aplicativos.
 ~ Registrar todos os fluxos de rede aceitos *e* bloqueados em firewalls.
-(veja [A09:2021-Monitoramento de Falhas e Registros de Segurança](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+(veja **A09:2021-Monitoramento de Falhas e Registros de Segurança**).
 ### **Para a Camada de Aplicação:**
 - Higienize e valide todos os dados de entrada fornecidos pelo cliente;
 - Aplique o esquema de URL, porta e destino com uma lista de permissões positiva;
@@ -5165,10 +5319,6 @@
 Para mais informações sobre as referências e a lista de CWEs mapeadas: https://top10.owasp.org/2021/pt-BR/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>SSRF hataları, bir web uygulaması kullanıcı tarafından sağlanan URL’yi doğrulamadan uzak bir kaynağı fetch ettiğinde ortaya çıkar. Bu, saldırganın uygulamayı, firewall, VPN veya başka bir network access control list (ACL) ile korunuyor olsa bile beklenmeyen bir hedefe crafted bir istek göndermeye zorlamasına imkân tanır.
-Modern web uygulamaları son kullanıcılara kullanışlı özellikler sundukça, bir URL’i fetch etmek yaygın bir senaryo hâline gelir. Sonuç olarak, SSRF’nin görülme sıklığı artıyor. Ayrıca cloud servisleri ve mimarilerin karmaşıklığı nedeniyle SSRF’nin ciddiyeti de yükseliyor.</t>
-  </si>
-  <si>
     <t>## Score table
 | CWEs Mapped | Max Incidence Rate | Avg Incidence Rate | Avg Weighted Exploit | Avg Weighted Impact | Max Coverage | Avg Coverage | Total Occurrences | Total CVEs |
 | :---------: | :----------------: | :----------------: | :------------------: | :-----------------: | :----------: | :----------: | :---------------: | :--------: |
@@ -5180,7 +5330,7 @@
 * “Varsayılan olarak reddet (deny by default)” firewall policy’leri veya network access control kuralları uygulayın; temel intranet trafiği dışındaki her şeyi engelleyin.&lt;br/&gt;
   *İpuçları:*&lt;br/&gt;
   \~ Firewall kuralları için uygulama bazlı sahiplik ve lifecycle oluşturun.&lt;br/&gt;
-  \~ Firewall’larda kabul edilen *ve* engellenen tüm network akışlarını log’layın (bkz. [A09:2021-Security Logging and Monitoring Failures](A09_2021-Security_Logging_and_Monitoring_Failures.md)).
+  \~ Firewall’larda kabul edilen *ve* engellenen tüm network akışlarını log’layın (bkz. **A09:2021-Security Logging and Monitoring Failures**).
 ### **Application katmanından**
 * Tüm client tarafından sağlanan input verisini sanitize ve validate edin.
 * URL schema, port ve destination’ı pozitif bir allow list ile zorunlu kılın.
@@ -5200,169 +5350,13 @@
 Referanslar ve eşlenen CWE listesi hakkında daha fazla bilgi: https://top10.owasp.org/2021/tr/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
   </si>
   <si>
-    <t>当网页应用程式正在取得远端资源，却未验证由使用者提供的网址，此时就会发生伪造服务端请求。即便有防火墙、VPN 或其他网路 ACL 保护的情况下，攻击者仍得以强迫网页应用程式发送一个经过捏造的请求给一个非预期的目的端。
-现今的网页应用程式提供终端使用者便利的特色，取得网址已经是常见的了。因此，伪造服务端请求的发生率是在增加当中的。而且，因为云端服务和云端结构的复杂性，伪造服务端请求的严重性将会愈来愈严峻。</t>
-  </si>
-  <si>
-    <t>## Score table
-| 可对照 CWEs 数量 | 最大发生率 | 平均发生率 |最大覆盖范围 | 平均覆盖范围 | 平均加权漏洞 | 平均加权影响 | 出现次数 | 所有相关 CVEs 数量 |
-| :-------------: | :------: | :------: | :--------: | :--------: | :---------: | :--------: | :-----: | :--------------: |
-| 1 | 2.72% | 2.72% | 67.72% | 67.72% | 8.28 | 6.72 | 9,503 | 385 |
-## How to prevent
-开发者可以预防伪造服务端请求，透过实施下列一部分或全部的纵身防御控制措施：
-## **From Network layer** (从网路层着手)
-- 将远端资源存取功能切割成不同子网路以降低伪造服务端请求之冲击
-- 于防火墙政策或于网路存取控制规则实施"预设全拒绝(deny by default)" ，以封锁全部来自外部之网路流量
-## **From Application layer:** (从应用层)
-- 过滤并验证来自于用户端提供之全部输入
-- 以正面表列方式列出 URL、port、目的地清单
-- 不传送原始回应给用户端
-- 停用 HTTP 重新导向
-- 留意网址之一致性，以避免例如 DNS rebinding 攻击、TOCTOU 攻击
-别透过拒绝清单或正规表示式来减缓伪造服务端请求。攻击者有 payload 清单、工具和技巧可以绕过这些拒绝清单
-## Example attack scenarios
-攻击者可以利用伪造服务端请求来攻击在 WAF、防火墙、或网路 ACL 后面的系统，可能采取之情境如下：
-**情境一**：对内部服务器 port scan。如果网路架构未被切割，攻击者可以透过连线结果或连线所经过的时间或拒绝 SSRF payload 连线的状态，加以对应出内部网路并且判断该等 port 在内部服务器是否开启或关闭状态
-**情境二**：机敏资料泄漏。攻击者可以存取本地端档案(例如 &lt;file:///etc/passwd&gt;) 或内部服务已取得机敏资料。
-**情境三**：存取云服务之 metadata storage。大部分云端提供者都有 metadata storage，例如&lt;http://169.254.169.254/&gt;。攻击者可以读取 metadata 以取得机敏资讯。
-**情境四**：渗透内部服务 - 攻击者可以滥用内部服务去执行更进一步的攻击，例如 RCE 或 Dos
-有關參考資料及已對應 CWE 清單的更多資訊： https://top10.owasp.org/2021/zh-Hant/A10_2021-Server-Side_Request_Forgery_%28SSRF%29/</t>
-  </si>
-  <si>
-    <t>annotation</t>
-  </si>
-  <si>
-    <t>name[ar]</t>
-  </si>
-  <si>
-    <t>description[ar]</t>
-  </si>
-  <si>
-    <t>annotation[ar]</t>
-  </si>
-  <si>
-    <t>name[de]</t>
-  </si>
-  <si>
-    <t>description[de]</t>
-  </si>
-  <si>
-    <t>annotation[de]</t>
-  </si>
-  <si>
-    <t>name[es]</t>
-  </si>
-  <si>
-    <t>description[es]</t>
-  </si>
-  <si>
-    <t>annotation[es]</t>
-  </si>
-  <si>
-    <t>name[fr]</t>
-  </si>
-  <si>
-    <t>description[fr]</t>
-  </si>
-  <si>
-    <t>annotation[fr]</t>
-  </si>
-  <si>
-    <t>name[id]</t>
-  </si>
-  <si>
-    <t>description[id]</t>
-  </si>
-  <si>
-    <t>annotation[id]</t>
-  </si>
-  <si>
-    <t>name[it]</t>
-  </si>
-  <si>
-    <t>description[it]</t>
-  </si>
-  <si>
-    <t>annotation[it]</t>
-  </si>
-  <si>
-    <t>name[ja]</t>
-  </si>
-  <si>
-    <t>description[ja]</t>
-  </si>
-  <si>
-    <t>annotation[ja]</t>
-  </si>
-  <si>
-    <t>name[pt]</t>
-  </si>
-  <si>
-    <t>description[pt]</t>
-  </si>
-  <si>
-    <t>annotation[pt]</t>
-  </si>
-  <si>
-    <t>name[tr]</t>
-  </si>
-  <si>
-    <t>description[tr]</t>
-  </si>
-  <si>
-    <t>annotation[tr]</t>
-  </si>
-  <si>
-    <t>name[zh]</t>
-  </si>
-  <si>
-    <t>description[zh]</t>
-  </si>
-  <si>
-    <t>annotation[zh]</t>
-  </si>
-  <si>
-    <t>OWASP Top 10 Web - 2021</t>
-  </si>
-  <si>
-    <t>مرحبًا بكم في أحدث إصدار من أعلى عشرة مخاطر من منظمة أواسب وهي النسخة الحديثة لعام 2021، والتي تأتي بشكل جديد تمامًا ومدعمة برسومات انفوجرافيك التي تستطيع طباعتها واستخدامها ويمكن الحصول عليها من صفحتنا الرئيسية.
-المصدر: https://top10.owasp.org/2021/ar/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>¡Bienvenido a la última entrega del OWASP Top 10! El OWASP Top 10 2021 ha sido totalmente renovado, con un nuevo diseño gráfico y una infografía de una sola página que puedes imprimir u obtener desde nuestra página web.
-Fuente: https://top10.owasp.org/2021/es/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>Bienvenue à cette nouvelle édition de l'OWASP Top 10 ! L'OWASP Top 10 2021 apporte de nombreux changements, avec notamment une nouvelle interface et une nouvelle infographie, disponible sur un format d'une page qu'il est possible de se procurer depuis notre page d'accueil.
-Source: https://top10.owasp.org/2021/fr/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>Selamat datang ke versi terakhir dari OWASP Top 10! OWASP Top 10 2021 semua baru, dengan desain grafis baru dan suatu infografis satu-halaman yang dapat Anda cetak atau dapatkan dari beranda kami.
-Sumber: https://top10.owasp.org/2021/id/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>Ecco a voi l'ultima versione della OWASP Top 10! La OWASP Top 10 2021 è tutta nuova, con un nuovo design grafico e un'infografica di una pagina che potete stampare o scaricare dalla nostra home page.
-Fonte: https://top10.owasp.org/2021/it/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>OWASP トップ 10 の最新版へようこそ! OWASP トップ 10 2021年版は、グラフィックデザインが一新され、1ページのインフォグラフィックになっています。インフォグラフィックは、ホームページから入手でき、印刷することができます。
-出典: https://top10.owasp.org/2021/ja/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>Bem-vindo à última edição do OWASP Top 10! O OWASP Top 10 2021 é totalmente novo, com um novo design gráfico e um infográfico  disponível que você pode imprimir ou obter em nossa página inicial.
-Fonte: https://top10.owasp.org/2021/pt-BR/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>OWASP Top 10’un en güncel sürümüne hoş geldiniz! OWASP Top 10 2021 tamamen yenilendi; yeni bir grafik tasarım ve ana sayfamızdan indirebileceğiniz ya da çıktısını alabileceğiniz tek sayfalık bir infografik ile geliyor.
-Kaynak: https://top10.owasp.org/2021/tr/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>欢迎來到最新版本的 OWASP Top 10！! OWASP Top 10 2021 是一个全新的名单，包含了你可以打印下來的新图示说明，若有需要的话，你可以从我们的网页上面下载。
-來源: https://top10.owasp.org/2021/zh-Hant/A00_2021_Introduction/</t>
-  </si>
-  <si>
-    <t>Willkommen zur neuesten Ausgabe der OWASP Top 10! Die OWASP Top 10:2021 sind völlig neu, mit einem neuen Grafikdesign mit Piktogrammen je Risiko und Mobilgeräte-freundlichen Webseiten.
-Quelle: https://top10.owasp.org/2021/de/A00_2021_Introduction/</t>
+    <t>Die Anwendung besitzt möglicherweise Schwachstellen, wenn folgendes zutrifft:
+- Fehlende Kenntnis über die Versionen aller verwendeten Komponenten der in der Anwendung (sowohl client- als auch serverseitig). Dies beinhaltet sowohl direkte als auch indirekte, verschachtelte Abhängigkeiten.
+- Die verwendete Software besitzt Schwachstellen, wird nicht mehr unterstützt oder ist veraltet. Dies beinhaltet das Betriebssystem, den Web-/Applikationsserver, das Datenbankmanagementsystem (DBMS), Anwendungen, APIs und alle verwendeten Komponenten, Laufzeitumgebungen sowie Bibliotheken.
+- Schwachstellenscans werden nicht regelmäßig durchgeführt und die sicherheitsrelevanten Bulletins der verwendeten Komponenten sind nicht abonniert.
+- Die zugrundeliegende Plattform, die Frameworks und die Abhängigkeiten werden nicht risikobasiert und rechtzeitig repariert oder aktualisiert. Dies geschiet in der Regel in Umgebungen, in denen Patchen eine monatliche oder quartalsweise Tätigkeit ist und einer Änderungskontrolle unterliegt. Dies setzt die Organisation unnötigerweise über Tage oder Monate dem Risiko von Schwachstellen aus, für die schon Patches existieren.
+- Softwareentwickler führen keine Kompatibilitäts-Tests der aktualisierten oder gepatchten Bibliotheken durch.
+- Die Komponenten sind nicht sicher konfiguriert (siehe **A05:2021-Sicherheitsrelevante Fehlkonfiguration**).</t>
   </si>
 </sst>
 </file>
@@ -5740,7 +5734,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="106.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="93" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -5750,162 +5744,162 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>348</v>
+        <v>299</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>349</v>
+        <v>300</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>379</v>
+        <v>330</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>351</v>
+        <v>302</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>352</v>
+        <v>303</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>388</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>354</v>
+        <v>305</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>355</v>
+        <v>306</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>380</v>
+        <v>331</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>357</v>
+        <v>308</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>358</v>
+        <v>309</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>381</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>360</v>
+        <v>311</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>361</v>
+        <v>312</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>382</v>
+        <v>333</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>363</v>
+        <v>314</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>364</v>
+        <v>315</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>383</v>
+        <v>334</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>366</v>
+        <v>317</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>367</v>
+        <v>318</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>384</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>369</v>
+        <v>320</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>370</v>
+        <v>321</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>385</v>
+        <v>336</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>372</v>
+        <v>323</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>373</v>
+        <v>324</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>386</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>375</v>
+        <v>326</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>378</v>
+        <v>329</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>376</v>
+        <v>327</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>387</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -5999,97 +5993,97 @@
         <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>347</v>
+        <v>298</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>348</v>
+        <v>299</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>349</v>
+        <v>300</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>350</v>
+        <v>301</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>351</v>
+        <v>302</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>352</v>
+        <v>303</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>353</v>
+        <v>304</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>354</v>
+        <v>305</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>355</v>
+        <v>306</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>356</v>
+        <v>307</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>357</v>
+        <v>308</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>358</v>
+        <v>309</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>359</v>
+        <v>310</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>360</v>
+        <v>311</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>361</v>
+        <v>312</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>362</v>
+        <v>313</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>363</v>
+        <v>314</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>364</v>
+        <v>315</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>365</v>
+        <v>316</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>366</v>
+        <v>317</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>367</v>
+        <v>318</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>368</v>
+        <v>319</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>369</v>
+        <v>320</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>370</v>
+        <v>321</v>
       </c>
       <c r="AC1" s="2" t="s">
-        <v>371</v>
+        <v>322</v>
       </c>
       <c r="AD1" s="2" t="s">
-        <v>372</v>
+        <v>323</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>373</v>
+        <v>324</v>
       </c>
       <c r="AF1" s="2" t="s">
-        <v>374</v>
+        <v>325</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>375</v>
+        <v>326</v>
       </c>
       <c r="AH1" s="2" t="s">
-        <v>376</v>
+        <v>327</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -6531,100 +6525,100 @@
         <v>29</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="I6" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="J6" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="M6" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="O6" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="P6" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="R6" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="S6" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="T6" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="P6" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="T6" s="5" t="s">
-        <v>187</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>29</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>188</v>
+        <v>348</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>189</v>
+        <v>349</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>191</v>
+        <v>350</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>192</v>
+        <v>351</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>194</v>
+        <v>352</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>195</v>
+        <v>353</v>
       </c>
       <c r="AD6" s="5" t="s">
         <v>29</v>
       </c>
       <c r="AE6" s="5" t="s">
-        <v>196</v>
+        <v>354</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>197</v>
+        <v>355</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -6638,100 +6632,100 @@
         <v>31</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>201</v>
+        <v>356</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>202</v>
+        <v>357</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>204</v>
+        <v>186</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>207</v>
+        <v>388</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>208</v>
+        <v>358</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>209</v>
+        <v>189</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>210</v>
+        <v>359</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>211</v>
+        <v>360</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="U7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="V7" s="5" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="X7" s="5" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>221</v>
+        <v>199</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="AA7" s="5" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>224</v>
+        <v>361</v>
       </c>
       <c r="AC7" s="5" t="s">
-        <v>225</v>
+        <v>362</v>
       </c>
       <c r="AD7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="AE7" s="5" t="s">
-        <v>226</v>
+        <v>363</v>
       </c>
       <c r="AF7" s="5" t="s">
-        <v>227</v>
+        <v>364</v>
       </c>
       <c r="AG7" s="5" t="s">
-        <v>228</v>
+        <v>202</v>
       </c>
       <c r="AH7" s="5" t="s">
-        <v>229</v>
+        <v>203</v>
       </c>
       <c r="AI7" s="5" t="s">
-        <v>230</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -6745,100 +6739,100 @@
         <v>33</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>231</v>
+        <v>365</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>232</v>
+        <v>205</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>233</v>
+        <v>206</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>234</v>
+        <v>207</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>235</v>
+        <v>208</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>236</v>
+        <v>209</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>237</v>
+        <v>366</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>238</v>
+        <v>210</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>239</v>
+        <v>211</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>240</v>
+        <v>367</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>241</v>
+        <v>212</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>242</v>
+        <v>213</v>
       </c>
       <c r="P8" s="5" t="s">
-        <v>243</v>
+        <v>368</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="S8" s="5" t="s">
-        <v>246</v>
+        <v>216</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
       <c r="U8" s="5" t="s">
         <v>33</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>248</v>
+        <v>218</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>251</v>
+        <v>221</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="AA8" s="5" t="s">
-        <v>253</v>
+        <v>223</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>254</v>
+        <v>369</v>
       </c>
       <c r="AC8" s="5" t="s">
-        <v>255</v>
+        <v>224</v>
       </c>
       <c r="AD8" s="5" t="s">
         <v>33</v>
       </c>
       <c r="AE8" s="5" t="s">
-        <v>256</v>
+        <v>370</v>
       </c>
       <c r="AF8" s="5" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="AG8" s="5" t="s">
-        <v>258</v>
+        <v>226</v>
       </c>
       <c r="AH8" s="5" t="s">
-        <v>259</v>
+        <v>227</v>
       </c>
       <c r="AI8" s="5" t="s">
-        <v>260</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -6852,100 +6846,100 @@
         <v>35</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>261</v>
+        <v>229</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>262</v>
+        <v>230</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>263</v>
+        <v>231</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>264</v>
+        <v>232</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>266</v>
+        <v>234</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>267</v>
+        <v>235</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>268</v>
+        <v>236</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>269</v>
+        <v>237</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>270</v>
+        <v>238</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>271</v>
+        <v>239</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>272</v>
+        <v>240</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>273</v>
+        <v>241</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>274</v>
+        <v>242</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="S9" s="5" t="s">
-        <v>276</v>
+        <v>244</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>277</v>
+        <v>245</v>
       </c>
       <c r="U9" s="5" t="s">
         <v>35</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>279</v>
+        <v>247</v>
       </c>
       <c r="X9" s="5" t="s">
-        <v>280</v>
+        <v>248</v>
       </c>
       <c r="Y9" s="5" t="s">
-        <v>281</v>
+        <v>249</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>282</v>
+        <v>250</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>283</v>
+        <v>251</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>284</v>
+        <v>252</v>
       </c>
       <c r="AC9" s="5" t="s">
-        <v>285</v>
+        <v>253</v>
       </c>
       <c r="AD9" s="5" t="s">
         <v>35</v>
       </c>
       <c r="AE9" s="5" t="s">
-        <v>286</v>
+        <v>254</v>
       </c>
       <c r="AF9" s="5" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="AG9" s="5" t="s">
         <v>35</v>
       </c>
       <c r="AH9" s="5" t="s">
-        <v>288</v>
+        <v>256</v>
       </c>
       <c r="AI9" s="5" t="s">
-        <v>289</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -6959,100 +6953,100 @@
         <v>37</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>290</v>
+        <v>371</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>291</v>
+        <v>258</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>292</v>
+        <v>259</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>293</v>
+        <v>260</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>294</v>
+        <v>261</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>295</v>
+        <v>262</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>296</v>
+        <v>372</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>297</v>
+        <v>263</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>299</v>
+        <v>373</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>300</v>
+        <v>265</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>301</v>
+        <v>266</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>302</v>
+        <v>374</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>303</v>
+        <v>267</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>304</v>
+        <v>268</v>
       </c>
       <c r="S10" s="5" t="s">
-        <v>305</v>
+        <v>269</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>306</v>
+        <v>270</v>
       </c>
       <c r="U10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="V10" s="5" t="s">
-        <v>307</v>
+        <v>375</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>308</v>
+        <v>271</v>
       </c>
       <c r="X10" s="5" t="s">
-        <v>309</v>
+        <v>272</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>310</v>
+        <v>376</v>
       </c>
       <c r="Z10" s="5" t="s">
-        <v>311</v>
+        <v>273</v>
       </c>
       <c r="AA10" s="5" t="s">
-        <v>312</v>
+        <v>274</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>313</v>
+        <v>377</v>
       </c>
       <c r="AC10" s="5" t="s">
-        <v>314</v>
+        <v>275</v>
       </c>
       <c r="AD10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="AE10" s="5" t="s">
-        <v>315</v>
+        <v>378</v>
       </c>
       <c r="AF10" s="5" t="s">
-        <v>316</v>
+        <v>276</v>
       </c>
       <c r="AG10" s="5" t="s">
         <v>37</v>
       </c>
       <c r="AH10" s="5" t="s">
-        <v>317</v>
+        <v>277</v>
       </c>
       <c r="AI10" s="5" t="s">
-        <v>318</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -7063,103 +7057,103 @@
         <v>38</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>320</v>
+        <v>280</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>321</v>
+        <v>379</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>322</v>
+        <v>281</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>323</v>
+        <v>282</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>324</v>
+        <v>283</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>325</v>
+        <v>284</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>326</v>
+        <v>380</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>327</v>
+        <v>285</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>328</v>
+        <v>286</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>329</v>
+        <v>381</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>330</v>
+        <v>287</v>
       </c>
       <c r="P11" s="5" t="s">
-        <v>331</v>
+        <v>288</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>332</v>
+        <v>382</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="S11" s="5" t="s">
-        <v>333</v>
+        <v>289</v>
       </c>
       <c r="T11" s="5" t="s">
-        <v>334</v>
+        <v>383</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>335</v>
+        <v>290</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>336</v>
+        <v>384</v>
       </c>
       <c r="X11" s="5" t="s">
-        <v>337</v>
+        <v>291</v>
       </c>
       <c r="Y11" s="5" t="s">
-        <v>338</v>
+        <v>292</v>
       </c>
       <c r="Z11" s="5" t="s">
-        <v>339</v>
+        <v>385</v>
       </c>
       <c r="AA11" s="5" t="s">
-        <v>340</v>
+        <v>293</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>341</v>
+        <v>294</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>342</v>
+        <v>386</v>
       </c>
       <c r="AD11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="AE11" s="5" t="s">
-        <v>343</v>
+        <v>295</v>
       </c>
       <c r="AF11" s="5" t="s">
-        <v>344</v>
+        <v>387</v>
       </c>
       <c r="AG11" s="5" t="s">
-        <v>319</v>
+        <v>279</v>
       </c>
       <c r="AH11" s="5" t="s">
-        <v>345</v>
+        <v>296</v>
       </c>
       <c r="AI11" s="5" t="s">
-        <v>346</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[YAML] Update OWASP Top 10 Web 2021
Chinese Threat name fixes
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web_2021.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web_2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E26D88B-FDBD-4B02-B906-FED3CDC65BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCECEC2B-33F6-4BA8-AC63-F3744030ABB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1650" yWindow="-15870" windowWidth="25440" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="400">
   <si>
     <t>type</t>
   </si>
@@ -603,9 +603,6 @@
   </si>
   <si>
     <t>Componentes Vulneráveis e Desatualizados</t>
-  </si>
-  <si>
-    <t>易受攻击和已淘汰的组件(Vulnerable and Outdated Components)</t>
   </si>
   <si>
     <t>您可能容易受到攻击：
@@ -4163,6 +4160,18 @@
 Secure design; tehditleri sürekli değerlendiren ve kodu bilinen attack method’larına karşı sağlam olacak şekilde tasarlayıp test eden bir kültür ve metodolojidir. Threat modeling, refinement session’larına (veya benzer aktivitelere) entegre edilmelidir; data flow’lar ve access control veya diğer security control’lerdeki değişikliklere bakın. User story geliştirme sırasında doğru akışı ve failure state’lerini belirleyin; sorumlu ve etkilenen taraflarca iyi anlaşıldığından ve üzerinde mutabık kalındığından emin olun. Varsayımları ve koşulları hem beklenen hem de failure flow’ları için analiz edin; hâlâ doğru ve arzu edilir olduklarını doğrulayın. Varsayımların nasıl validate edileceğini ve doğru davranışlar için gerekli koşulların nasıl enforce edileceğini belirleyin. Sonuçların user story içinde dokümante edilmesini sağlayın. Hatalardan öğrenin ve iyileştirmeleri teşvik etmek için pozitif teşvikler sunun. Secure design, yazılıma sonradan eklenebilecek bir eklenti ya da bir tool değildir.
 ### Güvenli Yazılım Geliştirme Döngüsü
 Güvenli yazılım, bir Secure Development Lifecycle, bir tür secure design pattern, paved road methodology, secured component library, tooling ve threat modeling gerektirir. Yazılım projesinin en başından tüm proje ve bakım süreci boyunca security specialist’lerinize ulaşın. Güvenli yazılım geliştirme çabalarınızı yapılandırmaya yardımcı olması için [OWASP Software Assurance Maturity Model (SAMM)](https://owaspsamm.org) kullanılmasını düşünün.</t>
+  </si>
+  <si>
+    <t>易受攻击和已淘汰的组件</t>
+  </si>
+  <si>
+    <t>软体及资料完整性失效</t>
+  </si>
+  <si>
+    <t xml:space="preserve">安全记录及监控失效 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">服务端请求伪造 </t>
   </si>
 </sst>
 </file>
@@ -4514,7 +4523,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -4522,7 +4531,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -4559,162 +4568,162 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -4808,97 +4817,97 @@
         <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -4912,10 +4921,10 @@
         <v>20</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>228</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>229</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>50</v>
@@ -4924,7 +4933,7 @@
         <v>51</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>52</v>
@@ -4933,7 +4942,7 @@
         <v>53</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>54</v>
@@ -4942,7 +4951,7 @@
         <v>55</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>56</v>
@@ -4951,25 +4960,25 @@
         <v>57</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>58</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="U2" s="5" t="s">
         <v>20</v>
       </c>
       <c r="V2" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="W2" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="X2" s="5" t="s">
         <v>59</v>
@@ -4978,25 +4987,25 @@
         <v>60</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AA2" s="5" t="s">
         <v>61</v>
       </c>
       <c r="AB2" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="AC2" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="AC2" s="5" t="s">
-        <v>238</v>
-      </c>
       <c r="AD2" s="10" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AE2" s="5" t="s">
         <v>62</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AG2" s="5" t="s">
         <v>63</v>
@@ -5005,7 +5014,7 @@
         <v>64</v>
       </c>
       <c r="AI2" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5019,10 +5028,10 @@
         <v>22</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>242</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>65</v>
@@ -5031,25 +5040,25 @@
         <v>66</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>67</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>68</v>
       </c>
       <c r="M3" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>245</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>246</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>69</v>
@@ -5058,52 +5067,52 @@
         <v>70</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>71</v>
       </c>
       <c r="S3" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="T3" s="5" t="s">
         <v>248</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>249</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>22</v>
       </c>
       <c r="V3" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="W3" s="5" t="s">
         <v>250</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>251</v>
       </c>
       <c r="X3" s="5" t="s">
         <v>72</v>
       </c>
       <c r="Y3" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="Z3" s="5" t="s">
         <v>252</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>253</v>
       </c>
       <c r="AA3" s="5" t="s">
         <v>73</v>
       </c>
       <c r="AB3" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="AC3" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="AC3" s="5" t="s">
-        <v>255</v>
-      </c>
       <c r="AD3" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="AE3" s="5" t="s">
         <v>74</v>
       </c>
       <c r="AF3" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AG3" s="5" t="s">
         <v>75</v>
@@ -5112,7 +5121,7 @@
         <v>76</v>
       </c>
       <c r="AI3" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5126,10 +5135,10 @@
         <v>24</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>258</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>259</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>77</v>
@@ -5138,7 +5147,7 @@
         <v>78</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>24</v>
@@ -5147,7 +5156,7 @@
         <v>79</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>80</v>
@@ -5156,7 +5165,7 @@
         <v>81</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>24</v>
@@ -5165,52 +5174,52 @@
         <v>82</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>83</v>
       </c>
       <c r="S4" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="T4" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="T4" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>24</v>
       </c>
       <c r="V4" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="W4" s="5" t="s">
         <v>266</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>267</v>
       </c>
       <c r="X4" s="5" t="s">
         <v>84</v>
       </c>
       <c r="Y4" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="Z4" s="5" t="s">
         <v>268</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>269</v>
       </c>
       <c r="AA4" s="5" t="s">
         <v>85</v>
       </c>
       <c r="AB4" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="AC4" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="AC4" s="5" t="s">
-        <v>271</v>
-      </c>
       <c r="AD4" s="10" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="AE4" s="5" t="s">
         <v>86</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="AG4" s="5" t="s">
         <v>87</v>
@@ -5219,7 +5228,7 @@
         <v>88</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5236,7 +5245,7 @@
         <v>89</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>90</v>
@@ -5245,7 +5254,7 @@
         <v>91</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>92</v>
@@ -5254,7 +5263,7 @@
         <v>93</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>94</v>
@@ -5263,7 +5272,7 @@
         <v>95</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>96</v>
@@ -5272,7 +5281,7 @@
         <v>97</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="R5" s="5" t="s">
         <v>98</v>
@@ -5281,7 +5290,7 @@
         <v>99</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="U5" s="5" t="s">
         <v>26</v>
@@ -5290,34 +5299,34 @@
         <v>100</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="X5" s="5" t="s">
         <v>101</v>
       </c>
       <c r="Y5" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="Z5" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>282</v>
       </c>
       <c r="AA5" s="5" t="s">
         <v>102</v>
       </c>
       <c r="AB5" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="AC5" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="AC5" s="5" t="s">
+      <c r="AD5" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="AE5" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="AF5" s="5" t="s">
         <v>284</v>
-      </c>
-      <c r="AD5" s="10" t="s">
-        <v>383</v>
-      </c>
-      <c r="AE5" s="10" t="s">
-        <v>396</v>
-      </c>
-      <c r="AF5" s="5" t="s">
-        <v>285</v>
       </c>
       <c r="AG5" s="5" t="s">
         <v>103</v>
@@ -5326,7 +5335,7 @@
         <v>104</v>
       </c>
       <c r="AI5" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5340,10 +5349,10 @@
         <v>28</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>287</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>288</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>105</v>
@@ -5352,34 +5361,34 @@
         <v>106</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>107</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>108</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>109</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>110</v>
@@ -5388,43 +5397,43 @@
         <v>111</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>28</v>
       </c>
       <c r="V6" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="W6" s="5" t="s">
         <v>294</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>295</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>112</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AA6" s="5" t="s">
         <v>113</v>
       </c>
       <c r="AB6" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="AC6" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="AC6" s="5" t="s">
+      <c r="AD6" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="AE6" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="AF6" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="AD6" s="10" t="s">
-        <v>384</v>
-      </c>
-      <c r="AE6" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="AF6" s="5" t="s">
-        <v>299</v>
       </c>
       <c r="AG6" s="5" t="s">
         <v>114</v>
@@ -5433,7 +5442,7 @@
         <v>115</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5447,10 +5456,10 @@
         <v>30</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>300</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>301</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>116</v>
@@ -5459,25 +5468,25 @@
         <v>117</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>118</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>119</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>120</v>
@@ -5486,7 +5495,7 @@
         <v>121</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="R7" s="5" t="s">
         <v>122</v>
@@ -5495,52 +5504,52 @@
         <v>123</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="U7" s="5" t="s">
         <v>30</v>
       </c>
       <c r="V7" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="W7" s="5" t="s">
         <v>307</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>308</v>
       </c>
       <c r="X7" s="5" t="s">
         <v>124</v>
       </c>
       <c r="Y7" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="Z7" s="5" t="s">
         <v>309</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>310</v>
       </c>
       <c r="AA7" s="5" t="s">
         <v>125</v>
       </c>
       <c r="AB7" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="AC7" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="AC7" s="5" t="s">
-        <v>312</v>
-      </c>
       <c r="AD7" s="10" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AE7" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="AF7" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="AG7" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="AH7" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="AH7" s="5" t="s">
-        <v>127</v>
-      </c>
       <c r="AI7" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5554,100 +5563,100 @@
         <v>32</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="G8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="K8" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="J8" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="K8" s="5" t="s">
+      <c r="M8" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="N8" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="O8" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="P8" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="Q8" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="O8" s="5" t="s">
+      <c r="R8" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="P8" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q8" s="5" t="s">
+      <c r="S8" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="R8" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="S8" s="5" t="s">
+      <c r="T8" s="5" t="s">
         <v>320</v>
-      </c>
-      <c r="T8" s="5" t="s">
-        <v>321</v>
       </c>
       <c r="U8" s="5" t="s">
         <v>32</v>
       </c>
       <c r="V8" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="W8" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="W8" s="5" t="s">
+      <c r="X8" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y8" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="X8" s="5" t="s">
+      <c r="Z8" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="AA8" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="Y8" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="Z8" s="5" t="s">
+      <c r="AB8" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="AA8" s="5" t="s">
+      <c r="AC8" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="AD8" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="AE8" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="AF8" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="AG8" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="AB8" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="AC8" s="5" t="s">
+      <c r="AH8" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="AI8" s="5" t="s">
         <v>327</v>
-      </c>
-      <c r="AD8" s="10" t="s">
-        <v>386</v>
-      </c>
-      <c r="AE8" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="AF8" s="10" t="s">
-        <v>391</v>
-      </c>
-      <c r="AG8" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="AH8" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="AI8" s="5" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="9" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5661,100 +5670,100 @@
         <v>34</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="J9" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="J9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="M9" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="N9" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="O9" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="M9" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="N9" s="5" t="s">
+      <c r="P9" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q9" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="O9" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="P9" s="5" t="s">
+      <c r="R9" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="Q9" s="5" t="s">
+      <c r="S9" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="R9" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="S9" s="5" t="s">
+      <c r="T9" s="5" t="s">
         <v>336</v>
-      </c>
-      <c r="T9" s="5" t="s">
-        <v>337</v>
       </c>
       <c r="U9" s="5" t="s">
         <v>34</v>
       </c>
       <c r="V9" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="W9" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="W9" s="5" t="s">
+      <c r="X9" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y9" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="X9" s="5" t="s">
+      <c r="Z9" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="AA9" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="Y9" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="Z9" s="5" t="s">
+      <c r="AB9" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="AA9" s="5" t="s">
+      <c r="AC9" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="AD9" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="AE9" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="AB9" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="AC9" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="AD9" s="10" t="s">
-        <v>387</v>
-      </c>
-      <c r="AE9" s="5" t="s">
+      <c r="AF9" s="10" t="s">
+        <v>391</v>
+      </c>
+      <c r="AG9" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="AH9" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="AF9" s="10" t="s">
-        <v>392</v>
-      </c>
-      <c r="AG9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="AH9" s="5" t="s">
-        <v>149</v>
-      </c>
       <c r="AI9" s="5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5768,100 +5777,100 @@
         <v>36</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="J10" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="K10" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="L10" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="M10" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="N10" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="L10" s="5" t="s">
+      <c r="O10" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="M10" s="5" t="s">
+      <c r="P10" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="N10" s="5" t="s">
+      <c r="Q10" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="O10" s="5" t="s">
+      <c r="R10" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="P10" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="Q10" s="5" t="s">
+      <c r="S10" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="R10" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="S10" s="5" t="s">
+      <c r="T10" s="5" t="s">
         <v>350</v>
-      </c>
-      <c r="T10" s="5" t="s">
-        <v>351</v>
       </c>
       <c r="U10" s="5" t="s">
         <v>36</v>
       </c>
       <c r="V10" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="W10" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="W10" s="5" t="s">
+      <c r="X10" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y10" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="X10" s="5" t="s">
+      <c r="Z10" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="AA10" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="Y10" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="Z10" s="5" t="s">
+      <c r="AB10" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="AA10" s="5" t="s">
+      <c r="AC10" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="AD10" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="AE10" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="AF10" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="AG10" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="AH10" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="AB10" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="AC10" s="5" t="s">
+      <c r="AI10" s="5" t="s">
         <v>357</v>
-      </c>
-      <c r="AD10" s="10" t="s">
-        <v>388</v>
-      </c>
-      <c r="AE10" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="AF10" s="10" t="s">
-        <v>393</v>
-      </c>
-      <c r="AG10" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="AH10" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="AI10" s="5" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="11" spans="1:35" ht="409.6" x14ac:dyDescent="0.3">
@@ -5872,103 +5881,103 @@
         <v>37</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="E11" s="5" t="s">
+      <c r="G11" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="G11" s="5" t="s">
+      <c r="I11" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="L11" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="K11" s="5" t="s">
+      <c r="M11" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q11" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="L11" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="N11" s="5" t="s">
+      <c r="R11" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="S11" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="T11" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="O11" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="P11" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q11" s="5" t="s">
+      <c r="U11" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="V11" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="R11" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="S11" s="5" t="s">
+      <c r="W11" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="X11" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="T11" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="U11" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="V11" s="5" t="s">
+      <c r="Y11" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="W11" s="5" t="s">
+      <c r="Z11" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="X11" s="5" t="s">
+      <c r="AA11" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="Y11" s="5" t="s">
-        <v>366</v>
-      </c>
-      <c r="Z11" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="AA11" s="5" t="s">
+      <c r="AB11" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="AB11" s="5" t="s">
+      <c r="AC11" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="AD11" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="AE11" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="AC11" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="AD11" s="10" t="s">
-        <v>389</v>
-      </c>
-      <c r="AE11" s="5" t="s">
+      <c r="AF11" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="AG11" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="AH11" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="AF11" s="10" t="s">
-        <v>394</v>
-      </c>
-      <c r="AG11" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="AH11" s="5" t="s">
-        <v>170</v>
-      </c>
       <c r="AI11" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>